<commit_message>
auto: anime list update (PC) 2026-07-27
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>600478</v>
+        <v>623743</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -9110,7 +9110,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-07-18T09:00:38</t>
+          <t>2026-07-27T09:00:34</t>
         </is>
       </c>
     </row>
@@ -9696,15 +9696,15 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=hFldDZZcrQo</t>
+          <t>https://www.youtube.com/watch?v=_wL4-eA8JmU</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>67022</v>
+        <v>94236</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>GOOD SMILE CHANNEL</t>
+          <t>METANICK</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -9713,7 +9713,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>254165</v>
+        <v>254406</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -9722,7 +9722,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-07-18T09:01:01</t>
+          <t>2026-07-27T09:00:57</t>
         </is>
       </c>
     </row>
@@ -9767,7 +9767,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>170434</v>
+        <v>352935</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -9780,7 +9780,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>10929</v>
+        <v>16101</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -9789,7 +9789,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-07-17T09:00:31</t>
+          <t>2026-07-27T09:01:06</t>
         </is>
       </c>
     </row>
@@ -9834,7 +9834,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>64180</v>
+        <v>78109</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -9847,7 +9847,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>64180</v>
+        <v>78109</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-07-17T09:00:40</t>
+          <t>2026-07-27T09:01:15</t>
         </is>
       </c>
     </row>
@@ -9897,11 +9897,11 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=0_xM9UeELDc</t>
+          <t>https://www.youtube.com/watch?v=pU3P4At856Q</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>450371</v>
+        <v>224608</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -9910,11 +9910,11 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=0_xM9UeELDc</t>
+          <t>https://www.youtube.com/watch?v=pU3P4At856Q</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>450371</v>
+        <v>224608</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -9923,7 +9923,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-07-17T09:00:50</t>
+          <t>2026-07-27T09:01:24</t>
         </is>
       </c>
     </row>
@@ -10145,7 +10145,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>6832555</v>
+        <v>6854885</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -10158,7 +10158,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>91671</v>
+        <v>101281</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-07-18T09:01:14</t>
+          <t>2026-07-27T09:01:36</t>
         </is>
       </c>
     </row>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>325501</v>
+        <v>505716</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -10689,7 +10689,7 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>126318</v>
+        <v>275390</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -10698,7 +10698,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-07-17T09:01:02</t>
+          <t>2026-07-27T09:01:52</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>10735</v>
+        <v>15126</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -10946,7 +10946,7 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-07-18T09:01:42</t>
+          <t>2026-07-27T09:02:20</t>
         </is>
       </c>
     </row>
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>1336939</v>
+        <v>1878959</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -11358,7 +11358,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>1336939</v>
+        <v>1878959</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -11367,7 +11367,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-07-17T09:01:21</t>
+          <t>2026-07-27T09:02:40</t>
         </is>
       </c>
     </row>
@@ -11613,7 +11613,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>31702</v>
+        <v>38537</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -11626,7 +11626,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>31702</v>
+        <v>38537</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -11635,7 +11635,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-07-18T09:02:00</t>
+          <t>2026-07-27T09:02:49</t>
         </is>
       </c>
     </row>
@@ -12416,7 +12416,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>51511</v>
+        <v>66730</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -12429,7 +12429,7 @@
         </is>
       </c>
       <c r="M58" t="n">
-        <v>6837</v>
+        <v>7982</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -12438,7 +12438,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-07-18T09:02:15</t>
+          <t>2026-07-27T09:03:03</t>
         </is>
       </c>
     </row>
@@ -13038,7 +13038,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>356566</v>
+        <v>454824</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -13051,7 +13051,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>68342</v>
+        <v>136493</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -13060,7 +13060,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-07-18T09:02:25</t>
+          <t>2026-07-27T09:03:13</t>
         </is>
       </c>
     </row>
@@ -13412,33 +13412,33 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=wFoEFV8pWH8</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>294153</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>SPYAIR Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=_j3Bm3tr7dA</t>
         </is>
       </c>
-      <c r="J74" t="n">
-        <v>115779</v>
-      </c>
-      <c r="K74" t="inlineStr">
+      <c r="M74" t="n">
+        <v>129526</v>
+      </c>
+      <c r="N74" t="inlineStr">
         <is>
           <t>SHOCHIKU anime Channel</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=_j3Bm3tr7dA</t>
-        </is>
-      </c>
-      <c r="M74" t="n">
-        <v>115779</v>
-      </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>SHOCHIKU anime Channel</t>
-        </is>
-      </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-07-18T09:02:37</t>
+          <t>2026-07-27T09:03:24</t>
         </is>
       </c>
     </row>
@@ -13483,7 +13483,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>184427</v>
+        <v>225375</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -13495,7 +13495,7 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-07-18T09:02:47</t>
+          <t>2026-07-27T09:03:33</t>
         </is>
       </c>
     </row>
@@ -13536,33 +13536,23 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=wTQdf37-OBk</t>
+          <t>https://www.youtube.com/watch?v=REA6cv8IZqc</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>113128</v>
+        <v>790046</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=wTQdf37-OBk</t>
-        </is>
-      </c>
-      <c r="M76" t="n">
-        <v>113128</v>
-      </c>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
+          <t>原因は自分にある。Official</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-07-18T09:02:56</t>
+          <t>2026-07-27T09:03:58</t>
         </is>
       </c>
     </row>
@@ -13975,7 +13965,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>1958</v>
+        <v>8176</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -13988,7 +13978,7 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>1958</v>
+        <v>8176</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -13997,7 +13987,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-07-18T09:03:14</t>
+          <t>2026-07-27T09:04:10</t>
         </is>
       </c>
     </row>
@@ -14176,7 +14166,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>9108593</v>
+        <v>9189529</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -14189,7 +14179,7 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>181286</v>
+        <v>197569</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -14198,7 +14188,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-07-18T09:03:24</t>
+          <t>2026-07-27T09:04:19</t>
         </is>
       </c>
     </row>
@@ -14243,7 +14233,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>181286</v>
+        <v>197569</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -14256,7 +14246,7 @@
         </is>
       </c>
       <c r="M87" t="n">
-        <v>181286</v>
+        <v>197569</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -14265,7 +14255,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-07-18T09:03:33</t>
+          <t>2026-07-27T09:04:28</t>
         </is>
       </c>
     </row>
@@ -14353,7 +14343,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>48617</v>
+        <v>69746</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -14365,7 +14355,7 @@
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-07-18T09:04:00</t>
+          <t>2026-07-27T09:04:59</t>
         </is>
       </c>
     </row>
@@ -14453,7 +14443,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>61500</v>
+        <v>7160043</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -14466,7 +14456,7 @@
         </is>
       </c>
       <c r="M91" t="n">
-        <v>52279</v>
+        <v>493171</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -14475,7 +14465,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-07-18T09:04:15</t>
+          <t>2026-07-27T09:05:15</t>
         </is>
       </c>
     </row>
@@ -14764,7 +14754,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>34408</v>
+        <v>47550</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -14777,7 +14767,7 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>4316</v>
+        <v>10705</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -14786,7 +14776,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-07-18T09:04:24</t>
+          <t>2026-07-27T09:05:27</t>
         </is>
       </c>
     </row>
@@ -15319,7 +15309,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1346995</v>
+        <v>1619234</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -15332,7 +15322,7 @@
         </is>
       </c>
       <c r="M105" t="n">
-        <v>386727</v>
+        <v>461618</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -15341,7 +15331,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-07-18T09:04:46</t>
+          <t>2026-07-27T09:05:47</t>
         </is>
       </c>
     </row>
@@ -15386,7 +15376,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>1346995</v>
+        <v>1619234</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -15399,7 +15389,7 @@
         </is>
       </c>
       <c r="M106" t="n">
-        <v>386727</v>
+        <v>461618</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -15408,7 +15398,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-07-18T09:04:55</t>
+          <t>2026-07-27T09:05:56</t>
         </is>
       </c>
     </row>
@@ -15496,7 +15486,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>562336</v>
+        <v>619072</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -15509,7 +15499,7 @@
         </is>
       </c>
       <c r="M108" t="n">
-        <v>562336</v>
+        <v>619072</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -15518,7 +15508,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-07-18T09:05:07</t>
+          <t>2026-07-27T09:06:07</t>
         </is>
       </c>
     </row>
@@ -15630,7 +15620,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>24509</v>
+        <v>36389</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -15643,7 +15633,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>15643</v>
+        <v>20749</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -15652,7 +15642,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-07-18T09:05:16</t>
+          <t>2026-07-27T09:06:16</t>
         </is>
       </c>
     </row>
@@ -15898,19 +15888,29 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>750794</v>
+        <v>816551</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
           <t>TOHO animation</t>
         </is>
       </c>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
-      <c r="N114" t="inlineStr"/>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=T3gqwRlME5Q</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>109473</v>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-07-17T09:02:42</t>
+          <t>2026-07-27T09:06:25</t>
         </is>
       </c>
     </row>
@@ -16018,11 +16018,11 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=PWN4MO0ILIM</t>
+          <t>https://www.youtube.com/watch?v=r-4zKDCNjwM</t>
         </is>
       </c>
       <c r="J116" t="n">
-        <v>266997</v>
+        <v>26835</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -16035,7 +16035,7 @@
         </is>
       </c>
       <c r="M116" t="n">
-        <v>21316</v>
+        <v>25808</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -16044,7 +16044,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-07-18T09:05:26</t>
+          <t>2026-07-27T09:06:34</t>
         </is>
       </c>
     </row>
@@ -16462,7 +16462,7 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>20179</v>
+        <v>20601</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -16474,7 +16474,7 @@
       <c r="N124" t="inlineStr"/>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-07-18T09:05:55</t>
+          <t>2026-07-27T09:07:02</t>
         </is>
       </c>
     </row>
@@ -16873,7 +16873,7 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>15823</v>
+        <v>21904</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -16886,7 +16886,7 @@
         </is>
       </c>
       <c r="M131" t="n">
-        <v>12311</v>
+        <v>17351</v>
       </c>
       <c r="N131" t="inlineStr">
         <is>
@@ -16895,7 +16895,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-07-17T09:03:20</t>
+          <t>2026-07-27T09:07:18</t>
         </is>
       </c>
     </row>
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>492</v>
+        <v>2758</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
@@ -17197,7 +17197,7 @@
         </is>
       </c>
       <c r="M136" t="n">
-        <v>492</v>
+        <v>2758</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
@@ -17206,7 +17206,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-07-17T09:03:29</t>
+          <t>2026-07-27T09:07:31</t>
         </is>
       </c>
     </row>
@@ -17887,7 +17887,7 @@
         </is>
       </c>
       <c r="J147" t="n">
-        <v>55063</v>
+        <v>70444</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -17899,7 +17899,7 @@
       <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-07-18T09:06:30</t>
+          <t>2026-07-27T09:08:03</t>
         </is>
       </c>
     </row>
@@ -18274,7 +18274,7 @@
         </is>
       </c>
       <c r="J154" t="n">
-        <v>103834</v>
+        <v>135157</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
@@ -18287,7 +18287,7 @@
         </is>
       </c>
       <c r="M154" t="n">
-        <v>103834</v>
+        <v>135157</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -18296,7 +18296,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-07-18T09:06:42</t>
+          <t>2026-07-27T09:08:15</t>
         </is>
       </c>
     </row>
@@ -18475,7 +18475,7 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>7403</v>
+        <v>11452</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18488,7 +18488,7 @@
         </is>
       </c>
       <c r="M157" t="n">
-        <v>7403</v>
+        <v>11452</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -18497,7 +18497,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-07-17T09:03:50</t>
+          <t>2026-07-27T09:08:24</t>
         </is>
       </c>
     </row>
@@ -18609,7 +18609,7 @@
         </is>
       </c>
       <c r="J159" t="n">
-        <v>298375</v>
+        <v>299471</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18622,7 +18622,7 @@
         </is>
       </c>
       <c r="M159" t="n">
-        <v>298375</v>
+        <v>299471</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -18631,7 +18631,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-07-18T09:06:52</t>
+          <t>2026-07-27T09:08:33</t>
         </is>
       </c>
     </row>
@@ -19473,13 +19473,27 @@
           <t>JO1</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wDY2s73E8DM</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v>84</v>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>テレビ公式</t>
+        </is>
+      </c>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>2026-07-27T09:09:53</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19646,7 +19660,7 @@
         </is>
       </c>
       <c r="J180" t="n">
-        <v>294655</v>
+        <v>298421</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
@@ -19659,7 +19673,7 @@
         </is>
       </c>
       <c r="M180" t="n">
-        <v>294655</v>
+        <v>298421</v>
       </c>
       <c r="N180" t="inlineStr">
         <is>
@@ -19668,7 +19682,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-07-18T09:08:01</t>
+          <t>2026-07-27T09:10:03</t>
         </is>
       </c>
     </row>
@@ -19713,7 +19727,7 @@
         </is>
       </c>
       <c r="J181" t="n">
-        <v>294656</v>
+        <v>298421</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
@@ -19726,7 +19740,7 @@
         </is>
       </c>
       <c r="M181" t="n">
-        <v>294656</v>
+        <v>298421</v>
       </c>
       <c r="N181" t="inlineStr">
         <is>
@@ -19735,7 +19749,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-07-18T09:08:11</t>
+          <t>2026-07-27T09:10:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-28
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -6791,7 +6791,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月7日（水）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -8801,7 +8801,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
+          <t>2026年10月3日（土）～ 日本テレビにて</t>
         </is>
       </c>
       <c r="H160" t="inlineStr"/>
@@ -8867,7 +8867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O185"/>
+  <dimension ref="A1:O186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9031,7 +9031,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>5774</v>
+        <v>8042</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -9044,7 +9044,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>5774</v>
+        <v>8042</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -9053,7 +9053,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-07-21T09:00:12</t>
+          <t>2026-07-28T09:00:18</t>
         </is>
       </c>
     </row>
@@ -18713,7 +18713,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D161" t="b">
@@ -18721,7 +18721,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -18729,12 +18729,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>THE RAMPAGE</t>
         </is>
       </c>
       <c r="I161" t="inlineStr"/>
@@ -18764,7 +18764,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -18772,12 +18772,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>krage</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I162" t="inlineStr"/>
@@ -18799,7 +18799,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D163" t="b">
@@ -18807,7 +18807,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -18815,12 +18815,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>amazarashi</t>
+          <t>krage</t>
         </is>
       </c>
       <c r="I163" t="inlineStr"/>
@@ -18842,7 +18842,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D164" t="b">
@@ -18858,12 +18858,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>amazarashi</t>
         </is>
       </c>
       <c r="I164" t="inlineStr"/>
@@ -18885,7 +18885,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D165" t="b">
@@ -18901,12 +18901,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I165" t="inlineStr"/>
@@ -18936,7 +18936,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -18944,12 +18944,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -18971,7 +18971,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D167" t="b">
@@ -18979,7 +18979,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -18987,12 +18987,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>跡部景吾＆忍足侑士</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -19022,7 +19022,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -19030,12 +19030,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -19057,7 +19057,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D169" t="b">
@@ -19065,7 +19065,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19073,45 +19073,21 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J169" t="n">
-        <v>682181</v>
-      </c>
-      <c r="K169" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L169" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M169" t="n">
-        <v>682181</v>
-      </c>
-      <c r="N169" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O169" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:16:41</t>
-        </is>
-      </c>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="inlineStr"/>
+      <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -19132,7 +19108,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -19140,21 +19116,21 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
+          <t>Kucci</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
         </is>
       </c>
       <c r="J170" t="n">
-        <v>372964</v>
+        <v>682181</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -19163,11 +19139,11 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
         </is>
       </c>
       <c r="M170" t="n">
-        <v>372964</v>
+        <v>682181</v>
       </c>
       <c r="N170" t="inlineStr">
         <is>
@@ -19176,7 +19152,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-07-22T09:16:49</t>
+          <t>2026-07-22T09:16:41</t>
         </is>
       </c>
     </row>
@@ -19191,7 +19167,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D171" t="b">
@@ -19207,21 +19183,45 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
-      <c r="M171" t="inlineStr"/>
-      <c r="N171" t="inlineStr"/>
-      <c r="O171" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>372964</v>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M171" t="n">
+        <v>372964</v>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:16:49</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -19234,7 +19234,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D172" t="b">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -19250,12 +19250,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Ado</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I172" t="inlineStr"/>
@@ -19277,7 +19277,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -19293,12 +19293,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I173" t="inlineStr"/>
@@ -19328,7 +19328,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -19336,12 +19336,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -19363,7 +19363,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -19371,7 +19371,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -19379,12 +19379,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I175" t="inlineStr"/>
@@ -19414,7 +19414,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -19422,12 +19422,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>East Of Eden</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -19449,7 +19449,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -19457,7 +19457,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -19465,35 +19465,21 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=wDY2s73E8DM</t>
-        </is>
-      </c>
-      <c r="J177" t="n">
-        <v>84</v>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>テレビ公式</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr">
-        <is>
-          <t>2026-07-27T09:09:53</t>
-        </is>
-      </c>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19506,7 +19492,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -19522,43 +19508,33 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>JO1</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+          <t>https://www.youtube.com/watch?v=wDY2s73E8DM</t>
         </is>
       </c>
       <c r="J178" t="n">
-        <v>2587</v>
+        <v>84</v>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L178" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M178" t="n">
-        <v>2587</v>
-      </c>
-      <c r="N178" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
+          <t>テレビ公式</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-07-22T09:17:34</t>
+          <t>2026-07-27T09:09:53</t>
         </is>
       </c>
     </row>
@@ -19573,7 +19549,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -19589,33 +19565,43 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J179" t="n">
-        <v>106403</v>
+        <v>2587</v>
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L179" t="inlineStr"/>
-      <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M179" t="n">
+        <v>2587</v>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-07-22T09:17:48</t>
+          <t>2026-07-22T09:17:34</t>
         </is>
       </c>
     </row>
@@ -19630,7 +19616,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -19646,43 +19632,33 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J180" t="n">
-        <v>298421</v>
+        <v>106403</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L180" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M180" t="n">
-        <v>298421</v>
-      </c>
-      <c r="N180" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-07-27T09:10:03</t>
+          <t>2026-07-22T09:17:48</t>
         </is>
       </c>
     </row>
@@ -19705,7 +19681,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -19713,12 +19689,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -19749,7 +19725,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-07-27T09:10:13</t>
+          <t>2026-07-27T09:10:03</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19740,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -19772,7 +19748,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -19780,21 +19756,45 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr"/>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
-      <c r="M182" t="inlineStr"/>
-      <c r="N182" t="inlineStr"/>
-      <c r="O182" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>298421</v>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M182" t="n">
+        <v>298421</v>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>2026-07-27T09:10:13</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -19815,7 +19815,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -19823,12 +19823,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -19850,7 +19850,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -19858,7 +19858,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -19866,45 +19866,21 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J184" t="n">
-        <v>776489</v>
-      </c>
-      <c r="K184" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M184" t="n">
-        <v>367020</v>
-      </c>
-      <c r="N184" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O184" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:18:09</t>
-        </is>
-      </c>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19925,7 +19901,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -19933,41 +19909,108 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J185" t="n">
+        <v>776489</v>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M185" t="n">
+        <v>367020</v>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D186" t="b">
+        <v>0</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>1</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr">
+      <c r="H186" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I185" t="inlineStr">
+      <c r="I186" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="J185" t="n">
+      <c r="J186" t="n">
         <v>384697</v>
       </c>
-      <c r="K185" t="inlineStr">
+      <c r="K186" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L185" t="inlineStr">
+      <c r="L186" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M185" t="n">
+      <c r="M186" t="n">
         <v>384697</v>
       </c>
-      <c r="N185" t="inlineStr">
+      <c r="N186" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O185" t="inlineStr">
+      <c r="O186" t="inlineStr">
         <is>
           <t>2026-07-22T09:18:19</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-29
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M161"/>
+  <dimension ref="A1:M162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>氷の城壁 第2期</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -6157,12 +6157,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026年10月1日（木）～ TBS系28局にて</t>
+          <t>2026年9月5日（土）～ テレビ愛知・テレ東系列6局ネットほか</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>スタジオKAI</t>
+          <t>AtoriE</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -6171,7 +6171,7 @@
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28854</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>サイバーパンク：エッジランナーズ2</t>
+          <t>氷の城壁 第2期</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -6197,17 +6197,17 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年秋 Netflixにて</t>
+          <t>2026年10月1日（木）～ TBS系28局にて</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TRIGGER</t>
+          <t>スタジオKAI</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -6216,7 +6216,7 @@
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
         </is>
       </c>
     </row>
@@ -6234,7 +6234,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PSYREN -サイレン-</t>
+          <t>サイバーパンク：エッジランナーズ2</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -6242,17 +6242,17 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX・BS11ほか</t>
+          <t>2026年秋 Netflixにて</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>サテライト</t>
+          <t>TRIGGER</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -6261,7 +6261,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>佐々木とピーちゃん シーズン２</t>
+          <t>PSYREN -サイレン-</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -6292,12 +6292,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
+          <t>サテライト</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -6306,7 +6306,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
         </is>
       </c>
     </row>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>塩対応の佐藤さんが俺にだけ甘い</t>
+          <t>佐々木とピーちゃん シーズン２</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -6340,14 +6340,18 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
         </is>
       </c>
     </row>
@@ -6365,7 +6369,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>紫禁・御猫房〜紫禁城猫警備室〜</t>
+          <t>塩対応の佐藤さんが俺にだけ甘い</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -6388,7 +6392,7 @@
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28779</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6410,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>ジャンケットバンク</t>
+          <t>紫禁・御猫房〜紫禁城猫警備室〜</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -6419,21 +6423,17 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28779</t>
         </is>
       </c>
     </row>
@@ -6451,7 +6451,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>朱色の仮面</t>
+          <t>ジャンケットバンク</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6464,17 +6464,21 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr"/>
+          <t>2026年10月～ テレ東系列にて</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6496,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6505,29 +6509,17 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>曲名未発表</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
+          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6537,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>しろたん</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6558,21 +6550,29 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>レスプリ</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
         </is>
       </c>
     </row>
@@ -6590,7 +6590,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>信者ゼロの女神サマと始める異世界攻略</t>
+          <t>しろたん</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6603,12 +6603,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレビ朝日にて</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>HORNETS</t>
+          <t>レスプリ</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -6617,7 +6617,7 @@
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>信者ゼロの女神サマと始める異世界攻略</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6648,33 +6648,21 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>Walls And Bridges</t>
-        </is>
-      </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
-        </is>
-      </c>
-      <c r="K115" t="inlineStr">
-        <is>
-          <t>金環蝕 phenomenal</t>
-        </is>
-      </c>
-      <c r="L115" t="inlineStr">
-        <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>HORNETS</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
         </is>
       </c>
     </row>
@@ -6692,7 +6680,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6700,26 +6688,38 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Walls And Bridges</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>金環蝕 phenomenal</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -6737,7 +6737,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6745,22 +6745,26 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr"/>
+          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>david production</t>
+        </is>
+      </c>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr"/>
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
         </is>
       </c>
     </row>
@@ -6778,7 +6782,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6791,21 +6795,17 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ TOKYO MX・BS11ほか</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>ブリッジ</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
         </is>
       </c>
     </row>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6836,17 +6836,21 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr"/>
+          <t>2026年10月7日（水）～ TOKYO MX・BS11ほか</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -6864,7 +6868,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6877,37 +6881,17 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>OLM</t>
-        </is>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>Let's Go Crazy</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>Baby Canta</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="L120" t="inlineStr">
-        <is>
-          <t>SUPER★DRAGON</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -6925,7 +6909,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6938,17 +6922,37 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
+          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Let's Go Crazy</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6970,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6979,21 +6983,17 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr"/>
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7011,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -7024,12 +7024,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -7056,7 +7056,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7069,37 +7069,21 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>feel.</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>ライアー</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>陽炎</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
+          <t>ENGI</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -7117,7 +7101,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7130,21 +7114,37 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
+          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
+          <t>feel.</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>ライアー</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>陽炎</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>サイダーガール</t>
+        </is>
+      </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
         </is>
       </c>
     </row>
@@ -7162,7 +7162,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7175,12 +7175,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -7189,7 +7189,7 @@
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -7207,7 +7207,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7220,29 +7220,21 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>わたし未来線</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7252,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7278,16 +7270,24 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>わたし未来線</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+        </is>
+      </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -7305,7 +7305,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7313,34 +7313,26 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026年11月6日（金） Prime Videoにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>シンカ</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>Ado</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7350,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7366,26 +7358,34 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年11月6日（金） Prime Videoにて</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
+          <t>Production I.G</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>シンカ</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Ado</t>
+        </is>
+      </c>
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
         </is>
       </c>
     </row>
@@ -7403,7 +7403,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7416,12 +7416,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I131" t="inlineStr"/>
@@ -7430,7 +7430,7 @@
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -7448,7 +7448,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7466,32 +7466,16 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -7509,7 +7493,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7527,16 +7511,32 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7554,7 +7554,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7567,37 +7567,21 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>Ghost Sequence</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t>East Of Eden</t>
-        </is>
-      </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>原子崩し(メルトダウナー)</t>
-        </is>
-      </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
+          <t>C2C</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7615,7 +7599,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7628,29 +7612,37 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年10月9日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="K135" t="inlineStr"/>
-      <c r="L135" t="inlineStr"/>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>原子崩し(メルトダウナー)</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -7668,7 +7660,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7681,17 +7673,29 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>IGNITE</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -7709,7 +7713,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7722,21 +7726,17 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -7754,7 +7754,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7767,17 +7767,21 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -7795,7 +7799,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>dreamland</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7808,7 +7812,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年10月～ ABCテレビ・テレビ朝日ほか</t>
+          <t>2026年秋 フジテレビにて</t>
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
@@ -7818,7 +7822,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28811</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -7836,7 +7840,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>dreamland</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7844,26 +7848,22 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年10月～ ABCテレビ・テレビ朝日ほか</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr"/>
       <c r="I140" t="inlineStr"/>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28811</t>
         </is>
       </c>
     </row>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7889,17 +7889,17 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I141" t="inlineStr"/>
@@ -7908,7 +7908,7 @@
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7939,17 +7939,21 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H142" t="inlineStr"/>
+          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I142" t="inlineStr"/>
       <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -7967,7 +7971,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -7980,7 +7984,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H143" t="inlineStr"/>
@@ -7990,7 +7994,7 @@
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -8008,7 +8012,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -8021,7 +8025,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H144" t="inlineStr"/>
@@ -8031,7 +8035,7 @@
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8053,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8062,21 +8066,17 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8107,29 +8107,21 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8139,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8160,21 +8152,29 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -8192,7 +8192,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8205,12 +8205,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I148" t="inlineStr"/>
@@ -8219,7 +8219,7 @@
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -8237,7 +8237,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8250,12 +8250,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -8264,7 +8264,7 @@
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -8282,7 +8282,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8295,12 +8295,12 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I150" t="inlineStr"/>
@@ -8309,7 +8309,7 @@
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8327,7 +8327,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8340,12 +8340,12 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I151" t="inlineStr"/>
@@ -8354,7 +8354,7 @@
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8372,7 +8372,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8385,29 +8385,21 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8417,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8438,37 +8430,29 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8470,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E154" t="b">
@@ -8499,21 +8483,37 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -8531,7 +8531,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E155" t="b">
@@ -8544,37 +8544,21 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -8592,7 +8576,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E156" t="b">
@@ -8605,21 +8589,37 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8637,7 +8637,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E157" t="b">
@@ -8650,37 +8650,21 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -8698,7 +8682,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E158" t="b">
@@ -8711,21 +8695,37 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr"/>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -8743,11 +8743,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -8756,12 +8756,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
@@ -8770,7 +8770,7 @@
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -8788,11 +8788,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E160" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -8801,17 +8801,21 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ 日本テレビにて</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr"/>
       <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -8829,7 +8833,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E161" t="b">
@@ -8837,12 +8841,12 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月3日（土）～ 日本テレビにて</t>
         </is>
       </c>
       <c r="H161" t="inlineStr"/>
@@ -8851,6 +8855,47 @@
       <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>74</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E162" t="b">
+        <v>0</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -8867,7 +8912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O186"/>
+  <dimension ref="A1:O188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10877,7 +10922,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>84295</v>
+        <v>99818</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -10889,7 +10934,7 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-07-21T09:00:40</t>
+          <t>2026-07-29T09:00:49</t>
         </is>
       </c>
     </row>
@@ -12152,27 +12197,13 @@
           <t>スキマスイッチ</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=xLU_wlNciSI</t>
-        </is>
-      </c>
-      <c r="J54" t="n">
-        <v>1041</v>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>【公式】石森プロ</t>
-        </is>
-      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>2026-07-21T09:01:04</t>
-        </is>
-      </c>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -12278,33 +12309,33 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=BgtayXSaaOI</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>44567</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Hana Hope</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=od3XN58Gnws</t>
         </is>
       </c>
-      <c r="J56" t="n">
-        <v>16719</v>
-      </c>
-      <c r="K56" t="inlineStr">
+      <c r="M56" t="n">
+        <v>32651</v>
+      </c>
+      <c r="N56" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=od3XN58Gnws</t>
-        </is>
-      </c>
-      <c r="M56" t="n">
-        <v>16719</v>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-07-21T09:01:13</t>
+          <t>2026-07-29T09:01:25</t>
         </is>
       </c>
     </row>
@@ -13593,33 +13624,33 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=3uVd4WGNgy0</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>113758</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>えむにみに</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=1tc784esysA</t>
         </is>
       </c>
-      <c r="J77" t="n">
-        <v>7476</v>
-      </c>
-      <c r="K77" t="inlineStr">
+      <c r="M77" t="n">
+        <v>22064</v>
+      </c>
+      <c r="N77" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1tc784esysA</t>
-        </is>
-      </c>
-      <c r="M77" t="n">
-        <v>7476</v>
-      </c>
-      <c r="N77" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-07-21T09:01:25</t>
+          <t>2026-07-29T09:01:38</t>
         </is>
       </c>
     </row>
@@ -14683,15 +14714,15 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k3NwKLjfEOw</t>
+          <t>https://www.youtube.com/watch?v=ZH8xYK5vac0</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>178868</v>
+        <v>120641</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>suis from Yorushika - Topic</t>
+          <t>宝島社公式</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -14700,7 +14731,7 @@
         </is>
       </c>
       <c r="M95" t="n">
-        <v>108510</v>
+        <v>120641</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -14709,7 +14740,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-07-21T09:01:54</t>
+          <t>2026-07-29T09:02:11</t>
         </is>
       </c>
     </row>
@@ -15175,7 +15206,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>36586</v>
+        <v>44952</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -15188,7 +15219,7 @@
         </is>
       </c>
       <c r="M103" t="n">
-        <v>36586</v>
+        <v>44952</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -15197,7 +15228,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-07-21T09:02:13</t>
+          <t>2026-07-29T09:02:31</t>
         </is>
       </c>
     </row>
@@ -15955,7 +15986,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>501334</v>
+        <v>524568</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -15968,7 +15999,7 @@
         </is>
       </c>
       <c r="M115" t="n">
-        <v>501334</v>
+        <v>524568</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -15977,7 +16008,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-07-21T09:02:25</t>
+          <t>2026-07-29T09:02:43</t>
         </is>
       </c>
     </row>
@@ -16352,7 +16383,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>17994</v>
+        <v>20638</v>
       </c>
       <c r="K122" t="inlineStr">
         <is>
@@ -16365,7 +16396,7 @@
         </is>
       </c>
       <c r="M122" t="n">
-        <v>17994</v>
+        <v>20638</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -16374,7 +16405,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-07-21T09:02:49</t>
+          <t>2026-07-29T09:03:07</t>
         </is>
       </c>
     </row>
@@ -18030,7 +18061,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>7627</v>
+        <v>10636</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -18043,7 +18074,7 @@
         </is>
       </c>
       <c r="M150" t="n">
-        <v>7627</v>
+        <v>10636</v>
       </c>
       <c r="N150" t="inlineStr">
         <is>
@@ -18052,7 +18083,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-07-21T09:03:18</t>
+          <t>2026-07-29T09:03:39</t>
         </is>
       </c>
     </row>
@@ -18097,7 +18128,7 @@
         </is>
       </c>
       <c r="J151" t="n">
-        <v>55761</v>
+        <v>58027</v>
       </c>
       <c r="K151" t="inlineStr">
         <is>
@@ -18110,7 +18141,7 @@
         </is>
       </c>
       <c r="M151" t="n">
-        <v>55761</v>
+        <v>58027</v>
       </c>
       <c r="N151" t="inlineStr">
         <is>
@@ -18119,7 +18150,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-07-21T09:03:27</t>
+          <t>2026-07-29T09:03:49</t>
         </is>
       </c>
     </row>
@@ -18207,7 +18238,7 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>186682</v>
+        <v>194933</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
@@ -18220,7 +18251,7 @@
         </is>
       </c>
       <c r="M153" t="n">
-        <v>186682</v>
+        <v>194933</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -18229,7 +18260,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-07-21T09:03:39</t>
+          <t>2026-07-29T09:04:01</t>
         </is>
       </c>
     </row>
@@ -18713,7 +18744,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="D161" t="b">
@@ -18729,21 +18760,35 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>Escape</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>THE RAMPAGE</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr"/>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
+          <t>Kis-My-Ft2</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>51838</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
       <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr"/>
       <c r="N161" t="inlineStr"/>
-      <c r="O161" t="inlineStr"/>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>2026-07-29T09:04:12</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -18756,7 +18801,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D162" t="b">
@@ -18764,7 +18809,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -18772,12 +18817,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>THE RAMPAGE</t>
         </is>
       </c>
       <c r="I162" t="inlineStr"/>
@@ -18807,7 +18852,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -18815,12 +18860,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>krage</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I163" t="inlineStr"/>
@@ -18842,7 +18887,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D164" t="b">
@@ -18850,7 +18895,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -18858,12 +18903,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>amazarashi</t>
+          <t>krage</t>
         </is>
       </c>
       <c r="I164" t="inlineStr"/>
@@ -18885,7 +18930,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D165" t="b">
@@ -18901,12 +18946,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>amazarashi</t>
         </is>
       </c>
       <c r="I165" t="inlineStr"/>
@@ -18928,7 +18973,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D166" t="b">
@@ -18936,7 +18981,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -18944,12 +18989,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -18971,7 +19016,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D167" t="b">
@@ -18979,7 +19024,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -18987,12 +19032,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -19014,7 +19059,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D168" t="b">
@@ -19030,12 +19075,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -19057,7 +19102,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D169" t="b">
@@ -19073,12 +19118,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>跡部景吾＆忍足侑士</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -19100,7 +19145,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D170" t="b">
@@ -19116,45 +19161,21 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J170" t="n">
-        <v>682181</v>
-      </c>
-      <c r="K170" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L170" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M170" t="n">
-        <v>682181</v>
-      </c>
-      <c r="N170" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O170" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:16:41</t>
-        </is>
-      </c>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -19167,7 +19188,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D171" t="b">
@@ -19183,45 +19204,21 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="J171" t="n">
-        <v>372964</v>
-      </c>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L171" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M171" t="n">
-        <v>372964</v>
-      </c>
-      <c r="N171" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O171" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:16:49</t>
-        </is>
-      </c>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -19234,7 +19231,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D172" t="b">
@@ -19242,7 +19239,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -19250,21 +19247,45 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr"/>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>682181</v>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M172" t="n">
+        <v>682181</v>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:16:41</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -19277,7 +19298,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -19285,7 +19306,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -19293,21 +19314,45 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr"/>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
-      <c r="M173" t="inlineStr"/>
-      <c r="N173" t="inlineStr"/>
-      <c r="O173" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J173" t="n">
+        <v>372964</v>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M173" t="n">
+        <v>372964</v>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:16:49</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -19320,7 +19365,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -19328,7 +19373,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -19336,12 +19381,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -19363,7 +19408,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -19371,7 +19416,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -19379,12 +19424,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I175" t="inlineStr"/>
@@ -19406,7 +19451,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -19422,12 +19467,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -19449,7 +19494,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -19465,12 +19510,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -19492,7 +19537,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -19508,35 +19553,21 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=wDY2s73E8DM</t>
-        </is>
-      </c>
-      <c r="J178" t="n">
-        <v>84</v>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>テレビ公式</t>
-        </is>
-      </c>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr">
-        <is>
-          <t>2026-07-27T09:09:53</t>
-        </is>
-      </c>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -19549,7 +19580,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -19557,7 +19588,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -19565,45 +19596,21 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I179" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J179" t="n">
-        <v>2587</v>
-      </c>
-      <c r="K179" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L179" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M179" t="n">
-        <v>2587</v>
-      </c>
-      <c r="N179" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O179" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:17:34</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -19616,7 +19623,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -19632,25 +19639,25 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>JO1</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=wDY2s73E8DM</t>
         </is>
       </c>
       <c r="J180" t="n">
-        <v>106403</v>
+        <v>84</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+          <t>テレビ公式</t>
         </is>
       </c>
       <c r="L180" t="inlineStr"/>
@@ -19658,7 +19665,7 @@
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-07-22T09:17:48</t>
+          <t>2026-07-27T09:09:53</t>
         </is>
       </c>
     </row>
@@ -19673,7 +19680,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -19689,43 +19696,43 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J181" t="n">
-        <v>298421</v>
+        <v>2587</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
+          <t>Anime Trailer アニメ</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="M181" t="n">
-        <v>298421</v>
+        <v>2587</v>
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
+          <t>Anime Trailer アニメ</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-07-27T09:10:03</t>
+          <t>2026-07-22T09:17:34</t>
         </is>
       </c>
     </row>
@@ -19740,7 +19747,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -19748,7 +19755,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -19756,43 +19763,33 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J182" t="n">
-        <v>298421</v>
+        <v>106403</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L182" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M182" t="n">
-        <v>298421</v>
-      </c>
-      <c r="N182" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-07-27T09:10:13</t>
+          <t>2026-07-22T09:17:48</t>
         </is>
       </c>
     </row>
@@ -19807,7 +19804,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -19823,21 +19820,45 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr"/>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
-      <c r="M183" t="inlineStr"/>
-      <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>298421</v>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M183" t="n">
+        <v>298421</v>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>2026-07-27T09:10:03</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19850,7 +19871,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -19866,21 +19887,45 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr"/>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
-      <c r="M184" t="inlineStr"/>
-      <c r="N184" t="inlineStr"/>
-      <c r="O184" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J184" t="n">
+        <v>298421</v>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M184" t="n">
+        <v>298421</v>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>2026-07-27T09:10:13</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19893,7 +19938,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -19909,45 +19954,21 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J185" t="n">
-        <v>776489</v>
-      </c>
-      <c r="K185" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L185" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M185" t="n">
-        <v>367020</v>
-      </c>
-      <c r="N185" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O185" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:18:09</t>
-        </is>
-      </c>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -19960,7 +19981,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -19976,41 +19997,151 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D187" t="b">
+        <v>0</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>1</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J187" t="n">
+        <v>776489</v>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M187" t="n">
+        <v>367020</v>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D188" t="b">
+        <v>0</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>1</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr">
+      <c r="H188" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I186" t="inlineStr">
+      <c r="I188" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="J186" t="n">
+      <c r="J188" t="n">
         <v>384697</v>
       </c>
-      <c r="K186" t="inlineStr">
+      <c r="K188" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L186" t="inlineStr">
+      <c r="L188" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M186" t="n">
+      <c r="M188" t="n">
         <v>384697</v>
       </c>
-      <c r="N186" t="inlineStr">
+      <c r="N188" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O186" t="inlineStr">
+      <c r="O188" t="inlineStr">
         <is>
           <t>2026-07-22T09:18:19</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-30
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -5981,7 +5981,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月6日（火）～ TOKYO MX・MBS ほか</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -9200,7 +9200,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>62106</v>
+        <v>75815</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9213,7 +9213,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>62106</v>
+        <v>75815</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -9222,7 +9222,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-07-22T09:01:15</t>
+          <t>2026-07-30T09:00:33</t>
         </is>
       </c>
     </row>
@@ -9310,7 +9310,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>159820</v>
+        <v>165237</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>159820</v>
+        <v>165237</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -9332,7 +9332,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-07-22T09:01:27</t>
+          <t>2026-07-30T09:00:45</t>
         </is>
       </c>
     </row>
@@ -9373,33 +9373,33 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=ItNWR7OPAN4</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>1702305</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>WOLF HOWL HARMONY</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=WM9BicFEhKs</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>17391</v>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="n">
+        <v>20069</v>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>ヤンジャン漫画TV【集英社ヤングジャンプ公式】</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WM9BicFEhKs</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>17391</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>ヤンジャン漫画TV【集英社ヤングジャンプ公式】</t>
-        </is>
-      </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-07-22T09:01:37</t>
+          <t>2026-07-30T09:00:54</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>61861</v>
+        <v>68688</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -9457,7 +9457,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>61861</v>
+        <v>68688</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-07-22T09:01:47</t>
+          <t>2026-07-30T09:01:03</t>
         </is>
       </c>
     </row>
@@ -9511,7 +9511,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>31053</v>
+        <v>47083</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -9524,7 +9524,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>28791</v>
+        <v>30331</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -9533,7 +9533,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-07-22T09:01:56</t>
+          <t>2026-07-30T09:01:12</t>
         </is>
       </c>
     </row>
@@ -9578,7 +9578,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>547354</v>
+        <v>579478</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -9591,7 +9591,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>104573</v>
+        <v>113583</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -9600,7 +9600,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-07-22T09:02:05</t>
+          <t>2026-07-30T09:01:21</t>
         </is>
       </c>
     </row>
@@ -9688,7 +9688,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>99639</v>
+        <v>130245</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -9700,7 +9700,7 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-07-22T09:02:34</t>
+          <t>2026-07-30T09:01:52</t>
         </is>
       </c>
     </row>
@@ -10056,7 +10056,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>326197</v>
+        <v>367767</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -10069,7 +10069,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>231732</v>
+        <v>263378</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -10078,7 +10078,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-07-22T09:02:46</t>
+          <t>2026-07-30T09:02:04</t>
         </is>
       </c>
     </row>
@@ -10123,7 +10123,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>184826</v>
+        <v>356064</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -10136,7 +10136,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>105628</v>
+        <v>115048</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -10145,7 +10145,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-07-22T09:02:56</t>
+          <t>2026-07-30T09:02:13</t>
         </is>
       </c>
     </row>
@@ -10257,7 +10257,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>379715</v>
+        <v>385557</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -10270,7 +10270,7 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>7359</v>
+        <v>9945</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -10279,7 +10279,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-07-22T09:03:05</t>
+          <t>2026-07-30T09:02:22</t>
         </is>
       </c>
     </row>
@@ -10367,7 +10367,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>60541</v>
+        <v>67522</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -10380,7 +10380,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>60541</v>
+        <v>67522</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -10389,7 +10389,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-07-22T09:03:16</t>
+          <t>2026-07-30T09:02:39</t>
         </is>
       </c>
     </row>
@@ -10434,7 +10434,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>155830</v>
+        <v>161920</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -10447,7 +10447,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>155830</v>
+        <v>161920</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -10456,7 +10456,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-07-22T09:03:26</t>
+          <t>2026-07-30T09:02:48</t>
         </is>
       </c>
     </row>
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>2090790</v>
+        <v>2492291</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -10514,7 +10514,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>38860</v>
+        <v>45168</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-07-22T09:03:34</t>
+          <t>2026-07-30T09:02:57</t>
         </is>
       </c>
     </row>
@@ -10568,7 +10568,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>706561</v>
+        <v>829762</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>44003</v>
+        <v>50172</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -10590,7 +10590,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-07-22T09:03:44</t>
+          <t>2026-07-30T09:03:06</t>
         </is>
       </c>
     </row>
@@ -10784,33 +10784,33 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=1T92vMhjHtA</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>111768</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>sajou no hana Official Channel</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=bszg61aM_7E</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>50384</v>
-      </c>
-      <c r="K31" t="inlineStr">
+      <c r="M31" t="n">
+        <v>62189</v>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=bszg61aM_7E</t>
-        </is>
-      </c>
-      <c r="M31" t="n">
-        <v>50384</v>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-07-22T09:03:53</t>
+          <t>2026-07-30T09:03:15</t>
         </is>
       </c>
     </row>
@@ -10851,11 +10851,11 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=cBhaKIqvUrQ</t>
+          <t>https://www.youtube.com/watch?v=5cXLBCc_O5U</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>6419043</v>
+        <v>1277161</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -10864,11 +10864,11 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=cBhaKIqvUrQ</t>
+          <t>https://www.youtube.com/watch?v=5cXLBCc_O5U</t>
         </is>
       </c>
       <c r="M32" t="n">
-        <v>6419043</v>
+        <v>1277161</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -10877,7 +10877,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-07-22T09:04:02</t>
+          <t>2026-07-30T09:03:24</t>
         </is>
       </c>
     </row>
@@ -11256,7 +11256,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>252886</v>
+        <v>307087</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -11269,7 +11269,7 @@
         </is>
       </c>
       <c r="M39" t="n">
-        <v>252886</v>
+        <v>307087</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -11278,7 +11278,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-07-22T09:04:22</t>
+          <t>2026-07-30T09:03:47</t>
         </is>
       </c>
     </row>
@@ -11323,7 +11323,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>39221</v>
+        <v>45960</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>39221</v>
+        <v>45960</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -11345,7 +11345,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-07-22T09:04:32</t>
+          <t>2026-07-30T09:03:55</t>
         </is>
       </c>
     </row>
@@ -11457,7 +11457,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>1644212</v>
+        <v>2006628</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -11470,7 +11470,7 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>240187</v>
+        <v>263466</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -11479,7 +11479,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-07-22T09:04:41</t>
+          <t>2026-07-30T09:04:04</t>
         </is>
       </c>
     </row>
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1828287</v>
+        <v>1837473</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -11537,7 +11537,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>1828287</v>
+        <v>1837473</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -11546,7 +11546,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-07-22T09:04:50</t>
+          <t>2026-07-30T09:04:14</t>
         </is>
       </c>
     </row>
@@ -11591,7 +11591,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1828287</v>
+        <v>1837473</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -11604,7 +11604,7 @@
         </is>
       </c>
       <c r="M44" t="n">
-        <v>413118</v>
+        <v>416316</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -11613,7 +11613,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-07-22T09:05:01</t>
+          <t>2026-07-30T09:04:23</t>
         </is>
       </c>
     </row>
@@ -11725,7 +11725,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>14127</v>
+        <v>16467</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -11738,7 +11738,7 @@
         </is>
       </c>
       <c r="M46" t="n">
-        <v>14127</v>
+        <v>16467</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -11747,7 +11747,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-07-22T09:05:10</t>
+          <t>2026-07-30T09:04:32</t>
         </is>
       </c>
     </row>
@@ -11792,7 +11792,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>528804</v>
+        <v>664554</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -11805,7 +11805,7 @@
         </is>
       </c>
       <c r="M47" t="n">
-        <v>138686</v>
+        <v>173187</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -11814,7 +11814,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-07-22T09:05:19</t>
+          <t>2026-07-30T09:04:40</t>
         </is>
       </c>
     </row>
@@ -11859,7 +11859,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>4777256</v>
+        <v>4795540</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -11872,7 +11872,7 @@
         </is>
       </c>
       <c r="M48" t="n">
-        <v>19472</v>
+        <v>24188</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -11881,7 +11881,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-07-22T09:05:29</t>
+          <t>2026-07-30T09:04:49</t>
         </is>
       </c>
     </row>
@@ -11926,7 +11926,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>64540</v>
+        <v>72777</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -11939,7 +11939,7 @@
         </is>
       </c>
       <c r="M49" t="n">
-        <v>64540</v>
+        <v>72777</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -11948,7 +11948,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-07-22T09:05:38</t>
+          <t>2026-07-30T09:04:57</t>
         </is>
       </c>
     </row>
@@ -11993,7 +11993,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>5343</v>
+        <v>6640</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -12006,7 +12006,7 @@
         </is>
       </c>
       <c r="M50" t="n">
-        <v>13374</v>
+        <v>15978</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -12015,7 +12015,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-07-22T09:05:47</t>
+          <t>2026-07-30T09:05:06</t>
         </is>
       </c>
     </row>
@@ -12142,23 +12142,33 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=wc1Npu2_IFs</t>
+          <t>https://www.youtube.com/watch?v=5d81RgISG5o</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>37458</v>
+        <v>65904</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>杏子</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+          <t>【公式】石森プロ</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5d81RgISG5o</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>65904</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>【公式】石森プロ</t>
+        </is>
+      </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-07-22T09:06:09</t>
+          <t>2026-07-30T09:05:21</t>
         </is>
       </c>
     </row>
@@ -12246,7 +12256,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>280363</v>
+        <v>332179</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -12259,7 +12269,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>334286</v>
+        <v>337243</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -12268,7 +12278,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-07-22T09:06:18</t>
+          <t>2026-07-30T09:05:38</t>
         </is>
       </c>
     </row>
@@ -12380,7 +12390,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>291332</v>
+        <v>361399</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -12393,7 +12403,7 @@
         </is>
       </c>
       <c r="M57" t="n">
-        <v>24799</v>
+        <v>33132</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -12402,7 +12412,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-07-22T09:06:28</t>
+          <t>2026-07-30T09:05:47</t>
         </is>
       </c>
     </row>
@@ -12514,7 +12524,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>6493879</v>
+        <v>6532226</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -12527,7 +12537,7 @@
         </is>
       </c>
       <c r="M59" t="n">
-        <v>723496</v>
+        <v>742066</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -12536,7 +12546,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-07-22T09:06:37</t>
+          <t>2026-07-30T09:05:56</t>
         </is>
       </c>
     </row>
@@ -12581,7 +12591,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>190059</v>
+        <v>265765</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -12594,7 +12604,7 @@
         </is>
       </c>
       <c r="M60" t="n">
-        <v>57839</v>
+        <v>69448</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -12603,7 +12613,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-07-22T09:06:46</t>
+          <t>2026-07-30T09:06:06</t>
         </is>
       </c>
     </row>
@@ -12648,7 +12658,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>56724</v>
+        <v>59772</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -12661,7 +12671,7 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>56724</v>
+        <v>59772</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -12670,7 +12680,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-07-22T09:06:54</t>
+          <t>2026-07-30T09:06:14</t>
         </is>
       </c>
     </row>
@@ -12715,7 +12725,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>8390</v>
+        <v>9947</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -12728,7 +12738,7 @@
         </is>
       </c>
       <c r="M62" t="n">
-        <v>8390</v>
+        <v>9947</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -12737,7 +12747,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:03</t>
+          <t>2026-07-30T09:06:22</t>
         </is>
       </c>
     </row>
@@ -12868,11 +12878,11 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>4311589</v>
+        <v>4443835</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>乃紫(noa)</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -12881,7 +12891,7 @@
         </is>
       </c>
       <c r="M65" t="n">
-        <v>1957977</v>
+        <v>2008367</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -12890,7 +12900,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:12</t>
+          <t>2026-07-30T09:06:31</t>
         </is>
       </c>
     </row>
@@ -12935,7 +12945,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>246135</v>
+        <v>288816</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -12948,7 +12958,7 @@
         </is>
       </c>
       <c r="M66" t="n">
-        <v>246135</v>
+        <v>288816</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -12957,7 +12967,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:21</t>
+          <t>2026-07-30T09:06:40</t>
         </is>
       </c>
     </row>
@@ -12998,33 +13008,33 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=ZUTDe90QrsU</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>310919</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>PAS TASTA</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=A6aH9jPW8ZY</t>
         </is>
       </c>
-      <c r="J67" t="n">
-        <v>302467</v>
-      </c>
-      <c r="K67" t="inlineStr">
+      <c r="M67" t="n">
+        <v>309249</v>
+      </c>
+      <c r="N67" t="inlineStr">
         <is>
           <t>SHOCHIKU anime Channel</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=A6aH9jPW8ZY</t>
-        </is>
-      </c>
-      <c r="M67" t="n">
-        <v>302467</v>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>SHOCHIKU anime Channel</t>
-        </is>
-      </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:30</t>
+          <t>2026-07-30T09:06:50</t>
         </is>
       </c>
     </row>
@@ -13136,7 +13146,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>20909</v>
+        <v>26099</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -13149,7 +13159,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>20909</v>
+        <v>26099</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -13158,7 +13168,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:39</t>
+          <t>2026-07-30T09:06:59</t>
         </is>
       </c>
     </row>
@@ -13203,7 +13213,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>6846</v>
+        <v>8238</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -13216,7 +13226,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>6846</v>
+        <v>8238</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -13225,7 +13235,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:48</t>
+          <t>2026-07-30T09:07:08</t>
         </is>
       </c>
     </row>
@@ -13270,7 +13280,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>109896</v>
+        <v>129334</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -13283,7 +13293,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>109896</v>
+        <v>129334</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -13292,7 +13302,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:57</t>
+          <t>2026-07-30T09:07:17</t>
         </is>
       </c>
     </row>
@@ -13333,33 +13343,33 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=0cZFkZd2-CQ</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>17164</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>halca Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=GKtdRThIuuE</t>
         </is>
       </c>
-      <c r="J72" t="n">
-        <v>14881</v>
-      </c>
-      <c r="K72" t="inlineStr">
+      <c r="M72" t="n">
+        <v>17141</v>
+      </c>
+      <c r="N72" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GKtdRThIuuE</t>
-        </is>
-      </c>
-      <c r="M72" t="n">
-        <v>14881</v>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-07-22T09:08:08</t>
+          <t>2026-07-30T09:07:27</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13705,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>759690</v>
+        <v>762820</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -13708,7 +13718,7 @@
         </is>
       </c>
       <c r="M78" t="n">
-        <v>759690</v>
+        <v>762820</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -13717,7 +13727,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-07-22T09:08:20</t>
+          <t>2026-07-30T09:07:38</t>
         </is>
       </c>
     </row>
@@ -13762,7 +13772,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>173022</v>
+        <v>175406</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -13775,7 +13785,7 @@
         </is>
       </c>
       <c r="M79" t="n">
-        <v>173022</v>
+        <v>175406</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -13784,7 +13794,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-07-22T09:08:29</t>
+          <t>2026-07-30T09:07:49</t>
         </is>
       </c>
     </row>
@@ -13829,7 +13839,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>337585</v>
+        <v>356222</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -13841,7 +13851,7 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-07-22T09:08:48</t>
+          <t>2026-07-30T09:08:06</t>
         </is>
       </c>
     </row>
@@ -13929,7 +13939,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>219613</v>
+        <v>222273</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -13942,7 +13952,7 @@
         </is>
       </c>
       <c r="M82" t="n">
-        <v>76983</v>
+        <v>84049</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -13951,7 +13961,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-07-22T09:08:59</t>
+          <t>2026-07-30T09:08:18</t>
         </is>
       </c>
     </row>
@@ -14063,7 +14073,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>999686</v>
+        <v>1197912</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -14076,7 +14086,7 @@
         </is>
       </c>
       <c r="M84" t="n">
-        <v>999686</v>
+        <v>1197912</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -14085,7 +14095,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-07-22T09:09:08</t>
+          <t>2026-07-30T09:08:26</t>
         </is>
       </c>
     </row>
@@ -14130,7 +14140,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>209282</v>
+        <v>296529</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -14143,7 +14153,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>202801</v>
+        <v>238009</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -14152,7 +14162,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-07-22T09:09:18</t>
+          <t>2026-07-30T09:08:35</t>
         </is>
       </c>
     </row>
@@ -14580,11 +14590,11 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-UMzc7BI6y4</t>
+          <t>https://www.youtube.com/watch?v=PX-b7KO3HOw</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>76156</v>
+        <v>99642</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -14593,11 +14603,11 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-UMzc7BI6y4</t>
+          <t>https://www.youtube.com/watch?v=PX-b7KO3HOw</t>
         </is>
       </c>
       <c r="M93" t="n">
-        <v>76156</v>
+        <v>99642</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -14606,7 +14616,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-07-22T09:09:46</t>
+          <t>2026-07-30T09:09:05</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14661,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>34898</v>
+        <v>41577</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -14664,7 +14674,7 @@
         </is>
       </c>
       <c r="M94" t="n">
-        <v>34898</v>
+        <v>41577</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -14673,7 +14683,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-07-22T09:09:54</t>
+          <t>2026-07-30T09:09:14</t>
         </is>
       </c>
     </row>
@@ -14938,7 +14948,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>447499</v>
+        <v>455618</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -14951,7 +14961,7 @@
         </is>
       </c>
       <c r="M99" t="n">
-        <v>447499</v>
+        <v>455618</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -14960,7 +14970,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-07-22T09:10:15</t>
+          <t>2026-07-30T09:09:33</t>
         </is>
       </c>
     </row>
@@ -15005,7 +15015,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>368945</v>
+        <v>388622</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -15018,7 +15028,7 @@
         </is>
       </c>
       <c r="M100" t="n">
-        <v>368945</v>
+        <v>388622</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -15027,7 +15037,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-07-22T09:10:24</t>
+          <t>2026-07-30T09:09:42</t>
         </is>
       </c>
     </row>
@@ -15072,7 +15082,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>363595</v>
+        <v>376687</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -15085,7 +15095,7 @@
         </is>
       </c>
       <c r="M101" t="n">
-        <v>333028</v>
+        <v>341177</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -15094,7 +15104,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-07-22T09:10:33</t>
+          <t>2026-07-30T09:09:52</t>
         </is>
       </c>
     </row>
@@ -15139,7 +15149,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>59349</v>
+        <v>62622</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -15152,7 +15162,7 @@
         </is>
       </c>
       <c r="M102" t="n">
-        <v>59349</v>
+        <v>62622</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -15161,7 +15171,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-07-22T09:10:43</t>
+          <t>2026-07-30T09:10:00</t>
         </is>
       </c>
     </row>
@@ -15273,7 +15283,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>48160</v>
+        <v>62141</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -15286,7 +15296,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>48160</v>
+        <v>62141</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -15295,7 +15305,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-07-22T09:10:52</t>
+          <t>2026-07-30T09:10:09</t>
         </is>
       </c>
     </row>
@@ -15584,7 +15594,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>61093</v>
+        <v>76795</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -15597,7 +15607,7 @@
         </is>
       </c>
       <c r="M109" t="n">
-        <v>61093</v>
+        <v>76795</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -15606,7 +15616,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-07-22T09:11:03</t>
+          <t>2026-07-30T09:10:20</t>
         </is>
       </c>
     </row>
@@ -15718,7 +15728,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>76020</v>
+        <v>89616</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -15731,7 +15741,7 @@
         </is>
       </c>
       <c r="M111" t="n">
-        <v>28300</v>
+        <v>32482</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -15740,7 +15750,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-07-22T09:11:12</t>
+          <t>2026-07-30T09:10:29</t>
         </is>
       </c>
     </row>
@@ -15785,7 +15795,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>12625</v>
+        <v>15035</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -15798,7 +15808,7 @@
         </is>
       </c>
       <c r="M112" t="n">
-        <v>12625</v>
+        <v>15035</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -15807,7 +15817,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-07-22T09:11:21</t>
+          <t>2026-07-30T09:10:37</t>
         </is>
       </c>
     </row>
@@ -15852,7 +15862,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>1161574</v>
+        <v>1967511</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -15865,7 +15875,7 @@
         </is>
       </c>
       <c r="M113" t="n">
-        <v>170674</v>
+        <v>219062</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -15874,7 +15884,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-07-22T09:11:31</t>
+          <t>2026-07-30T09:10:47</t>
         </is>
       </c>
     </row>
@@ -16159,11 +16169,11 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=g2iWIWqJ39s</t>
+          <t>https://www.youtube.com/watch?v=IJONbpfIlUg</t>
         </is>
       </c>
       <c r="J118" t="n">
-        <v>2044408</v>
+        <v>1959323</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -16172,20 +16182,20 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TGTYrh-kFbA</t>
+          <t>https://www.youtube.com/watch?v=9idm6v9jNbg</t>
         </is>
       </c>
       <c r="M118" t="n">
-        <v>3261209</v>
+        <v>962806</v>
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>アニプレックス チャンネル</t>
+          <t>『BLEACH』アニメ公式チャンネル</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-07-22T09:11:50</t>
+          <t>2026-07-30T09:10:58</t>
         </is>
       </c>
     </row>
@@ -16230,7 +16240,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>2044408</v>
+        <v>2064700</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -16239,11 +16249,11 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=O63cbh6EyQ8</t>
+          <t>https://www.youtube.com/watch?v=E2c3V6nxjCw</t>
         </is>
       </c>
       <c r="M119" t="n">
-        <v>294037</v>
+        <v>770979</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -16252,7 +16262,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-07-22T09:12:00</t>
+          <t>2026-07-30T09:11:07</t>
         </is>
       </c>
     </row>
@@ -16593,7 +16603,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>90868</v>
+        <v>97123</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -16606,7 +16616,7 @@
         </is>
       </c>
       <c r="M126" t="n">
-        <v>90868</v>
+        <v>97123</v>
       </c>
       <c r="N126" t="inlineStr">
         <is>
@@ -16615,7 +16625,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-07-22T09:12:27</t>
+          <t>2026-07-30T09:11:34</t>
         </is>
       </c>
     </row>
@@ -16660,7 +16670,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>233999</v>
+        <v>288696</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -16673,7 +16683,7 @@
         </is>
       </c>
       <c r="M127" t="n">
-        <v>71495</v>
+        <v>79202</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -16682,7 +16692,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-07-22T09:12:34</t>
+          <t>2026-07-30T09:11:41</t>
         </is>
       </c>
     </row>
@@ -16727,7 +16737,7 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>638988</v>
+        <v>641016</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -16740,7 +16750,7 @@
         </is>
       </c>
       <c r="M128" t="n">
-        <v>335415</v>
+        <v>385763</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -16749,7 +16759,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-07-22T09:12:44</t>
+          <t>2026-07-30T09:11:51</t>
         </is>
       </c>
     </row>
@@ -16794,7 +16804,7 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>638997</v>
+        <v>641017</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -16807,7 +16817,7 @@
         </is>
       </c>
       <c r="M129" t="n">
-        <v>75656</v>
+        <v>89176</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -16816,7 +16826,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-07-22T09:12:53</t>
+          <t>2026-07-30T09:12:00</t>
         </is>
       </c>
     </row>
@@ -17010,11 +17020,11 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=hZ6TnKvB2rc</t>
+          <t>https://www.youtube.com/watch?v=mUZEnAeUvgA</t>
         </is>
       </c>
       <c r="J133" t="n">
-        <v>12320622</v>
+        <v>7023574</v>
       </c>
       <c r="K133" t="inlineStr">
         <is>
@@ -17027,7 +17037,7 @@
         </is>
       </c>
       <c r="M133" t="n">
-        <v>2518108</v>
+        <v>2543471</v>
       </c>
       <c r="N133" t="inlineStr">
         <is>
@@ -17036,7 +17046,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-07-22T09:13:12</t>
+          <t>2026-07-30T09:12:16</t>
         </is>
       </c>
     </row>
@@ -17081,7 +17091,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>1366866</v>
+        <v>1375213</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -17094,7 +17104,7 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>2518108</v>
+        <v>2543471</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -17103,7 +17113,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-07-22T09:13:30</t>
+          <t>2026-07-30T09:12:34</t>
         </is>
       </c>
     </row>
@@ -17148,7 +17158,7 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>42584</v>
+        <v>44830</v>
       </c>
       <c r="K135" t="inlineStr">
         <is>
@@ -17161,7 +17171,7 @@
         </is>
       </c>
       <c r="M135" t="n">
-        <v>7672</v>
+        <v>12353</v>
       </c>
       <c r="N135" t="inlineStr">
         <is>
@@ -17170,7 +17180,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-07-22T09:13:39</t>
+          <t>2026-07-30T09:12:43</t>
         </is>
       </c>
     </row>
@@ -17282,7 +17292,7 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>1712928</v>
+        <v>2348041</v>
       </c>
       <c r="K137" t="inlineStr">
         <is>
@@ -17295,7 +17305,7 @@
         </is>
       </c>
       <c r="M137" t="n">
-        <v>1087035</v>
+        <v>1446845</v>
       </c>
       <c r="N137" t="inlineStr">
         <is>
@@ -17304,7 +17314,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-07-22T09:13:49</t>
+          <t>2026-07-30T09:12:52</t>
         </is>
       </c>
     </row>
@@ -17349,7 +17359,7 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>1087035</v>
+        <v>1446845</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
@@ -17362,7 +17372,7 @@
         </is>
       </c>
       <c r="M138" t="n">
-        <v>486862</v>
+        <v>559411</v>
       </c>
       <c r="N138" t="inlineStr">
         <is>
@@ -17371,7 +17381,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-07-22T09:14:07</t>
+          <t>2026-07-30T09:13:11</t>
         </is>
       </c>
     </row>
@@ -17416,7 +17426,7 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>43164</v>
+        <v>47184</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -17428,7 +17438,7 @@
       <c r="N139" t="inlineStr"/>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-07-22T09:14:30</t>
+          <t>2026-07-30T09:13:34</t>
         </is>
       </c>
     </row>
@@ -17607,7 +17617,7 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>613244</v>
+        <v>615432</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
@@ -17620,7 +17630,7 @@
         </is>
       </c>
       <c r="M142" t="n">
-        <v>613244</v>
+        <v>615432</v>
       </c>
       <c r="N142" t="inlineStr">
         <is>
@@ -17629,7 +17639,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-07-22T09:14:40</t>
+          <t>2026-07-30T09:13:43</t>
         </is>
       </c>
     </row>
@@ -17670,11 +17680,11 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
         </is>
       </c>
       <c r="J143" t="n">
-        <v>81043</v>
+        <v>76056</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -17687,7 +17697,7 @@
         </is>
       </c>
       <c r="M143" t="n">
-        <v>75564</v>
+        <v>76056</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -17696,7 +17706,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-07-22T09:14:50</t>
+          <t>2026-07-30T09:13:52</t>
         </is>
       </c>
     </row>
@@ -17741,7 +17751,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>9499221</v>
+        <v>9514127</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -17754,7 +17764,7 @@
         </is>
       </c>
       <c r="M144" t="n">
-        <v>155923</v>
+        <v>157069</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -17763,7 +17773,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-07-22T09:14:59</t>
+          <t>2026-07-30T09:14:02</t>
         </is>
       </c>
     </row>
@@ -17808,7 +17818,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>81036</v>
+        <v>81672</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -17821,7 +17831,7 @@
         </is>
       </c>
       <c r="M145" t="n">
-        <v>81036</v>
+        <v>81672</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -17830,7 +17840,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-07-22T09:15:08</t>
+          <t>2026-07-30T09:14:11</t>
         </is>
       </c>
     </row>
@@ -18372,7 +18382,7 @@
         </is>
       </c>
       <c r="J155" t="n">
-        <v>703321</v>
+        <v>778659</v>
       </c>
       <c r="K155" t="inlineStr">
         <is>
@@ -18385,7 +18395,7 @@
         </is>
       </c>
       <c r="M155" t="n">
-        <v>703321</v>
+        <v>778659</v>
       </c>
       <c r="N155" t="inlineStr">
         <is>
@@ -18394,7 +18404,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-07-22T09:15:29</t>
+          <t>2026-07-30T09:14:33</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18449,7 @@
         </is>
       </c>
       <c r="J156" t="n">
-        <v>165088</v>
+        <v>185276</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18452,7 +18462,7 @@
         </is>
       </c>
       <c r="M156" t="n">
-        <v>66754</v>
+        <v>73980</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -18461,7 +18471,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-07-22T09:15:38</t>
+          <t>2026-07-30T09:14:42</t>
         </is>
       </c>
     </row>
@@ -18573,7 +18583,7 @@
         </is>
       </c>
       <c r="J158" t="n">
-        <v>320459</v>
+        <v>323046</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18586,7 +18596,7 @@
         </is>
       </c>
       <c r="M158" t="n">
-        <v>320459</v>
+        <v>323046</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -18595,7 +18605,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-07-22T09:15:48</t>
+          <t>2026-07-30T09:14:51</t>
         </is>
       </c>
     </row>
@@ -18707,7 +18717,7 @@
         </is>
       </c>
       <c r="J160" t="n">
-        <v>594681</v>
+        <v>616872</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -18720,7 +18730,7 @@
         </is>
       </c>
       <c r="M160" t="n">
-        <v>594681</v>
+        <v>616872</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -18729,7 +18739,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-07-22T09:15:57</t>
+          <t>2026-07-30T09:15:00</t>
         </is>
       </c>
     </row>
@@ -19261,7 +19271,7 @@
         </is>
       </c>
       <c r="J172" t="n">
-        <v>682181</v>
+        <v>688952</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -19274,7 +19284,7 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>682181</v>
+        <v>688952</v>
       </c>
       <c r="N172" t="inlineStr">
         <is>
@@ -19283,7 +19293,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-07-22T09:16:41</t>
+          <t>2026-07-30T09:15:56</t>
         </is>
       </c>
     </row>
@@ -19328,7 +19338,7 @@
         </is>
       </c>
       <c r="J173" t="n">
-        <v>372964</v>
+        <v>378322</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -19341,7 +19351,7 @@
         </is>
       </c>
       <c r="M173" t="n">
-        <v>372964</v>
+        <v>378322</v>
       </c>
       <c r="N173" t="inlineStr">
         <is>
@@ -19350,7 +19360,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-07-22T09:16:49</t>
+          <t>2026-07-30T09:16:05</t>
         </is>
       </c>
     </row>
@@ -19710,7 +19720,7 @@
         </is>
       </c>
       <c r="J181" t="n">
-        <v>2587</v>
+        <v>3017</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
@@ -19723,7 +19733,7 @@
         </is>
       </c>
       <c r="M181" t="n">
-        <v>2587</v>
+        <v>3017</v>
       </c>
       <c r="N181" t="inlineStr">
         <is>
@@ -19732,7 +19742,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-07-22T09:17:34</t>
+          <t>2026-07-30T09:16:51</t>
         </is>
       </c>
     </row>
@@ -19777,7 +19787,7 @@
         </is>
       </c>
       <c r="J182" t="n">
-        <v>106403</v>
+        <v>106729</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
@@ -19789,7 +19799,7 @@
       <c r="N182" t="inlineStr"/>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-07-22T09:17:48</t>
+          <t>2026-07-30T09:17:06</t>
         </is>
       </c>
     </row>
@@ -20054,7 +20064,7 @@
         </is>
       </c>
       <c r="J187" t="n">
-        <v>776489</v>
+        <v>828328</v>
       </c>
       <c r="K187" t="inlineStr">
         <is>
@@ -20067,7 +20077,7 @@
         </is>
       </c>
       <c r="M187" t="n">
-        <v>367020</v>
+        <v>375681</v>
       </c>
       <c r="N187" t="inlineStr">
         <is>
@@ -20076,7 +20086,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-07-22T09:18:09</t>
+          <t>2026-07-30T09:17:26</t>
         </is>
       </c>
     </row>
@@ -20121,7 +20131,7 @@
         </is>
       </c>
       <c r="J188" t="n">
-        <v>384697</v>
+        <v>391042</v>
       </c>
       <c r="K188" t="inlineStr">
         <is>
@@ -20134,7 +20144,7 @@
         </is>
       </c>
       <c r="M188" t="n">
-        <v>384697</v>
+        <v>391042</v>
       </c>
       <c r="N188" t="inlineStr">
         <is>
@@ -20143,7 +20153,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-07-22T09:18:19</t>
+          <t>2026-07-30T09:17:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-31
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -12207,13 +12207,37 @@
           <t>スキマスイッチ</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dFPEYdbTAD4</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>8647</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>【公式】石森プロ</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dFPEYdbTAD4</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>8647</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>【公式】石森プロ</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>2026-07-31T09:00:54</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-03
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10318,13 +10318,37 @@
           <t>入野自由</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1jwY-WG1XcQ</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>36254</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PROJECT R.E.D. チャンネル</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1jwY-WG1XcQ</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>36254</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>PROJECT R.E.D. チャンネル</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-08-03T09:00:27</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -11122,7 +11146,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>50264</v>
+        <v>76339</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -11135,7 +11159,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>50264</v>
+        <v>76339</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -11144,7 +11168,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-07-24T09:00:42</t>
+          <t>2026-08-03T09:00:49</t>
         </is>
       </c>
     </row>
@@ -11185,15 +11209,15 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=9hrlfMldegI</t>
+          <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>228049</v>
+        <v>26712</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID Official Channel</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -11202,7 +11226,7 @@
         </is>
       </c>
       <c r="M38" t="n">
-        <v>21447</v>
+        <v>26712</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -11211,7 +11235,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-07-24T09:00:51</t>
+          <t>2026-08-03T09:00:58</t>
         </is>
       </c>
     </row>
@@ -17507,7 +17531,7 @@
         </is>
       </c>
       <c r="J140" t="n">
-        <v>334778</v>
+        <v>445767</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
@@ -17520,7 +17544,7 @@
         </is>
       </c>
       <c r="M140" t="n">
-        <v>334778</v>
+        <v>445767</v>
       </c>
       <c r="N140" t="inlineStr">
         <is>
@@ -17529,7 +17553,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-07-24T09:02:09</t>
+          <t>2026-08-03T09:02:13</t>
         </is>
       </c>
     </row>
@@ -17574,7 +17598,7 @@
         </is>
       </c>
       <c r="J141" t="n">
-        <v>11469371</v>
+        <v>11659948</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
@@ -17587,7 +17611,7 @@
         </is>
       </c>
       <c r="M141" t="n">
-        <v>107568</v>
+        <v>127183</v>
       </c>
       <c r="N141" t="inlineStr">
         <is>
@@ -17596,7 +17620,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-07-24T09:02:18</t>
+          <t>2026-08-03T09:02:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-05
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9227,7 +9227,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>8042</v>
+        <v>9949</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -9240,7 +9240,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>8042</v>
+        <v>9949</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -9249,7 +9249,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-07-28T09:00:18</t>
+          <t>2026-08-05T09:00:16</t>
         </is>
       </c>
     </row>
@@ -14558,13 +14558,37 @@
           <t>秦基博</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OhRKTSgC7Es</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>4257</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OhRKTSgC7Es</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>4257</v>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>2026-08-05T09:00:48</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-10
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -12649,7 +12649,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>8647</v>
+        <v>19188</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -12662,7 +12662,7 @@
         </is>
       </c>
       <c r="M54" t="n">
-        <v>8647</v>
+        <v>19188</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -12671,7 +12671,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-07-31T09:00:54</t>
+          <t>2026-08-10T09:00:36</t>
         </is>
       </c>
     </row>
@@ -17038,13 +17038,37 @@
           <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
-      <c r="O125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=H4J8Kh65Qu8</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>94083</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>FRONTIERWORKS</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=H4J8Kh65Qu8</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>94083</v>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>FRONTIERWORKS</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>2026-08-10T09:01:42</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -20375,13 +20399,27 @@
           <t>TOOBOE</t>
         </is>
       </c>
-      <c r="I184" t="inlineStr"/>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+        </is>
+      </c>
+      <c r="J184" t="n">
+        <v>737238</v>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
       <c r="L184" t="inlineStr"/>
       <c r="M184" t="inlineStr"/>
       <c r="N184" t="inlineStr"/>
-      <c r="O184" t="inlineStr"/>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>2026-08-10T09:03:46</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-13
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M171"/>
+  <dimension ref="A1:M172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月10日（土）〜 TOKYO MXにて</t>
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
@@ -7887,8 +7887,16 @@
           <t>JO1</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>トリックスター</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
       <c r="M140" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
@@ -8122,7 +8130,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8135,21 +8143,17 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>SMDE</t>
-        </is>
-      </c>
+          <t>2026年10月3日（土）～ NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26728</t>
         </is>
       </c>
     </row>
@@ -8167,7 +8171,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8180,17 +8184,21 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H147" t="inlineStr"/>
+          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I147" t="inlineStr"/>
       <c r="J147" t="inlineStr"/>
       <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -8208,7 +8216,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8221,25 +8229,17 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>パンどろぼうのうた</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -8257,7 +8257,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>人付き合いが苦手な未亡人の雪女さんと呪いの指輪</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8270,21 +8270,25 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>studio HōKIBOSHI</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
+          <t>2026年10月〜 NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>パンどろぼうのうた</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
       <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28885</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -8302,7 +8306,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>人付き合いが苦手な未亡人の雪女さんと呪いの指輪</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8315,17 +8319,21 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>studio HōKIBOSHI</t>
+        </is>
+      </c>
       <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28885</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8351,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8356,21 +8364,17 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026年10月〜 TBS・BS11にて</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -8388,7 +8392,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8401,29 +8405,21 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜 TBS・BS11にて</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8437,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>僕らが選んだベストアドベンチャー</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8454,17 +8450,29 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ フジテレビほか</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
+          <t>2026年10月～ テレ東系列ほか</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16416</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -8482,7 +8490,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>僕らが選んだベストアドベンチャー</t>
         </is>
       </c>
       <c r="E154" t="b">
@@ -8495,29 +8503,17 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ 全国フジテレビ系“ ノイタミナ ”にて</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
+          <t>2026年10月4日（日）～ フジテレビほか</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr">
-        <is>
-          <t>夢心地</t>
-        </is>
-      </c>
-      <c r="L154" t="inlineStr">
-        <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16416</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8531,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E155" t="b">
@@ -8548,21 +8544,29 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月9日（金）～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>夢心地</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>TOOBOE</t>
+        </is>
+      </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -8580,7 +8584,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E156" t="b">
@@ -8593,12 +8597,12 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I156" t="inlineStr"/>
@@ -8607,7 +8611,7 @@
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -8625,7 +8629,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E157" t="b">
@@ -8638,12 +8642,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -8652,7 +8656,7 @@
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8670,7 +8674,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E158" t="b">
@@ -8683,12 +8687,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I158" t="inlineStr"/>
@@ -8697,7 +8701,7 @@
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8719,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E159" t="b">
@@ -8728,29 +8732,21 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J159" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -8768,7 +8764,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E160" t="b">
@@ -8781,37 +8777,29 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K160" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L160" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -8829,7 +8817,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E161" t="b">
@@ -8842,21 +8830,37 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr"/>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8878,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E162" t="b">
@@ -8887,37 +8891,21 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年10月3日（土）～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K162" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L162" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
       <c r="M162" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -8935,7 +8923,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E163" t="b">
@@ -8948,29 +8936,37 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MXほか</t>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>ワオワールド</t>
+          <t>studio A-CAT</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
-        </is>
-      </c>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8988,7 +8984,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>ゆうさんち！from 遊ハち</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="E164" t="b">
@@ -9001,21 +8997,29 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026年10月～ フジテレビ・カンテレにて</t>
+          <t>2026年10月〜 TOKYO MXほか</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>ファンワークス</t>
-        </is>
-      </c>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
+          <t>ワオワールド</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28884</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27288</t>
         </is>
       </c>
     </row>
@@ -9033,7 +9037,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>ゆうさんち！from 遊ハち</t>
         </is>
       </c>
       <c r="E165" t="b">
@@ -9046,12 +9050,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年10月～ フジテレビ・カンテレにて</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
+          <t>ファンワークス</t>
         </is>
       </c>
       <c r="I165" t="inlineStr"/>
@@ -9060,7 +9064,7 @@
       <c r="L165" t="inlineStr"/>
       <c r="M165" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28884</t>
         </is>
       </c>
     </row>
@@ -9078,7 +9082,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E166" t="b">
@@ -9091,37 +9095,21 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J166" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K166" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L166" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
+      <c r="L166" t="inlineStr"/>
       <c r="M166" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -9139,7 +9127,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E167" t="b">
@@ -9152,21 +9140,37 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr"/>
-      <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -9184,11 +9188,11 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E168" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
@@ -9197,12 +9201,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -9211,7 +9215,7 @@
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -9229,11 +9233,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
@@ -9242,17 +9246,21 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ 日本テレビにて</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -9270,7 +9278,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E170" t="b">
@@ -9278,12 +9286,12 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月3日（土）～ 日本テレビにて</t>
         </is>
       </c>
       <c r="H170" t="inlineStr"/>
@@ -9293,7 +9301,7 @@
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9319,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>ロメリア戦記</t>
+          <t>LEGO® ONE PIECE</t>
         </is>
       </c>
       <c r="E171" t="b">
@@ -9319,24 +9327,65 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>Atra</t>
-        </is>
-      </c>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr"/>
       <c r="J171" t="inlineStr"/>
       <c r="K171" t="inlineStr"/>
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>84</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>ロメリア戦記</t>
+        </is>
+      </c>
+      <c r="E172" t="b">
+        <v>0</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>2026年10月〜 TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Atra</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr"/>
+      <c r="M172" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27077</t>
         </is>
@@ -9353,7 +9402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O193"/>
+  <dimension ref="A1:O195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9517,7 +9566,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>9949</v>
+        <v>11563</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -9530,7 +9579,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>9949</v>
+        <v>11563</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -9539,7 +9588,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-08-05T09:00:16</t>
+          <t>2026-08-13T09:00:16</t>
         </is>
       </c>
     </row>
@@ -20405,7 +20454,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -20413,7 +20462,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -20421,35 +20470,21 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dUSYa-7rKpM</t>
-        </is>
-      </c>
-      <c r="J183" t="n">
-        <v>212832</v>
-      </c>
-      <c r="K183" t="inlineStr">
-        <is>
-          <t>パンどろぼう / PANDOROBO【公式】</t>
-        </is>
-      </c>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:03</t>
-        </is>
-      </c>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -20462,7 +20497,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -20470,7 +20505,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -20478,45 +20513,21 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J184" t="n">
-        <v>3405</v>
-      </c>
-      <c r="K184" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M184" t="n">
-        <v>3405</v>
-      </c>
-      <c r="N184" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O184" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:08</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -20529,7 +20540,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -20537,7 +20548,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -20545,25 +20556,25 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+          <t>https://www.youtube.com/watch?v=dUSYa-7rKpM</t>
         </is>
       </c>
       <c r="J185" t="n">
-        <v>737238</v>
+        <v>212832</v>
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>john / TOOBOE</t>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
         </is>
       </c>
       <c r="L185" t="inlineStr"/>
@@ -20571,7 +20582,7 @@
       <c r="N185" t="inlineStr"/>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-08-10T09:03:46</t>
+          <t>2026-08-06T09:21:03</t>
         </is>
       </c>
     </row>
@@ -20586,7 +20597,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -20602,33 +20613,43 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J186" t="n">
-        <v>107027</v>
+        <v>3405</v>
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L186" t="inlineStr"/>
-      <c r="M186" t="inlineStr"/>
-      <c r="N186" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M186" t="n">
+        <v>3405</v>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-08-06T09:21:27</t>
+          <t>2026-08-06T09:21:08</t>
         </is>
       </c>
     </row>
@@ -20643,7 +20664,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D187" t="b">
@@ -20651,7 +20672,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -20659,43 +20680,33 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>TOOBOE</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
         </is>
       </c>
       <c r="J187" t="n">
-        <v>304602</v>
+        <v>737238</v>
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L187" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M187" t="n">
-        <v>304602</v>
-      </c>
-      <c r="N187" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="inlineStr"/>
+      <c r="N187" t="inlineStr"/>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-08-12T09:11:22</t>
+          <t>2026-08-10T09:03:46</t>
         </is>
       </c>
     </row>
@@ -20710,7 +20721,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D188" t="b">
@@ -20718,7 +20729,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -20726,43 +20737,33 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J188" t="n">
-        <v>304602</v>
+        <v>107027</v>
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L188" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M188" t="n">
-        <v>304602</v>
-      </c>
-      <c r="N188" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr"/>
+      <c r="M188" t="inlineStr"/>
+      <c r="N188" t="inlineStr"/>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-08-12T09:11:31</t>
+          <t>2026-08-06T09:21:27</t>
         </is>
       </c>
     </row>
@@ -20777,7 +20778,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D189" t="b">
@@ -20793,21 +20794,45 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr"/>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
-      <c r="O189" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J189" t="n">
+        <v>304602</v>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M189" t="n">
+        <v>304602</v>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:11:22</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -20820,7 +20845,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D190" t="b">
@@ -20836,21 +20861,45 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr"/>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
-      <c r="M190" t="inlineStr"/>
-      <c r="N190" t="inlineStr"/>
-      <c r="O190" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J190" t="n">
+        <v>304602</v>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M190" t="n">
+        <v>304602</v>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:11:31</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -20863,7 +20912,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D191" t="b">
@@ -20879,12 +20928,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I191" t="inlineStr"/>
@@ -20906,7 +20955,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D192" t="b">
@@ -20914,7 +20963,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -20922,45 +20971,21 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J192" t="n">
-        <v>871807</v>
-      </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M192" t="n">
-        <v>383462</v>
-      </c>
-      <c r="N192" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O192" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:48</t>
-        </is>
-      </c>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
+      <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -20973,7 +20998,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -20981,7 +21006,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -20989,41 +21014,151 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="inlineStr"/>
+      <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D194" t="b">
+        <v>0</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>1</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J194" t="n">
+        <v>871807</v>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M194" t="n">
+        <v>383462</v>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>2026-08-06T09:21:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D195" t="b">
+        <v>0</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>1</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr">
+      <c r="H195" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I193" t="inlineStr">
+      <c r="I195" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
-      <c r="J193" t="n">
+      <c r="J195" t="n">
         <v>396434</v>
       </c>
-      <c r="K193" t="inlineStr">
+      <c r="K195" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="L193" t="inlineStr">
+      <c r="L195" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M193" t="n">
+      <c r="M195" t="n">
         <v>396213</v>
       </c>
-      <c r="N193" t="inlineStr">
+      <c r="N195" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O193" t="inlineStr">
+      <c r="O195" t="inlineStr">
         <is>
           <t>2026-08-06T09:21:58</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-14
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -2225,7 +2225,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026年7月8日（水）～ フジテレビ「+Ultra」にて</t>
+          <t>2026年7月8日（水）～ フジテレビ「+Ultra」ほか</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026年7月6日（月）～ TOKYO MX・BSフジほか</t>
+          <t>2026年7月6日（月）～ TOKYO MX・サンテレビほか</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -6095,8 +6095,16 @@
           <t>KONAMI animation</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>リスポーン!!</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>角巻わため</t>
+        </is>
+      </c>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
@@ -7220,7 +7228,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月4日（日）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -7228,10 +7236,26 @@
           <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>DALALA</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Daoko</t>
+        </is>
+      </c>
       <c r="M127" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
@@ -9402,7 +9426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O195"/>
+  <dimension ref="A1:O198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9690,7 +9714,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>87263</v>
+        <v>101532</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9703,7 +9727,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>87263</v>
+        <v>101532</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -9712,7 +9736,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-08-06T09:01:00</t>
+          <t>2026-08-14T09:00:21</t>
         </is>
       </c>
     </row>
@@ -9800,7 +9824,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>169583</v>
+        <v>173748</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -9813,7 +9837,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>169583</v>
+        <v>173748</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -9822,7 +9846,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-08-06T09:01:16</t>
+          <t>2026-08-14T09:00:33</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9891,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1716610</v>
+        <v>1734513</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -9880,7 +9904,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>22357</v>
+        <v>24460</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -9889,7 +9913,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-08-06T09:01:27</t>
+          <t>2026-08-14T09:00:43</t>
         </is>
       </c>
     </row>
@@ -9934,7 +9958,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>74640</v>
+        <v>79712</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -9947,7 +9971,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>74640</v>
+        <v>79712</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -9956,7 +9980,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-08-06T09:01:39</t>
+          <t>2026-08-14T09:00:52</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10025,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>63066</v>
+        <v>81531</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -10014,7 +10038,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>31544</v>
+        <v>32558</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -10023,7 +10047,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-08-06T09:01:51</t>
+          <t>2026-08-14T09:01:02</t>
         </is>
       </c>
     </row>
@@ -10068,7 +10092,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>603404</v>
+        <v>629682</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -10081,7 +10105,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>120326</v>
+        <v>127635</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -10090,7 +10114,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-08-06T09:02:00</t>
+          <t>2026-08-14T09:01:11</t>
         </is>
       </c>
     </row>
@@ -10178,19 +10202,29 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>154889</v>
+        <v>166616</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>ASTRO DONUTS - Topic</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ilQY7YoJ8o4</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>4227</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>tokusatsu vocalo channel</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-08-06T09:02:34</t>
+          <t>2026-08-14T09:01:41</t>
         </is>
       </c>
     </row>
@@ -10546,7 +10580,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>403884</v>
+        <v>444209</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -10559,7 +10593,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>289526</v>
+        <v>314964</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -10568,7 +10602,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-08-06T09:02:47</t>
+          <t>2026-08-14T09:01:53</t>
         </is>
       </c>
     </row>
@@ -10613,7 +10647,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>357410</v>
+        <v>359123</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -10626,7 +10660,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>123625</v>
+        <v>132584</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -10635,7 +10669,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-08-06T09:02:58</t>
+          <t>2026-08-14T09:02:02</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10781,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>390476</v>
+        <v>396097</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -10760,7 +10794,7 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>11957</v>
+        <v>13998</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -10769,7 +10803,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-08-06T09:03:08</t>
+          <t>2026-08-14T09:02:12</t>
         </is>
       </c>
     </row>
@@ -10881,7 +10915,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>73462</v>
+        <v>80870</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -10894,7 +10928,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>73462</v>
+        <v>80870</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -10903,7 +10937,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-08-06T09:03:19</t>
+          <t>2026-08-14T09:02:21</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10982,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>169549</v>
+        <v>178610</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -10961,7 +10995,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>169549</v>
+        <v>178610</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -10970,7 +11004,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-08-06T09:03:29</t>
+          <t>2026-08-14T09:02:31</t>
         </is>
       </c>
     </row>
@@ -11015,7 +11049,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>2520195</v>
+        <v>2546091</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -11028,7 +11062,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>51209</v>
+        <v>56533</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -11037,7 +11071,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-08-06T09:03:39</t>
+          <t>2026-08-14T09:02:40</t>
         </is>
       </c>
     </row>
@@ -11082,7 +11116,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>946691</v>
+        <v>1373842</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -11095,7 +11129,7 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>61678</v>
+        <v>68482</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -11104,7 +11138,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-08-06T09:03:49</t>
+          <t>2026-08-14T09:02:50</t>
         </is>
       </c>
     </row>
@@ -11302,7 +11336,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>70673</v>
+        <v>79464</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -11315,7 +11349,7 @@
         </is>
       </c>
       <c r="M31" t="n">
-        <v>70673</v>
+        <v>79464</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -11324,7 +11358,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-08-06T09:03:59</t>
+          <t>2026-08-14T09:03:00</t>
         </is>
       </c>
     </row>
@@ -11369,7 +11403,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>6480278</v>
+        <v>6512250</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -11382,7 +11416,7 @@
         </is>
       </c>
       <c r="M32" t="n">
-        <v>6480278</v>
+        <v>6512250</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -11391,7 +11425,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-08-06T09:04:08</t>
+          <t>2026-08-14T09:03:10</t>
         </is>
       </c>
     </row>
@@ -11436,7 +11470,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>116382</v>
+        <v>134115</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -11448,7 +11482,7 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-08-06T09:04:32</t>
+          <t>2026-08-14T09:03:33</t>
         </is>
       </c>
     </row>
@@ -11794,7 +11828,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>342388</v>
+        <v>389173</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -11807,7 +11841,7 @@
         </is>
       </c>
       <c r="M39" t="n">
-        <v>342388</v>
+        <v>389173</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -11816,7 +11850,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-08-06T09:04:46</t>
+          <t>2026-08-14T09:03:45</t>
         </is>
       </c>
     </row>
@@ -11861,7 +11895,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>52144</v>
+        <v>60596</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -11874,7 +11908,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>52144</v>
+        <v>60596</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -11883,7 +11917,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-08-06T09:04:56</t>
+          <t>2026-08-14T09:03:54</t>
         </is>
       </c>
     </row>
@@ -11995,7 +12029,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>2180260</v>
+        <v>2300855</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -12008,7 +12042,7 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>281133</v>
+        <v>299574</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -12017,7 +12051,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-08-06T09:05:06</t>
+          <t>2026-08-14T09:04:04</t>
         </is>
       </c>
     </row>
@@ -12062,7 +12096,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1844216</v>
+        <v>1851085</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -12075,7 +12109,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>1844216</v>
+        <v>1851085</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -12084,7 +12118,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-08-06T09:05:16</t>
+          <t>2026-08-14T09:04:13</t>
         </is>
       </c>
     </row>
@@ -12129,7 +12163,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1844216</v>
+        <v>1851085</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -12142,7 +12176,7 @@
         </is>
       </c>
       <c r="M44" t="n">
-        <v>419164</v>
+        <v>422190</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -12151,7 +12185,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-08-06T09:05:25</t>
+          <t>2026-08-14T09:04:22</t>
         </is>
       </c>
     </row>
@@ -12259,33 +12293,33 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=7HRmpCzDUsY</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>22466</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>名称非公開</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=UDD-U-c-m9Y</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>18579</v>
-      </c>
-      <c r="K46" t="inlineStr">
+      <c r="M46" t="n">
+        <v>21162</v>
+      </c>
+      <c r="N46" t="inlineStr">
         <is>
           <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=UDD-U-c-m9Y</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
-        <v>18579</v>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
-        </is>
-      </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-08-06T09:05:36</t>
+          <t>2026-08-14T09:04:32</t>
         </is>
       </c>
     </row>
@@ -12326,15 +12360,15 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=bcEDagHXQEU</t>
+          <t>https://www.youtube.com/watch?v=AAw-rKQz52s</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>770741</v>
+        <v>296535</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>キタニタツヤ / Tatsuya Kitani</t>
+          <t>VAP Official</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -12343,7 +12377,7 @@
         </is>
       </c>
       <c r="M47" t="n">
-        <v>203664</v>
+        <v>245341</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -12352,7 +12386,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-08-06T09:05:45</t>
+          <t>2026-08-14T09:04:40</t>
         </is>
       </c>
     </row>
@@ -12393,33 +12427,33 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=jI61NtGuxV4</t>
+          <t>https://www.youtube.com/watch?v=-2IX1FDR8aw</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>95142</v>
+        <v>4833258</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
+          <t>リーガルリリー Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BHS-_AXCWrc</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>33964</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
           <t>VAP Official</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=BHS-_AXCWrc</t>
-        </is>
-      </c>
-      <c r="M48" t="n">
-        <v>28617</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>VAP Official</t>
-        </is>
-      </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-08-06T09:05:55</t>
+          <t>2026-08-14T09:04:50</t>
         </is>
       </c>
     </row>
@@ -12464,7 +12498,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>34902</v>
+        <v>42008</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -12477,7 +12511,7 @@
         </is>
       </c>
       <c r="M49" t="n">
-        <v>79350</v>
+        <v>87373</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -12486,7 +12520,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-08-06T09:06:05</t>
+          <t>2026-08-14T09:04:59</t>
         </is>
       </c>
     </row>
@@ -12531,7 +12565,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>7779</v>
+        <v>9406</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -12544,7 +12578,7 @@
         </is>
       </c>
       <c r="M50" t="n">
-        <v>18094</v>
+        <v>20613</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -12553,7 +12587,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-08-06T09:06:16</t>
+          <t>2026-08-14T09:05:08</t>
         </is>
       </c>
     </row>
@@ -12684,7 +12718,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>78957</v>
+        <v>85949</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -12697,7 +12731,7 @@
         </is>
       </c>
       <c r="M53" t="n">
-        <v>78957</v>
+        <v>85949</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -12706,7 +12740,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-08-06T09:06:32</t>
+          <t>2026-08-14T09:05:22</t>
         </is>
       </c>
     </row>
@@ -12818,7 +12852,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>374281</v>
+        <v>432720</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -12831,7 +12865,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>374281</v>
+        <v>432720</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -12840,7 +12874,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-08-06T09:06:42</t>
+          <t>2026-08-14T09:05:32</t>
         </is>
       </c>
     </row>
@@ -12885,7 +12919,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>59153</v>
+        <v>69421</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -12898,7 +12932,7 @@
         </is>
       </c>
       <c r="M56" t="n">
-        <v>41781</v>
+        <v>52085</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -12907,7 +12941,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-08-06T09:06:52</t>
+          <t>2026-08-14T09:05:41</t>
         </is>
       </c>
     </row>
@@ -12952,7 +12986,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>416222</v>
+        <v>471361</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -12965,7 +12999,7 @@
         </is>
       </c>
       <c r="M57" t="n">
-        <v>39778</v>
+        <v>46263</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -12974,7 +13008,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-08-06T09:07:01</t>
+          <t>2026-08-14T09:05:50</t>
         </is>
       </c>
     </row>
@@ -13086,7 +13120,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>6564732</v>
+        <v>6598720</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -13099,7 +13133,7 @@
         </is>
       </c>
       <c r="M59" t="n">
-        <v>757348</v>
+        <v>772761</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -13108,7 +13142,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-08-06T09:07:12</t>
+          <t>2026-08-14T09:06:00</t>
         </is>
       </c>
     </row>
@@ -13153,7 +13187,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>349155</v>
+        <v>446796</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -13166,7 +13200,7 @@
         </is>
       </c>
       <c r="M60" t="n">
-        <v>82428</v>
+        <v>100210</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -13175,7 +13209,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-08-06T09:07:22</t>
+          <t>2026-08-14T09:06:09</t>
         </is>
       </c>
     </row>
@@ -13220,7 +13254,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>62698</v>
+        <v>66310</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -13233,7 +13267,7 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>62698</v>
+        <v>66310</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -13242,7 +13276,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-08-06T09:07:31</t>
+          <t>2026-08-14T09:06:18</t>
         </is>
       </c>
     </row>
@@ -13287,7 +13321,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>11258</v>
+        <v>12668</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -13300,7 +13334,7 @@
         </is>
       </c>
       <c r="M62" t="n">
-        <v>11258</v>
+        <v>12668</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -13309,7 +13343,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-08-06T09:07:40</t>
+          <t>2026-08-14T09:06:27</t>
         </is>
       </c>
     </row>
@@ -13440,7 +13474,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>4558998</v>
+        <v>4684541</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -13453,7 +13487,7 @@
         </is>
       </c>
       <c r="M65" t="n">
-        <v>2043307</v>
+        <v>2082134</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -13462,7 +13496,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-08-06T09:07:50</t>
+          <t>2026-08-14T09:06:36</t>
         </is>
       </c>
     </row>
@@ -13507,7 +13541,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>323307</v>
+        <v>362535</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -13520,7 +13554,7 @@
         </is>
       </c>
       <c r="M66" t="n">
-        <v>323307</v>
+        <v>362535</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -13529,7 +13563,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-08-06T09:08:00</t>
+          <t>2026-08-14T09:06:45</t>
         </is>
       </c>
     </row>
@@ -13574,7 +13608,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>322026</v>
+        <v>334590</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -13587,7 +13621,7 @@
         </is>
       </c>
       <c r="M67" t="n">
-        <v>314896</v>
+        <v>321566</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -13596,7 +13630,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-08-06T09:08:10</t>
+          <t>2026-08-14T09:06:55</t>
         </is>
       </c>
     </row>
@@ -13708,7 +13742,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>30331</v>
+        <v>35202</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -13721,7 +13755,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>30331</v>
+        <v>35202</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -13730,7 +13764,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-08-06T09:08:21</t>
+          <t>2026-08-14T09:07:04</t>
         </is>
       </c>
     </row>
@@ -13775,7 +13809,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>9491</v>
+        <v>10718</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -13788,7 +13822,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>9491</v>
+        <v>10718</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -13797,7 +13831,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-08-06T09:08:30</t>
+          <t>2026-08-14T09:07:14</t>
         </is>
       </c>
     </row>
@@ -13842,7 +13876,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>143202</v>
+        <v>160156</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -13855,7 +13889,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>143202</v>
+        <v>160156</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -13864,7 +13898,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-08-06T09:08:40</t>
+          <t>2026-08-14T09:07:24</t>
         </is>
       </c>
     </row>
@@ -13909,7 +13943,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>19991</v>
+        <v>23377</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -13922,7 +13956,7 @@
         </is>
       </c>
       <c r="M72" t="n">
-        <v>19486</v>
+        <v>22465</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
@@ -13931,7 +13965,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-08-06T09:08:50</t>
+          <t>2026-08-14T09:07:33</t>
         </is>
       </c>
     </row>
@@ -14200,7 +14234,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>134943</v>
+        <v>140178</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -14213,7 +14247,7 @@
         </is>
       </c>
       <c r="M77" t="n">
-        <v>26283</v>
+        <v>29707</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -14222,7 +14256,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-08-06T09:09:04</t>
+          <t>2026-08-14T09:07:44</t>
         </is>
       </c>
     </row>
@@ -14267,7 +14301,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>764673</v>
+        <v>766073</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -14280,7 +14314,7 @@
         </is>
       </c>
       <c r="M78" t="n">
-        <v>764673</v>
+        <v>766073</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -14289,7 +14323,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-08-06T09:09:14</t>
+          <t>2026-08-14T09:07:55</t>
         </is>
       </c>
     </row>
@@ -14334,7 +14368,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>176720</v>
+        <v>177928</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -14347,7 +14381,7 @@
         </is>
       </c>
       <c r="M79" t="n">
-        <v>176720</v>
+        <v>177928</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -14356,7 +14390,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-08-06T09:09:25</t>
+          <t>2026-08-14T09:08:07</t>
         </is>
       </c>
     </row>
@@ -14401,7 +14435,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>370897</v>
+        <v>387335</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -14413,7 +14447,7 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-08-06T09:09:45</t>
+          <t>2026-08-14T09:08:25</t>
         </is>
       </c>
     </row>
@@ -14501,7 +14535,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>224125</v>
+        <v>225887</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -14514,7 +14548,7 @@
         </is>
       </c>
       <c r="M82" t="n">
-        <v>90319</v>
+        <v>95741</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -14523,7 +14557,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-08-06T09:09:58</t>
+          <t>2026-08-14T09:08:37</t>
         </is>
       </c>
     </row>
@@ -14635,7 +14669,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>1335531</v>
+        <v>1467016</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -14648,7 +14682,7 @@
         </is>
       </c>
       <c r="M84" t="n">
-        <v>1335531</v>
+        <v>1467016</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -14657,7 +14691,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-08-06T09:10:09</t>
+          <t>2026-08-14T09:08:46</t>
         </is>
       </c>
     </row>
@@ -14702,7 +14736,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>519174</v>
+        <v>816396</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -14715,7 +14749,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>264474</v>
+        <v>292731</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -14724,7 +14758,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-08-06T09:10:20</t>
+          <t>2026-08-14T09:08:56</t>
         </is>
       </c>
     </row>
@@ -15190,7 +15224,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>106539</v>
+        <v>112928</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -15203,7 +15237,7 @@
         </is>
       </c>
       <c r="M93" t="n">
-        <v>106539</v>
+        <v>112928</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -15212,7 +15246,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-08-06T09:10:43</t>
+          <t>2026-08-14T09:09:15</t>
         </is>
       </c>
     </row>
@@ -15253,33 +15287,33 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=R7hcy44LFB4</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>95739</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Ginger Root</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=lJ6dDUwWOis</t>
         </is>
       </c>
-      <c r="J94" t="n">
-        <v>46516</v>
-      </c>
-      <c r="K94" t="inlineStr">
+      <c r="M94" t="n">
+        <v>51415</v>
+      </c>
+      <c r="N94" t="inlineStr">
         <is>
           <t>KyoaniChannel</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lJ6dDUwWOis</t>
-        </is>
-      </c>
-      <c r="M94" t="n">
-        <v>46516</v>
-      </c>
-      <c r="N94" t="inlineStr">
-        <is>
-          <t>KyoaniChannel</t>
-        </is>
-      </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-08-06T09:10:54</t>
+          <t>2026-08-14T09:09:25</t>
         </is>
       </c>
     </row>
@@ -15324,7 +15358,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>130422</v>
+        <v>140078</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -15337,7 +15371,7 @@
         </is>
       </c>
       <c r="M95" t="n">
-        <v>130422</v>
+        <v>140078</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -15346,7 +15380,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-08-06T09:11:03</t>
+          <t>2026-08-14T09:09:34</t>
         </is>
       </c>
     </row>
@@ -15544,7 +15578,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>462014</v>
+        <v>469137</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -15557,7 +15591,7 @@
         </is>
       </c>
       <c r="M99" t="n">
-        <v>462014</v>
+        <v>469137</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -15566,7 +15600,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-08-06T09:11:25</t>
+          <t>2026-08-14T09:09:54</t>
         </is>
       </c>
     </row>
@@ -15611,7 +15645,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>422702</v>
+        <v>457369</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -15624,7 +15658,7 @@
         </is>
       </c>
       <c r="M100" t="n">
-        <v>401791</v>
+        <v>415580</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -15633,7 +15667,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-08-06T09:11:36</t>
+          <t>2026-08-14T09:10:04</t>
         </is>
       </c>
     </row>
@@ -15678,7 +15712,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>387526</v>
+        <v>398990</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -15691,7 +15725,7 @@
         </is>
       </c>
       <c r="M101" t="n">
-        <v>347939</v>
+        <v>355219</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -15700,7 +15734,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-08-06T09:11:46</t>
+          <t>2026-08-14T09:10:14</t>
         </is>
       </c>
     </row>
@@ -15745,7 +15779,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>65208</v>
+        <v>67866</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -15758,7 +15792,7 @@
         </is>
       </c>
       <c r="M102" t="n">
-        <v>65208</v>
+        <v>67866</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -15767,7 +15801,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-08-06T09:11:56</t>
+          <t>2026-08-14T09:10:23</t>
         </is>
       </c>
     </row>
@@ -15812,7 +15846,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>52188</v>
+        <v>59733</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -15825,7 +15859,7 @@
         </is>
       </c>
       <c r="M103" t="n">
-        <v>52188</v>
+        <v>59733</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -15834,7 +15868,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-08-06T09:12:06</t>
+          <t>2026-08-14T09:10:33</t>
         </is>
       </c>
     </row>
@@ -15879,7 +15913,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>72834</v>
+        <v>87087</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -15892,7 +15926,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>72834</v>
+        <v>87087</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -15901,7 +15935,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-08-06T09:12:16</t>
+          <t>2026-08-14T09:10:42</t>
         </is>
       </c>
     </row>
@@ -16281,7 +16315,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>89798</v>
+        <v>105409</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -16294,7 +16328,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>89798</v>
+        <v>105409</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -16303,7 +16337,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-08-06T09:12:29</t>
+          <t>2026-08-14T09:10:50</t>
         </is>
       </c>
     </row>
@@ -16415,7 +16449,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>101652</v>
+        <v>116698</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -16428,7 +16462,7 @@
         </is>
       </c>
       <c r="M112" t="n">
-        <v>36008</v>
+        <v>40040</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -16437,7 +16471,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-08-06T09:12:40</t>
+          <t>2026-08-14T09:10:59</t>
         </is>
       </c>
     </row>
@@ -16482,7 +16516,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>18232</v>
+        <v>23895</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -16495,7 +16529,7 @@
         </is>
       </c>
       <c r="M113" t="n">
-        <v>16922</v>
+        <v>19117</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -16504,7 +16538,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-08-06T09:12:50</t>
+          <t>2026-08-14T09:11:08</t>
         </is>
       </c>
     </row>
@@ -16549,7 +16583,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>2384711</v>
+        <v>3479782</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -16562,7 +16596,7 @@
         </is>
       </c>
       <c r="M114" t="n">
-        <v>258842</v>
+        <v>320546</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -16571,7 +16605,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-08-06T09:13:00</t>
+          <t>2026-08-14T09:11:18</t>
         </is>
       </c>
     </row>
@@ -16683,7 +16717,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>549607</v>
+        <v>567420</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -16696,7 +16730,7 @@
         </is>
       </c>
       <c r="M116" t="n">
-        <v>549607</v>
+        <v>567420</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -16705,7 +16739,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-08-06T09:13:11</t>
+          <t>2026-08-14T09:11:27</t>
         </is>
       </c>
     </row>
@@ -16860,7 +16894,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>1992603</v>
+        <v>2026537</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -16873,7 +16907,7 @@
         </is>
       </c>
       <c r="M119" t="n">
-        <v>1351496</v>
+        <v>1620767</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -16882,7 +16916,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-08-06T09:13:26</t>
+          <t>2026-08-14T09:11:40</t>
         </is>
       </c>
     </row>
@@ -16927,7 +16961,7 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>1351496</v>
+        <v>1620767</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
@@ -16940,7 +16974,7 @@
         </is>
       </c>
       <c r="M120" t="n">
-        <v>954668</v>
+        <v>1067245</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -16949,7 +16983,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-08-06T09:13:36</t>
+          <t>2026-08-14T09:11:49</t>
         </is>
       </c>
     </row>
@@ -17080,7 +17114,7 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>23671</v>
+        <v>26916</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -17093,7 +17127,7 @@
         </is>
       </c>
       <c r="M123" t="n">
-        <v>23671</v>
+        <v>26916</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
@@ -17102,7 +17136,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-08-06T09:13:57</t>
+          <t>2026-08-14T09:12:10</t>
         </is>
       </c>
     </row>
@@ -17314,7 +17348,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>101759</v>
+        <v>106271</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -17327,7 +17361,7 @@
         </is>
       </c>
       <c r="M127" t="n">
-        <v>101759</v>
+        <v>106271</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -17336,7 +17370,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-08-06T09:14:15</t>
+          <t>2026-08-14T09:12:22</t>
         </is>
       </c>
     </row>
@@ -17381,7 +17415,7 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>301088</v>
+        <v>315546</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -17394,7 +17428,7 @@
         </is>
       </c>
       <c r="M128" t="n">
-        <v>83880</v>
+        <v>88494</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -17403,7 +17437,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-08-06T09:14:23</t>
+          <t>2026-08-14T09:12:31</t>
         </is>
       </c>
     </row>
@@ -17444,11 +17478,11 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+          <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>642527</v>
+        <v>481661</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -17461,7 +17495,7 @@
         </is>
       </c>
       <c r="M129" t="n">
-        <v>423904</v>
+        <v>481661</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -17470,7 +17504,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-08-06T09:14:34</t>
+          <t>2026-08-14T09:12:41</t>
         </is>
       </c>
     </row>
@@ -17511,11 +17545,11 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=0kgUsF8R7JM</t>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
         </is>
       </c>
       <c r="J130" t="n">
-        <v>506864</v>
+        <v>644424</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -17528,7 +17562,7 @@
         </is>
       </c>
       <c r="M130" t="n">
-        <v>98308</v>
+        <v>110594</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -17537,7 +17571,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-08-06T09:14:44</t>
+          <t>2026-08-14T09:12:51</t>
         </is>
       </c>
     </row>
@@ -17731,11 +17765,11 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=mUZEnAeUvgA</t>
+          <t>https://www.youtube.com/watch?v=NEh3-Qmq1LE</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>7055558</v>
+        <v>4172283</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -17748,7 +17782,7 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>235611</v>
+        <v>247200</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -17757,7 +17791,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-08-06T09:15:02</t>
+          <t>2026-08-14T09:13:06</t>
         </is>
       </c>
     </row>
@@ -17802,7 +17836,7 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>1382216</v>
+        <v>1389295</v>
       </c>
       <c r="K135" t="inlineStr">
         <is>
@@ -17815,7 +17849,7 @@
         </is>
       </c>
       <c r="M135" t="n">
-        <v>2564475</v>
+        <v>2583760</v>
       </c>
       <c r="N135" t="inlineStr">
         <is>
@@ -17824,7 +17858,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-08-06T09:15:21</t>
+          <t>2026-08-14T09:13:26</t>
         </is>
       </c>
     </row>
@@ -17869,7 +17903,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>46820</v>
+        <v>48731</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
@@ -17882,7 +17916,7 @@
         </is>
       </c>
       <c r="M136" t="n">
-        <v>13780</v>
+        <v>15184</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
@@ -17891,7 +17925,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-08-06T09:15:32</t>
+          <t>2026-08-14T09:13:35</t>
         </is>
       </c>
     </row>
@@ -17999,15 +18033,15 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=cyVDE5VFz04</t>
+          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
         </is>
       </c>
       <c r="J138" t="n">
-        <v>2923683</v>
+        <v>1878435</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -18016,7 +18050,7 @@
         </is>
       </c>
       <c r="M138" t="n">
-        <v>1662939</v>
+        <v>1878435</v>
       </c>
       <c r="N138" t="inlineStr">
         <is>
@@ -18025,7 +18059,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-08-06T09:15:42</t>
+          <t>2026-08-14T09:13:45</t>
         </is>
       </c>
     </row>
@@ -18070,7 +18104,7 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>1662939</v>
+        <v>1878435</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -18083,7 +18117,7 @@
         </is>
       </c>
       <c r="M139" t="n">
-        <v>614839</v>
+        <v>682471</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
@@ -18092,7 +18126,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-08-06T09:16:01</t>
+          <t>2026-08-14T09:14:04</t>
         </is>
       </c>
     </row>
@@ -18137,7 +18171,7 @@
         </is>
       </c>
       <c r="J140" t="n">
-        <v>49465</v>
+        <v>52502</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
@@ -18149,7 +18183,7 @@
       <c r="N140" t="inlineStr"/>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-08-06T09:16:23</t>
+          <t>2026-08-14T09:14:27</t>
         </is>
       </c>
     </row>
@@ -18328,7 +18362,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>617567</v>
+        <v>620248</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -18341,7 +18375,7 @@
         </is>
       </c>
       <c r="M143" t="n">
-        <v>617567</v>
+        <v>620248</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -18350,7 +18384,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-08-06T09:16:34</t>
+          <t>2026-08-14T09:14:37</t>
         </is>
       </c>
     </row>
@@ -18395,7 +18429,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>76395</v>
+        <v>76836</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -18408,7 +18442,7 @@
         </is>
       </c>
       <c r="M144" t="n">
-        <v>76395</v>
+        <v>76836</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -18417,7 +18451,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-08-06T09:16:43</t>
+          <t>2026-08-14T09:14:47</t>
         </is>
       </c>
     </row>
@@ -18462,7 +18496,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>9526339</v>
+        <v>9540278</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -18475,7 +18509,7 @@
         </is>
       </c>
       <c r="M145" t="n">
-        <v>158046</v>
+        <v>159358</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -18484,7 +18518,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-08-06T09:16:53</t>
+          <t>2026-08-14T09:14:57</t>
         </is>
       </c>
     </row>
@@ -18529,7 +18563,7 @@
         </is>
       </c>
       <c r="J146" t="n">
-        <v>82167</v>
+        <v>82663</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -18542,7 +18576,7 @@
         </is>
       </c>
       <c r="M146" t="n">
-        <v>82167</v>
+        <v>82663</v>
       </c>
       <c r="N146" t="inlineStr">
         <is>
@@ -18551,7 +18585,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-08-06T09:17:02</t>
+          <t>2026-08-14T09:15:06</t>
         </is>
       </c>
     </row>
@@ -18596,7 +18630,7 @@
         </is>
       </c>
       <c r="J147" t="n">
-        <v>3129</v>
+        <v>17187</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -18608,7 +18642,7 @@
       <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-08-06T09:17:24</t>
+          <t>2026-08-14T09:15:28</t>
         </is>
       </c>
     </row>
@@ -18796,7 +18830,7 @@
         </is>
       </c>
       <c r="J151" t="n">
-        <v>12759</v>
+        <v>15827</v>
       </c>
       <c r="K151" t="inlineStr">
         <is>
@@ -18809,7 +18843,7 @@
         </is>
       </c>
       <c r="M151" t="n">
-        <v>12759</v>
+        <v>15827</v>
       </c>
       <c r="N151" t="inlineStr">
         <is>
@@ -18818,7 +18852,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-08-06T09:17:34</t>
+          <t>2026-08-14T09:15:38</t>
         </is>
       </c>
     </row>
@@ -18863,7 +18897,7 @@
         </is>
       </c>
       <c r="J152" t="n">
-        <v>59493</v>
+        <v>60653</v>
       </c>
       <c r="K152" t="inlineStr">
         <is>
@@ -18876,7 +18910,7 @@
         </is>
       </c>
       <c r="M152" t="n">
-        <v>59493</v>
+        <v>60653</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -18885,7 +18919,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-08-06T09:17:43</t>
+          <t>2026-08-14T09:15:48</t>
         </is>
       </c>
     </row>
@@ -18973,7 +19007,7 @@
         </is>
       </c>
       <c r="J154" t="n">
-        <v>202738</v>
+        <v>210495</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
@@ -18986,7 +19020,7 @@
         </is>
       </c>
       <c r="M154" t="n">
-        <v>202738</v>
+        <v>210495</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -18995,7 +19029,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-08-06T09:17:54</t>
+          <t>2026-08-14T09:16:00</t>
         </is>
       </c>
     </row>
@@ -19107,7 +19141,7 @@
         </is>
       </c>
       <c r="J156" t="n">
-        <v>825870</v>
+        <v>873424</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -19120,7 +19154,7 @@
         </is>
       </c>
       <c r="M156" t="n">
-        <v>825870</v>
+        <v>873424</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -19129,7 +19163,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-08-06T09:18:03</t>
+          <t>2026-08-14T09:16:09</t>
         </is>
       </c>
     </row>
@@ -19174,7 +19208,7 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>202226</v>
+        <v>220163</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -19187,7 +19221,7 @@
         </is>
       </c>
       <c r="M157" t="n">
-        <v>79398</v>
+        <v>84624</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -19196,7 +19230,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-08-06T09:18:12</t>
+          <t>2026-08-14T09:16:19</t>
         </is>
       </c>
     </row>
@@ -19308,7 +19342,7 @@
         </is>
       </c>
       <c r="J159" t="n">
-        <v>324827</v>
+        <v>327343</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -19321,7 +19355,7 @@
         </is>
       </c>
       <c r="M159" t="n">
-        <v>324827</v>
+        <v>327343</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -19330,7 +19364,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-08-06T09:18:22</t>
+          <t>2026-08-14T09:16:28</t>
         </is>
       </c>
     </row>
@@ -19442,7 +19476,7 @@
         </is>
       </c>
       <c r="J161" t="n">
-        <v>632681</v>
+        <v>645741</v>
       </c>
       <c r="K161" t="inlineStr">
         <is>
@@ -19455,7 +19489,7 @@
         </is>
       </c>
       <c r="M161" t="n">
-        <v>632681</v>
+        <v>645741</v>
       </c>
       <c r="N161" t="inlineStr">
         <is>
@@ -19464,7 +19498,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-08-06T09:18:32</t>
+          <t>2026-08-14T09:16:38</t>
         </is>
       </c>
     </row>
@@ -19552,7 +19586,7 @@
         </is>
       </c>
       <c r="J163" t="n">
-        <v>57431</v>
+        <v>61702</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19565,7 +19599,7 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>620159</v>
+        <v>621764</v>
       </c>
       <c r="N163" t="inlineStr">
         <is>
@@ -19574,7 +19608,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-08-06T09:18:43</t>
+          <t>2026-08-14T09:16:50</t>
         </is>
       </c>
     </row>
@@ -19718,7 +19752,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="D167" t="b">
@@ -19734,12 +19768,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>リスポーン!!</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>amazarashi</t>
+          <t>角巻わため</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -19761,7 +19795,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ごーすと・みーつ・ぎゃる！</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D168" t="b">
@@ -19769,7 +19803,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -19777,12 +19811,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>にこいちミライ</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
+          <t>amazarashi</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -19804,7 +19838,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D169" t="b">
@@ -19812,7 +19846,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19820,12 +19854,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -19847,7 +19881,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D170" t="b">
@@ -19863,12 +19897,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -19898,7 +19932,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -19906,12 +19940,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I171" t="inlineStr"/>
@@ -19933,7 +19967,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D172" t="b">
@@ -19941,7 +19975,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -19949,12 +19983,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>跡部景吾＆忍足侑士</t>
         </is>
       </c>
       <c r="I172" t="inlineStr"/>
@@ -19984,7 +20018,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -19992,12 +20026,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I173" t="inlineStr"/>
@@ -20019,7 +20053,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -20027,7 +20061,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -20035,45 +20069,21 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J174" t="n">
-        <v>695135</v>
-      </c>
-      <c r="K174" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L174" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M174" t="n">
-        <v>695135</v>
-      </c>
-      <c r="N174" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O174" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:19:41</t>
-        </is>
-      </c>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -20086,7 +20096,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -20094,7 +20104,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -20102,45 +20112,21 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="J175" t="n">
-        <v>383226</v>
-      </c>
-      <c r="K175" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L175" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M175" t="n">
-        <v>383226</v>
-      </c>
-      <c r="N175" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O175" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:19:50</t>
-        </is>
-      </c>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -20153,7 +20139,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -20169,12 +20155,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+          <t>Daoko</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -20196,7 +20182,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -20212,21 +20198,45 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
-      <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v>702298</v>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M177" t="n">
+        <v>702298</v>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:17:59</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -20239,7 +20249,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -20247,7 +20257,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -20255,21 +20265,45 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr"/>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J178" t="n">
+        <v>389648</v>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M178" t="n">
+        <v>389648</v>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:18:08</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -20282,7 +20316,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -20298,12 +20332,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -20325,7 +20359,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -20341,12 +20375,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -20368,7 +20402,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -20376,7 +20410,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -20384,12 +20418,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I181" t="inlineStr"/>
@@ -20411,7 +20445,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -20419,7 +20453,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -20427,12 +20461,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>JO1</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -20454,7 +20488,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -20462,7 +20496,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -20470,12 +20504,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
+          <t>East Of Eden</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -20497,7 +20531,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -20505,7 +20539,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -20513,12 +20547,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
@@ -20540,7 +20574,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -20556,35 +20590,21 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dUSYa-7rKpM</t>
-        </is>
-      </c>
-      <c r="J185" t="n">
-        <v>212832</v>
-      </c>
-      <c r="K185" t="inlineStr">
-        <is>
-          <t>パンどろぼう / PANDOROBO【公式】</t>
-        </is>
-      </c>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr"/>
       <c r="N185" t="inlineStr"/>
-      <c r="O185" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:03</t>
-        </is>
-      </c>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -20597,7 +20617,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -20605,7 +20625,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -20613,45 +20633,21 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J186" t="n">
-        <v>3405</v>
-      </c>
-      <c r="K186" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L186" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M186" t="n">
-        <v>3405</v>
-      </c>
-      <c r="N186" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O186" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:08</t>
-        </is>
-      </c>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -20664,7 +20660,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D187" t="b">
@@ -20672,7 +20668,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -20680,35 +20676,21 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J187" t="n">
-        <v>737238</v>
-      </c>
-      <c r="K187" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
       <c r="L187" t="inlineStr"/>
       <c r="M187" t="inlineStr"/>
       <c r="N187" t="inlineStr"/>
-      <c r="O187" t="inlineStr">
-        <is>
-          <t>2026-08-10T09:03:46</t>
-        </is>
-      </c>
+      <c r="O187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -20721,7 +20703,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D188" t="b">
@@ -20737,35 +20719,21 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
-        </is>
-      </c>
-      <c r="J188" t="n">
-        <v>107027</v>
-      </c>
-      <c r="K188" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr"/>
-      <c r="O188" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:27</t>
-        </is>
-      </c>
+      <c r="O188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -20778,7 +20746,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D189" t="b">
@@ -20794,43 +20762,43 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J189" t="n">
-        <v>304602</v>
+        <v>3908</v>
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
+          <t>Anime Trailer アニメ</t>
         </is>
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="M189" t="n">
-        <v>304602</v>
+        <v>3908</v>
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
+          <t>Anime Trailer アニメ</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-08-12T09:11:22</t>
+          <t>2026-08-14T09:19:30</t>
         </is>
       </c>
     </row>
@@ -20845,7 +20813,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D190" t="b">
@@ -20861,43 +20829,33 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>TOOBOE</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
         </is>
       </c>
       <c r="J190" t="n">
-        <v>304602</v>
+        <v>737238</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L190" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M190" t="n">
-        <v>304602</v>
-      </c>
-      <c r="N190" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="inlineStr"/>
+      <c r="N190" t="inlineStr"/>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-08-12T09:11:31</t>
+          <t>2026-08-10T09:03:46</t>
         </is>
       </c>
     </row>
@@ -20912,7 +20870,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D191" t="b">
@@ -20928,21 +20886,35 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr"/>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J191" t="n">
+        <v>107293</v>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L191" t="inlineStr"/>
       <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr"/>
-      <c r="O191" t="inlineStr"/>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:19:44</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -20955,7 +20927,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D192" t="b">
@@ -20963,7 +20935,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -20971,21 +20943,45 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
-      <c r="M192" t="inlineStr"/>
-      <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J192" t="n">
+        <v>304602</v>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M192" t="n">
+        <v>304602</v>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:11:22</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -20998,7 +20994,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -21006,7 +21002,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -21014,21 +21010,45 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
-      <c r="N193" t="inlineStr"/>
-      <c r="O193" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J193" t="n">
+        <v>304602</v>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M193" t="n">
+        <v>304602</v>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:11:31</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -21041,7 +21061,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D194" t="b">
@@ -21057,45 +21077,21 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J194" t="n">
-        <v>871807</v>
-      </c>
-      <c r="K194" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L194" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M194" t="n">
-        <v>383462</v>
-      </c>
-      <c r="N194" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O194" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:48</t>
-        </is>
-      </c>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="inlineStr"/>
+      <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -21108,7 +21104,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D195" t="b">
@@ -21124,43 +21120,196 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr"/>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
+      <c r="N195" t="inlineStr"/>
+      <c r="O195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>野生のラスボスが現れた！ 第2期</t>
+        </is>
+      </c>
+      <c r="D196" t="b">
+        <v>0</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>1</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr"/>
+      <c r="L196" t="inlineStr"/>
+      <c r="M196" t="inlineStr"/>
+      <c r="N196" t="inlineStr"/>
+      <c r="O196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D197" t="b">
+        <v>0</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>1</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J197" t="n">
+        <v>917131</v>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M197" t="n">
+        <v>391594</v>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:20:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D198" t="b">
+        <v>0</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>1</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr">
+      <c r="H198" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr">
+      <c r="I198" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
-      <c r="J195" t="n">
-        <v>396434</v>
-      </c>
-      <c r="K195" t="inlineStr">
+      <c r="J198" t="n">
+        <v>411712</v>
+      </c>
+      <c r="K198" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="L195" t="inlineStr">
+      <c r="L198" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M195" t="n">
-        <v>396213</v>
-      </c>
-      <c r="N195" t="inlineStr">
+      <c r="M198" t="n">
+        <v>402485</v>
+      </c>
+      <c r="N198" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O195" t="inlineStr">
-        <is>
-          <t>2026-08-06T09:21:58</t>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:20:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-17
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -19819,13 +19819,37 @@
           <t>amazarashi</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
-      <c r="O168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="J168" t="n">
+        <v>187036</v>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="M168" t="n">
+        <v>187036</v>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:01:55</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -19991,13 +20015,27 @@
           <t>跡部景吾＆忍足侑士</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr"/>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>121723</v>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr"/>
       <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr"/>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:02:20</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -20843,7 +20881,7 @@
         </is>
       </c>
       <c r="J190" t="n">
-        <v>737238</v>
+        <v>747589</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -20855,7 +20893,7 @@
       <c r="N190" t="inlineStr"/>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-08-10T09:03:46</t>
+          <t>2026-08-17T09:04:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-18
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -4232,10 +4232,26 @@
           <t>オー・エル・エム（</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Invincible</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>i-dle</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Youth</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>aoen</t>
+        </is>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28670</t>
@@ -6140,12 +6156,24 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
+          <t>第1クール：2026年10月2日（金）～ 第2クール：2027年4月～ 日本テレビ系にて</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>雲を抜け風下へ私だけ</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>ヨルシカ</t>
+        </is>
+      </c>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
@@ -6852,10 +6880,14 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr"/>
+          <t>2026年9月30日（水）～ テレ東系列ほか</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>M.S.C</t>
+        </is>
+      </c>
       <c r="I119" t="inlineStr">
         <is>
           <t>Walls And Bridges</t>
@@ -7787,7 +7819,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月7日（水）～ TOKYO MX ほか</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -7795,10 +7827,26 @@
           <t>C2C</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr"/>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>DREAM OF BUTTERFLY</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>FZMZ</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>バリバリBuddy</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>花冷え。</t>
+        </is>
+      </c>
       <c r="M138" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
@@ -9426,7 +9474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O198"/>
+  <dimension ref="A1:O203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12785,7 +12833,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>19188</v>
+        <v>20934</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -12798,7 +12846,7 @@
         </is>
       </c>
       <c r="M54" t="n">
-        <v>19188</v>
+        <v>20934</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -12807,7 +12855,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-08-10T09:00:36</t>
+          <t>2026-08-18T09:03:46</t>
         </is>
       </c>
     </row>
@@ -17041,7 +17089,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>BEYBLADE X 真・未来編</t>
         </is>
       </c>
       <c r="D122" t="b">
@@ -17057,21 +17105,45 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>Invincible</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
-      <c r="N122" t="inlineStr"/>
-      <c r="O122" t="inlineStr"/>
+          <t>i-dle</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wONjimYg078</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>2342523</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ベイチューブ | BEYBLADE Channel</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wONjimYg078</t>
+        </is>
+      </c>
+      <c r="M122" t="n">
+        <v>2342523</v>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>ベイチューブ | BEYBLADE Channel</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>2026-08-18T09:05:05</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -17084,7 +17156,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>BEYBLADE X 真・未来編</t>
         </is>
       </c>
       <c r="D123" t="b">
@@ -17100,43 +17172,43 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Firetail</t>
+          <t>Youth</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>チョーキューメイ</t>
+          <t>aoen</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=SYpHpUiGcQU</t>
+          <t>https://www.youtube.com/watch?v=nrvbC5NDuDQ</t>
         </is>
       </c>
       <c r="J123" t="n">
-        <v>26916</v>
+        <v>224085</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>MBS animation 公式チャンネル</t>
+          <t>ベイチューブ | BEYBLADE Channel</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=SYpHpUiGcQU</t>
+          <t>https://www.youtube.com/watch?v=nrvbC5NDuDQ</t>
         </is>
       </c>
       <c r="M123" t="n">
-        <v>26916</v>
+        <v>224085</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>MBS animation 公式チャンネル</t>
+          <t>ベイチューブ | BEYBLADE Channel</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:10</t>
+          <t>2026-08-18T09:05:15</t>
         </is>
       </c>
     </row>
@@ -17151,7 +17223,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D124" t="b">
@@ -17167,12 +17239,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Blacker Co., Ltd.</t>
+          <t>○✕△□</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>イツカ▶</t>
+          <t>浪漫派マシュマロ</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -17194,7 +17266,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D125" t="b">
@@ -17210,33 +17282,43 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Elegy of the Enemies</t>
+          <t>Firetail</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>The Canbellz</t>
+          <t>チョーキューメイ</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_EEMJOr1NLA</t>
+          <t>https://www.youtube.com/watch?v=SYpHpUiGcQU</t>
         </is>
       </c>
       <c r="J125" t="n">
-        <v>21369</v>
+        <v>26916</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>神戸シンキ / The Canbellz</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SYpHpUiGcQU</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>26916</v>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-08-12T09:07:52</t>
+          <t>2026-08-14T09:12:10</t>
         </is>
       </c>
     </row>
@@ -17259,53 +17341,29 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>白い蝶が飛んだら</t>
+          <t>Blacker Co., Ltd.</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=H4J8Kh65Qu8</t>
-        </is>
-      </c>
-      <c r="J126" t="n">
-        <v>94083</v>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>FRONTIERWORKS</t>
-        </is>
-      </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=H4J8Kh65Qu8</t>
-        </is>
-      </c>
-      <c r="M126" t="n">
-        <v>94083</v>
-      </c>
-      <c r="N126" t="inlineStr">
-        <is>
-          <t>FRONTIERWORKS</t>
-        </is>
-      </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>2026-08-10T09:01:42</t>
-        </is>
-      </c>
+          <t>イツカ▶</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17318,7 +17376,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D127" t="b">
@@ -17326,7 +17384,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -17334,43 +17392,33 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>Elegy of the Enemies</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>The Canbellz</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=S5BYg1_0u7M</t>
+          <t>https://www.youtube.com/watch?v=_EEMJOr1NLA</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>106271</v>
+        <v>21369</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>avex pictures</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=S5BYg1_0u7M</t>
-        </is>
-      </c>
-      <c r="M127" t="n">
-        <v>106271</v>
-      </c>
-      <c r="N127" t="inlineStr">
-        <is>
-          <t>avex pictures</t>
-        </is>
-      </c>
+          <t>神戸シンキ / The Canbellz</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:22</t>
+          <t>2026-08-12T09:07:52</t>
         </is>
       </c>
     </row>
@@ -17385,7 +17433,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D128" t="b">
@@ -17397,47 +17445,47 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>白い蝶が飛んだら</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_wOZSulv0pY</t>
+          <t>https://www.youtube.com/watch?v=H4J8Kh65Qu8</t>
         </is>
       </c>
       <c r="J128" t="n">
-        <v>315546</v>
+        <v>160367</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>i☆Ris 公式チャンネル</t>
+          <t>FRONTIERWORKS</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=miLM7VnR08o</t>
+          <t>https://www.youtube.com/watch?v=H4J8Kh65Qu8</t>
         </is>
       </c>
       <c r="M128" t="n">
-        <v>88494</v>
+        <v>160367</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>avex pictures</t>
+          <t>FRONTIERWORKS</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:31</t>
+          <t>2026-08-18T09:05:26</t>
         </is>
       </c>
     </row>
@@ -17452,7 +17500,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D129" t="b">
@@ -17468,43 +17516,43 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
+          <t>https://www.youtube.com/watch?v=S5BYg1_0u7M</t>
         </is>
       </c>
       <c r="J129" t="n">
-        <v>481661</v>
+        <v>106271</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+          <t>avex pictures</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
+          <t>https://www.youtube.com/watch?v=S5BYg1_0u7M</t>
         </is>
       </c>
       <c r="M129" t="n">
-        <v>481661</v>
+        <v>106271</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+          <t>avex pictures</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:41</t>
+          <t>2026-08-14T09:12:22</t>
         </is>
       </c>
     </row>
@@ -17519,7 +17567,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D130" t="b">
@@ -17535,43 +17583,43 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+          <t>https://www.youtube.com/watch?v=_wOZSulv0pY</t>
         </is>
       </c>
       <c r="J130" t="n">
-        <v>644424</v>
+        <v>315546</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+          <t>i☆Ris 公式チャンネル</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=hHBu5YXhiXQ</t>
+          <t>https://www.youtube.com/watch?v=miLM7VnR08o</t>
         </is>
       </c>
       <c r="M130" t="n">
-        <v>110594</v>
+        <v>88494</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+          <t>avex pictures</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:51</t>
+          <t>2026-08-14T09:12:31</t>
         </is>
       </c>
     </row>
@@ -17586,7 +17634,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D131" t="b">
@@ -17594,7 +17642,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -17602,21 +17650,45 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>とけて煌る</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>neNna</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
-      <c r="M131" t="inlineStr"/>
-      <c r="N131" t="inlineStr"/>
-      <c r="O131" t="inlineStr"/>
+          <t>水樹奈々</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>481661</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
+        </is>
+      </c>
+      <c r="M131" t="n">
+        <v>481661</v>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:12:41</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -17629,7 +17701,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D132" t="b">
@@ -17637,7 +17709,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -17645,43 +17717,43 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=sg1p3sEU88Q</t>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
         </is>
       </c>
       <c r="J132" t="n">
-        <v>31605</v>
+        <v>644424</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kaya Official YouTube Channel </t>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TOj2RisiiwY</t>
+          <t>https://www.youtube.com/watch?v=hHBu5YXhiXQ</t>
         </is>
       </c>
       <c r="M132" t="n">
-        <v>22978</v>
+        <v>110594</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>【公式】アース・スター エンターテイメント</t>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:06</t>
+          <t>2026-08-14T09:12:51</t>
         </is>
       </c>
     </row>
@@ -17696,7 +17768,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
         </is>
       </c>
       <c r="D133" t="b">
@@ -17712,12 +17784,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>とけて煌る</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>neNna</t>
         </is>
       </c>
       <c r="I133" t="inlineStr"/>
@@ -17739,7 +17811,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D134" t="b">
@@ -17755,43 +17827,43 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=NEh3-Qmq1LE</t>
+          <t>https://www.youtube.com/watch?v=sg1p3sEU88Q</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>4172283</v>
+        <v>31605</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>大原ゆい子Official YouTube</t>
+          <t xml:space="preserve">Kaya Official YouTube Channel </t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=3F8-KF40VhI</t>
+          <t>https://www.youtube.com/watch?v=TOj2RisiiwY</t>
         </is>
       </c>
       <c r="M134" t="n">
-        <v>247200</v>
+        <v>22978</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>TOHO animation</t>
+          <t>【公式】アース・スター エンターテイメント</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:06</t>
+          <t>2026-08-12T09:08:06</t>
         </is>
       </c>
     </row>
@@ -17806,7 +17878,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D135" t="b">
@@ -17822,45 +17894,21 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>祈り、終われば</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>中島美嘉</t>
-        </is>
-      </c>
-      <c r="I135" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ODxfIvSgWuo</t>
-        </is>
-      </c>
-      <c r="J135" t="n">
-        <v>1389295</v>
-      </c>
-      <c r="K135" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="L135" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PINgF6rCuME</t>
-        </is>
-      </c>
-      <c r="M135" t="n">
-        <v>2583760</v>
-      </c>
-      <c r="N135" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="O135" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:13:26</t>
-        </is>
-      </c>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -17873,7 +17921,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D136" t="b">
@@ -17889,43 +17937,43 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=vJzWWkigrU8</t>
+          <t>https://www.youtube.com/watch?v=NEh3-Qmq1LE</t>
         </is>
       </c>
       <c r="J136" t="n">
-        <v>48731</v>
+        <v>4172283</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>大原ゆい子Official YouTube</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=DZIN7Fx_K48</t>
+          <t>https://www.youtube.com/watch?v=3F8-KF40VhI</t>
         </is>
       </c>
       <c r="M136" t="n">
-        <v>15184</v>
+        <v>247200</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>Project ANIMA チャンネル</t>
+          <t>TOHO animation</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:35</t>
+          <t>2026-08-14T09:13:06</t>
         </is>
       </c>
     </row>
@@ -17940,7 +17988,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D137" t="b">
@@ -17956,43 +18004,43 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>ジレンマ</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>冨岡愛</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=00D8aV_cT6c</t>
+          <t>https://www.youtube.com/watch?v=ODxfIvSgWuo</t>
         </is>
       </c>
       <c r="J137" t="n">
-        <v>4016</v>
+        <v>1389295</v>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Project ANIMA チャンネル</t>
+          <t>TOHO animation</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=00D8aV_cT6c</t>
+          <t>https://www.youtube.com/watch?v=PINgF6rCuME</t>
         </is>
       </c>
       <c r="M137" t="n">
-        <v>4016</v>
+        <v>2583760</v>
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>Project ANIMA チャンネル</t>
+          <t>TOHO animation</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:18</t>
+          <t>2026-08-14T09:13:26</t>
         </is>
       </c>
     </row>
@@ -18007,7 +18055,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D138" t="b">
@@ -18023,43 +18071,43 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
+          <t>https://www.youtube.com/watch?v=vJzWWkigrU8</t>
         </is>
       </c>
       <c r="J138" t="n">
-        <v>1878435</v>
+        <v>48731</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
+          <t>https://www.youtube.com/watch?v=DZIN7Fx_K48</t>
         </is>
       </c>
       <c r="M138" t="n">
-        <v>1878435</v>
+        <v>15184</v>
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+          <t>Project ANIMA チャンネル</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:45</t>
+          <t>2026-08-14T09:13:35</t>
         </is>
       </c>
     </row>
@@ -18074,7 +18122,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D139" t="b">
@@ -18090,43 +18138,43 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>煙とブルー</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>ネクライトーキー</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
+          <t>https://www.youtube.com/watch?v=00D8aV_cT6c</t>
         </is>
       </c>
       <c r="J139" t="n">
-        <v>1878435</v>
+        <v>4016</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+          <t>Project ANIMA チャンネル</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TwumA6YhQp4</t>
+          <t>https://www.youtube.com/watch?v=00D8aV_cT6c</t>
         </is>
       </c>
       <c r="M139" t="n">
-        <v>682471</v>
+        <v>4016</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+          <t>Project ANIMA チャンネル</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:04</t>
+          <t>2026-08-12T09:08:18</t>
         </is>
       </c>
     </row>
@@ -18141,7 +18189,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>闇芝居 十七期</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D140" t="b">
@@ -18149,7 +18197,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F140" t="n">
@@ -18157,33 +18205,43 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>闇芝居のブルース</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>風輪（徳間ジャパンコミュニケーションズ）</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=VYlvomHOnO4</t>
+          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
         </is>
       </c>
       <c r="J140" t="n">
-        <v>52502</v>
+        <v>1878435</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>闇芝居チャンネル</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr"/>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
+        </is>
+      </c>
+      <c r="M140" t="n">
+        <v>1878435</v>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+        </is>
+      </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:27</t>
+          <t>2026-08-14T09:13:45</t>
         </is>
       </c>
     </row>
@@ -18198,7 +18256,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D141" t="b">
@@ -18206,7 +18264,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -18214,43 +18272,43 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Why? RED induction</t>
+          <t>煙とブルー</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>ネクライトーキー</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IVyvkwvsqW0</t>
+          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
         </is>
       </c>
       <c r="J141" t="n">
-        <v>523872</v>
+        <v>1878435</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IVyvkwvsqW0</t>
+          <t>https://www.youtube.com/watch?v=TwumA6YhQp4</t>
         </is>
       </c>
       <c r="M141" t="n">
-        <v>523872</v>
+        <v>682471</v>
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:27</t>
+          <t>2026-08-14T09:14:04</t>
         </is>
       </c>
     </row>
@@ -18265,7 +18323,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>闇芝居 十七期</t>
         </is>
       </c>
       <c r="D142" t="b">
@@ -18281,43 +18339,33 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Weiter! Weiter!</t>
+          <t>闇芝居のブルース</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
+          <t>風輪（徳間ジャパンコミュニケーションズ）</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_werYjm5BmY</t>
+          <t>https://www.youtube.com/watch?v=VYlvomHOnO4</t>
         </is>
       </c>
       <c r="J142" t="n">
-        <v>11805532</v>
+        <v>52502</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧） - Topic</t>
-        </is>
-      </c>
-      <c r="L142" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
-        </is>
-      </c>
-      <c r="M142" t="n">
-        <v>142001</v>
-      </c>
-      <c r="N142" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>闇芝居チャンネル</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:37</t>
+          <t>2026-08-14T09:14:27</t>
         </is>
       </c>
     </row>
@@ -18332,7 +18380,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D143" t="b">
@@ -18348,43 +18396,43 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>Why? RED induction</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
+          <t>https://www.youtube.com/watch?v=IVyvkwvsqW0</t>
         </is>
       </c>
       <c r="J143" t="n">
-        <v>620248</v>
+        <v>523872</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
+          <t>https://www.youtube.com/watch?v=IVyvkwvsqW0</t>
         </is>
       </c>
       <c r="M143" t="n">
-        <v>620248</v>
+        <v>523872</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:37</t>
+          <t>2026-08-12T09:08:27</t>
         </is>
       </c>
     </row>
@@ -18399,7 +18447,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D144" t="b">
@@ -18407,51 +18455,51 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>Weiter! Weiter!</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=_werYjm5BmY</t>
         </is>
       </c>
       <c r="J144" t="n">
-        <v>76836</v>
+        <v>11805532</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+          <t>ターニャ・デグレチャフ（CV：悠木碧） - Topic</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
         </is>
       </c>
       <c r="M144" t="n">
-        <v>76836</v>
+        <v>142001</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:47</t>
+          <t>2026-08-12T09:08:37</t>
         </is>
       </c>
     </row>
@@ -18474,7 +18522,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F145" t="n">
@@ -18482,34 +18530,34 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=aw45Q_mr0_M</t>
+          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
         </is>
       </c>
       <c r="J145" t="n">
-        <v>9540278</v>
+        <v>620248</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=VJflo-z7e7A</t>
+          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
         </is>
       </c>
       <c r="M145" t="n">
-        <v>159358</v>
+        <v>620248</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -18518,7 +18566,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:57</t>
+          <t>2026-08-14T09:14:37</t>
         </is>
       </c>
     </row>
@@ -18541,7 +18589,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -18549,21 +18597,21 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
         </is>
       </c>
       <c r="J146" t="n">
-        <v>82663</v>
+        <v>76836</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -18572,11 +18620,11 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
         </is>
       </c>
       <c r="M146" t="n">
-        <v>82663</v>
+        <v>76836</v>
       </c>
       <c r="N146" t="inlineStr">
         <is>
@@ -18585,7 +18633,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-08-14T09:15:06</t>
+          <t>2026-08-14T09:14:47</t>
         </is>
       </c>
     </row>
@@ -18600,7 +18648,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D147" t="b">
@@ -18608,7 +18656,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F147" t="n">
@@ -18616,33 +18664,43 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>＋ENCOUNT</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=t4aVIi8sHzA</t>
+          <t>https://www.youtube.com/watch?v=aw45Q_mr0_M</t>
         </is>
       </c>
       <c r="J147" t="n">
-        <v>17187</v>
+        <v>9540278</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>FLOW Official YouTube Channel</t>
-        </is>
-      </c>
-      <c r="L147" t="inlineStr"/>
-      <c r="M147" t="inlineStr"/>
-      <c r="N147" t="inlineStr"/>
+          <t>ONE OR EIGHT</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VJflo-z7e7A</t>
+        </is>
+      </c>
+      <c r="M147" t="n">
+        <v>159358</v>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-08-14T09:15:28</t>
+          <t>2026-08-14T09:14:57</t>
         </is>
       </c>
     </row>
@@ -18657,7 +18715,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D148" t="b">
@@ -18669,37 +18727,47 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7hWVEf4JTrI</t>
+          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
         </is>
       </c>
       <c r="J148" t="n">
-        <v>105436</v>
+        <v>82663</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>TrySail（麻倉もも・雨宮天・夏川椎菜）official YouTube channel</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr"/>
-      <c r="M148" t="inlineStr"/>
-      <c r="N148" t="inlineStr"/>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
+        </is>
+      </c>
+      <c r="M148" t="n">
+        <v>82663</v>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:00</t>
+          <t>2026-08-14T09:15:06</t>
         </is>
       </c>
     </row>
@@ -18714,11 +18782,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D149" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -18730,21 +18798,35 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>虹色Passions！</t>
+          <t>＋ENCOUNT</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>虹ヶ咲学園スクールアイドル同好会</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=t4aVIi8sHzA</t>
+        </is>
+      </c>
+      <c r="J149" t="n">
+        <v>17187</v>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>FLOW Official YouTube Channel</t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr"/>
       <c r="N149" t="inlineStr"/>
-      <c r="O149" t="inlineStr"/>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:15:28</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -18757,11 +18839,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D150" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -18773,21 +18855,35 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>NEO SKY, NEO MAP!</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>虹ヶ咲学園スクールアイドル同好会</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
+          <t>TrySail</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hWVEf4JTrI</t>
+        </is>
+      </c>
+      <c r="J150" t="n">
+        <v>105436</v>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>TrySail（麻倉もも・雨宮天・夏川椎菜）official YouTube channel</t>
+        </is>
+      </c>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr"/>
       <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr"/>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:09:00</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -18800,11 +18896,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
         </is>
       </c>
       <c r="D151" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -18816,45 +18912,21 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>虹色Passions！</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=fCboU3XWuLU</t>
-        </is>
-      </c>
-      <c r="J151" t="n">
-        <v>15827</v>
-      </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=fCboU3XWuLU</t>
-        </is>
-      </c>
-      <c r="M151" t="n">
-        <v>15827</v>
-      </c>
-      <c r="N151" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O151" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:15:38</t>
-        </is>
-      </c>
+          <t>虹ヶ咲学園スクールアイドル同好会</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr"/>
+      <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -18867,11 +18939,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
         </is>
       </c>
       <c r="D152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -18883,45 +18955,21 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>NEO SKY, NEO MAP!</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dhAKFhT6pno</t>
-        </is>
-      </c>
-      <c r="J152" t="n">
-        <v>60653</v>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dhAKFhT6pno</t>
-        </is>
-      </c>
-      <c r="M152" t="n">
-        <v>60653</v>
-      </c>
-      <c r="N152" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O152" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:15:48</t>
-        </is>
-      </c>
+          <t>虹ヶ咲学園スクールアイドル同好会</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr"/>
+      <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -18934,7 +18982,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D153" t="b">
@@ -18950,21 +18998,45 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
-      <c r="M153" t="inlineStr"/>
-      <c r="N153" t="inlineStr"/>
-      <c r="O153" t="inlineStr"/>
+          <t>CROWN HEAD</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fCboU3XWuLU</t>
+        </is>
+      </c>
+      <c r="J153" t="n">
+        <v>15827</v>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fCboU3XWuLU</t>
+        </is>
+      </c>
+      <c r="M153" t="n">
+        <v>15827</v>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:15:38</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -18977,7 +19049,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D154" t="b">
@@ -18993,43 +19065,43 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=HjtjOaJz-_U</t>
+          <t>https://www.youtube.com/watch?v=dhAKFhT6pno</t>
         </is>
       </c>
       <c r="J154" t="n">
-        <v>210495</v>
+        <v>60653</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
+          <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=HjtjOaJz-_U</t>
+          <t>https://www.youtube.com/watch?v=dhAKFhT6pno</t>
         </is>
       </c>
       <c r="M154" t="n">
-        <v>210495</v>
+        <v>60653</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
+          <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:00</t>
+          <t>2026-08-14T09:15:48</t>
         </is>
       </c>
     </row>
@@ -19044,7 +19116,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>レッツゴー怪奇組</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D155" t="b">
@@ -19060,45 +19132,21 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>気味が悪いんだからねっ</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>SWEET STEADY</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GEZWCWyX-is</t>
-        </is>
-      </c>
-      <c r="J155" t="n">
-        <v>176941</v>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>TBSアニメ</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GEZWCWyX-is</t>
-        </is>
-      </c>
-      <c r="M155" t="n">
-        <v>176941</v>
-      </c>
-      <c r="N155" t="inlineStr">
-        <is>
-          <t>TBSアニメ</t>
-        </is>
-      </c>
-      <c r="O155" t="inlineStr">
-        <is>
-          <t>2026-08-12T09:09:11</t>
-        </is>
-      </c>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr"/>
+      <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -19111,7 +19159,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>レッツゴー怪奇組</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D156" t="b">
@@ -19127,43 +19175,43 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>呪わしてね？</t>
+          <t>ひなたぼっこ</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>雨穴</t>
+          <t>REIRIE</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=MnDO2Vv4ZkA</t>
+          <t>https://www.youtube.com/watch?v=HjtjOaJz-_U</t>
         </is>
       </c>
       <c r="J156" t="n">
-        <v>873424</v>
+        <v>210495</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>TBSアニメ</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=MnDO2Vv4ZkA</t>
+          <t>https://www.youtube.com/watch?v=HjtjOaJz-_U</t>
         </is>
       </c>
       <c r="M156" t="n">
-        <v>873424</v>
+        <v>210495</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>TBSアニメ</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:09</t>
+          <t>2026-08-14T09:16:00</t>
         </is>
       </c>
     </row>
@@ -19178,7 +19226,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>レッツゴー怪奇組</t>
         </is>
       </c>
       <c r="D157" t="b">
@@ -19194,43 +19242,43 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>気味が悪いんだからねっ</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>SWEET STEADY</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=9-RVzXLF53U</t>
+          <t>https://www.youtube.com/watch?v=GEZWCWyX-is</t>
         </is>
       </c>
       <c r="J157" t="n">
-        <v>220163</v>
+        <v>176941</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Itsuki Natsume / 棗いつき</t>
+          <t>TBSアニメ</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=4iRiuYov9pY</t>
+          <t>https://www.youtube.com/watch?v=GEZWCWyX-is</t>
         </is>
       </c>
       <c r="M157" t="n">
-        <v>84624</v>
+        <v>176941</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+          <t>TBSアニメ</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:19</t>
+          <t>2026-08-12T09:09:11</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19293,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>レッツゴー怪奇組</t>
         </is>
       </c>
       <c r="D158" t="b">
@@ -19261,43 +19309,43 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>呪わしてね？</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>雨穴</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=MgIol7kDcTE</t>
+          <t>https://www.youtube.com/watch?v=MnDO2Vv4ZkA</t>
         </is>
       </c>
       <c r="J158" t="n">
-        <v>17977</v>
+        <v>873424</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+          <t>TBSアニメ</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=MgIol7kDcTE</t>
+          <t>https://www.youtube.com/watch?v=MnDO2Vv4ZkA</t>
         </is>
       </c>
       <c r="M158" t="n">
-        <v>17977</v>
+        <v>873424</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+          <t>TBSアニメ</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:21</t>
+          <t>2026-08-14T09:16:09</t>
         </is>
       </c>
     </row>
@@ -19312,7 +19360,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D159" t="b">
@@ -19328,43 +19376,43 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+          <t>https://www.youtube.com/watch?v=9-RVzXLF53U</t>
         </is>
       </c>
       <c r="J159" t="n">
-        <v>327343</v>
+        <v>220163</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>SHOCHIKU anime Channel</t>
+          <t>Itsuki Natsume / 棗いつき</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+          <t>https://www.youtube.com/watch?v=4iRiuYov9pY</t>
         </is>
       </c>
       <c r="M159" t="n">
-        <v>327343</v>
+        <v>84624</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>SHOCHIKU anime Channel</t>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:28</t>
+          <t>2026-08-14T09:16:19</t>
         </is>
       </c>
     </row>
@@ -19379,7 +19427,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D160" t="b">
@@ -19395,43 +19443,43 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>名もない花</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>hockrockb</t>
+          <t>ゆきむら。</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=h2zytdkjAU8</t>
+          <t>https://www.youtube.com/watch?v=MgIol7kDcTE</t>
         </is>
       </c>
       <c r="J160" t="n">
-        <v>300689</v>
+        <v>17977</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>SHOCHIKU anime Channel</t>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=h2zytdkjAU8</t>
+          <t>https://www.youtube.com/watch?v=MgIol7kDcTE</t>
         </is>
       </c>
       <c r="M160" t="n">
-        <v>300689</v>
+        <v>17977</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>SHOCHIKU anime Channel</t>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:30</t>
+          <t>2026-08-12T09:09:21</t>
         </is>
       </c>
     </row>
@@ -19446,7 +19494,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>ONE PIECE HEROINES</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D161" t="b">
@@ -19454,7 +19502,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -19462,58 +19510,58 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Blue Shining Star</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>アイナ・ジ・エンド</t>
+          <t>マカロニえんぴつ</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=oDsll0GzhpY</t>
+          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
         </is>
       </c>
       <c r="J161" t="n">
-        <v>645741</v>
+        <v>327343</v>
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>ONE PIECE Official YouTube Channel</t>
+          <t>SHOCHIKU anime Channel</t>
         </is>
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=oDsll0GzhpY</t>
+          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
         </is>
       </c>
       <c r="M161" t="n">
-        <v>645741</v>
+        <v>327343</v>
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>ONE PIECE Official YouTube Channel</t>
+          <t>SHOCHIKU anime Channel</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:38</t>
+          <t>2026-08-14T09:16:28</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>FX戦士くるみちゃん</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D162" t="b">
@@ -19529,34 +19577,58 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>$・¥・€ （ドル・エン・ユーロ）</t>
+          <t>名もない花</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>福賀くるみ（CV：鈴木愛奈）</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr"/>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
-      <c r="M162" t="inlineStr"/>
-      <c r="N162" t="inlineStr"/>
-      <c r="O162" t="inlineStr"/>
+          <t>hockrockb</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=h2zytdkjAU8</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
+        <v>300689</v>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=h2zytdkjAU8</t>
+        </is>
+      </c>
+      <c r="M162" t="n">
+        <v>300689</v>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:09:30</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
+          <t>ONE PIECE HEROINES</t>
         </is>
       </c>
       <c r="D163" t="b">
@@ -19572,43 +19644,43 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Escape</t>
+          <t>Blue Shining Star</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Kis-My-Ft2</t>
+          <t>アイナ・ジ・エンド</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+          <t>https://www.youtube.com/watch?v=oDsll0GzhpY</t>
         </is>
       </c>
       <c r="J163" t="n">
-        <v>61702</v>
+        <v>645741</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+          <t>ONE PIECE Official YouTube Channel</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
+          <t>https://www.youtube.com/watch?v=oDsll0GzhpY</t>
         </is>
       </c>
       <c r="M163" t="n">
-        <v>621764</v>
+        <v>645741</v>
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+          <t>ONE PIECE Official YouTube Channel</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:50</t>
+          <t>2026-08-14T09:16:38</t>
         </is>
       </c>
     </row>
@@ -19623,7 +19695,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="D164" t="b">
@@ -19631,7 +19703,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -19639,12 +19711,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>$・¥・€ （ドル・エン・ユーロ）</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>THE RAMPAGE</t>
+          <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
       <c r="I164" t="inlineStr"/>
@@ -19666,7 +19738,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="D165" t="b">
@@ -19674,7 +19746,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -19682,21 +19754,45 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>Escape</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
-      <c r="N165" t="inlineStr"/>
-      <c r="O165" t="inlineStr"/>
+          <t>Kis-My-Ft2</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+        </is>
+      </c>
+      <c r="J165" t="n">
+        <v>61702</v>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
+        </is>
+      </c>
+      <c r="M165" t="n">
+        <v>621764</v>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:16:50</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -19709,7 +19805,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D166" t="b">
@@ -19717,7 +19813,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -19725,12 +19821,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>krage</t>
+          <t>THE RAMPAGE</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -19752,7 +19848,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D167" t="b">
@@ -19768,12 +19864,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>リスポーン!!</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>角巻わため</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -19795,7 +19891,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D168" t="b">
@@ -19803,7 +19899,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -19811,45 +19907,21 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>amazarashi</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="J168" t="n">
-        <v>187036</v>
-      </c>
-      <c r="K168" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="L168" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="M168" t="n">
-        <v>187036</v>
-      </c>
-      <c r="N168" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="O168" t="inlineStr">
-        <is>
-          <t>2026-08-17T09:01:55</t>
-        </is>
-      </c>
+          <t>krage</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr"/>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -19862,7 +19934,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ごーすと・みーつ・ぎゃる！</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="D169" t="b">
@@ -19870,7 +19942,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19878,12 +19950,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>にこいちミライ</t>
+          <t>リスポーン!!</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
+          <t>角巻わため</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -19905,7 +19977,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="D170" t="b">
@@ -19921,21 +19993,35 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>雲を抜け風下へ私だけ</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr"/>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
+          <t>ヨルシカ</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
+        </is>
+      </c>
+      <c r="J170" t="n">
+        <v>1189561</v>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr"/>
       <c r="N170" t="inlineStr"/>
-      <c r="O170" t="inlineStr"/>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>2026-08-18T09:06:27</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -19948,7 +20034,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D171" t="b">
@@ -19964,21 +20050,45 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
-      <c r="M171" t="inlineStr"/>
-      <c r="N171" t="inlineStr"/>
-      <c r="O171" t="inlineStr"/>
+          <t>amazarashi</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>187036</v>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="M171" t="n">
+        <v>187036</v>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:01:55</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -19991,7 +20101,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D172" t="b">
@@ -19999,7 +20109,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20007,35 +20117,21 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
-        </is>
-      </c>
-      <c r="J172" t="n">
-        <v>121723</v>
-      </c>
-      <c r="K172" t="inlineStr">
-        <is>
-          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
-        </is>
-      </c>
+          <t>夢限大みゅーたいぷ</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr"/>
       <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr">
-        <is>
-          <t>2026-08-17T09:02:20</t>
-        </is>
-      </c>
+      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -20048,7 +20144,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -20064,12 +20160,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I173" t="inlineStr"/>
@@ -20091,7 +20187,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -20099,7 +20195,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -20107,12 +20203,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -20134,7 +20230,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -20142,7 +20238,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -20150,21 +20246,35 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>SiM</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>121723</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr"/>
-      <c r="O175" t="inlineStr"/>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:02:20</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -20177,7 +20287,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -20185,7 +20295,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -20193,12 +20303,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -20220,7 +20330,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -20228,7 +20338,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -20236,45 +20346,21 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J177" t="n">
-        <v>702298</v>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L177" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M177" t="n">
-        <v>702298</v>
-      </c>
-      <c r="N177" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O177" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:17:59</t>
-        </is>
-      </c>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -20287,7 +20373,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -20295,7 +20381,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -20303,45 +20389,21 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="J178" t="n">
-        <v>389648</v>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L178" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M178" t="n">
-        <v>389648</v>
-      </c>
-      <c r="N178" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O178" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:18:08</t>
-        </is>
-      </c>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -20354,7 +20416,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -20370,12 +20432,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+          <t>Daoko</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -20397,7 +20459,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -20413,21 +20475,45 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr"/>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
-      <c r="O180" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J180" t="n">
+        <v>702298</v>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M180" t="n">
+        <v>702298</v>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:17:59</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -20440,7 +20526,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -20448,7 +20534,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -20456,21 +20542,45 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr"/>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
-      <c r="M181" t="inlineStr"/>
-      <c r="N181" t="inlineStr"/>
-      <c r="O181" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J181" t="n">
+        <v>389648</v>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M181" t="n">
+        <v>389648</v>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:18:08</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -20483,7 +20593,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -20499,12 +20609,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -20526,7 +20636,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -20542,12 +20652,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -20569,7 +20679,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -20577,7 +20687,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -20585,12 +20695,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
@@ -20612,7 +20722,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -20620,7 +20730,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -20628,12 +20738,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>JO1</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I185" t="inlineStr"/>
@@ -20655,7 +20765,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -20663,7 +20773,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -20671,12 +20781,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I186" t="inlineStr"/>
@@ -20698,7 +20808,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="D187" t="b">
@@ -20706,7 +20816,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -20714,12 +20824,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I187" t="inlineStr"/>
@@ -20741,7 +20851,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D188" t="b">
@@ -20757,12 +20867,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+          <t>East Of Eden</t>
         </is>
       </c>
       <c r="I188" t="inlineStr"/>
@@ -20784,7 +20894,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D189" t="b">
@@ -20792,7 +20902,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -20800,45 +20910,21 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J189" t="n">
-        <v>3908</v>
-      </c>
-      <c r="K189" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L189" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M189" t="n">
-        <v>3908</v>
-      </c>
-      <c r="N189" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O189" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:19:30</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="inlineStr"/>
+      <c r="N189" t="inlineStr"/>
+      <c r="O189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -20851,7 +20937,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D190" t="b">
@@ -20859,7 +20945,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -20867,35 +20953,21 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J190" t="n">
-        <v>747589</v>
-      </c>
-      <c r="K190" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr"/>
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr"/>
-      <c r="O190" t="inlineStr">
-        <is>
-          <t>2026-08-17T09:04:05</t>
-        </is>
-      </c>
+      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -20908,7 +20980,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D191" t="b">
@@ -20916,7 +20988,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -20924,35 +20996,21 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
-        </is>
-      </c>
-      <c r="J191" t="n">
-        <v>107293</v>
-      </c>
-      <c r="K191" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
       <c r="L191" t="inlineStr"/>
       <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr"/>
-      <c r="O191" t="inlineStr">
-        <is>
-          <t>2026-08-14T09:19:44</t>
-        </is>
-      </c>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -20965,7 +21023,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D192" t="b">
@@ -20973,7 +21031,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -20981,45 +21039,21 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J192" t="n">
-        <v>304602</v>
-      </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M192" t="n">
-        <v>304602</v>
-      </c>
-      <c r="N192" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O192" t="inlineStr">
-        <is>
-          <t>2026-08-12T09:11:22</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
+      <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -21032,7 +21066,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -21040,7 +21074,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -21048,45 +21082,21 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J193" t="n">
-        <v>304602</v>
-      </c>
-      <c r="K193" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L193" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M193" t="n">
-        <v>304602</v>
-      </c>
-      <c r="N193" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O193" t="inlineStr">
-        <is>
-          <t>2026-08-12T09:11:31</t>
-        </is>
-      </c>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="inlineStr"/>
+      <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -21099,7 +21109,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D194" t="b">
@@ -21115,21 +21125,45 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
-      <c r="M194" t="inlineStr"/>
-      <c r="N194" t="inlineStr"/>
-      <c r="O194" t="inlineStr"/>
+          <t>WANIMA</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="J194" t="n">
+        <v>3908</v>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M194" t="n">
+        <v>3908</v>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:19:30</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -21142,7 +21176,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D195" t="b">
@@ -21158,21 +21192,35 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
+          <t>TOOBOE</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+        </is>
+      </c>
+      <c r="J195" t="n">
+        <v>747589</v>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr"/>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:04:05</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -21185,7 +21233,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D196" t="b">
@@ -21201,21 +21249,35 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
-        </is>
-      </c>
-      <c r="I196" t="inlineStr"/>
-      <c r="J196" t="inlineStr"/>
-      <c r="K196" t="inlineStr"/>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J196" t="n">
+        <v>107293</v>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L196" t="inlineStr"/>
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr"/>
-      <c r="O196" t="inlineStr"/>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:19:44</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -21228,7 +21290,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D197" t="b">
@@ -21244,43 +21306,43 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
         </is>
       </c>
       <c r="J197" t="n">
-        <v>917131</v>
+        <v>304602</v>
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+          <t>Bandai Namco Filmworks Channel</t>
         </is>
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
         </is>
       </c>
       <c r="M197" t="n">
-        <v>391594</v>
+        <v>304602</v>
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>NBCUniversal Anime/Music</t>
+          <t>Bandai Namco Filmworks Channel</t>
         </is>
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-08-14T09:20:08</t>
+          <t>2026-08-12T09:11:22</t>
         </is>
       </c>
     </row>
@@ -21295,7 +21357,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D198" t="b">
@@ -21311,41 +21373,304 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J198" t="n">
+        <v>304602</v>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M198" t="n">
+        <v>304602</v>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>2026-08-12T09:11:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+        </is>
+      </c>
+      <c r="D199" t="b">
+        <v>0</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>1</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
+      <c r="L199" t="inlineStr"/>
+      <c r="M199" t="inlineStr"/>
+      <c r="N199" t="inlineStr"/>
+      <c r="O199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+        </is>
+      </c>
+      <c r="D200" t="b">
+        <v>0</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>1</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr"/>
+      <c r="L200" t="inlineStr"/>
+      <c r="M200" t="inlineStr"/>
+      <c r="N200" t="inlineStr"/>
+      <c r="O200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>野生のラスボスが現れた！ 第2期</t>
+        </is>
+      </c>
+      <c r="D201" t="b">
+        <v>0</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>1</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="inlineStr"/>
+      <c r="M201" t="inlineStr"/>
+      <c r="N201" t="inlineStr"/>
+      <c r="O201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D202" t="b">
+        <v>0</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>1</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J202" t="n">
+        <v>917131</v>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M202" t="n">
+        <v>391594</v>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>2026-08-14T09:20:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D203" t="b">
+        <v>0</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>1</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr">
+      <c r="H203" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I198" t="inlineStr">
+      <c r="I203" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
-      <c r="J198" t="n">
+      <c r="J203" t="n">
         <v>411712</v>
       </c>
-      <c r="K198" t="inlineStr">
+      <c r="K203" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="L198" t="inlineStr">
+      <c r="L203" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M198" t="n">
+      <c r="M203" t="n">
         <v>402485</v>
       </c>
-      <c r="N198" t="inlineStr">
+      <c r="N203" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O198" t="inlineStr">
+      <c r="O203" t="inlineStr">
         <is>
           <t>2026-08-14T09:20:18</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-19
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M172"/>
+  <dimension ref="A1:M173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9305,34 +9305,30 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>楽楽飯店</t>
         </is>
       </c>
       <c r="E169" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>サンライズ</t>
-        </is>
-      </c>
+          <t>2026年9月下旬 公式YouTubeチャンネルにて</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28945</t>
         </is>
       </c>
     </row>
@@ -9350,11 +9346,11 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E170" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -9363,17 +9359,21 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ 日本テレビにて</t>
-        </is>
-      </c>
-      <c r="H170" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I170" t="inlineStr"/>
       <c r="J170" t="inlineStr"/>
       <c r="K170" t="inlineStr"/>
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -9391,7 +9391,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E171" t="b">
@@ -9399,12 +9399,12 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月3日（土）～ 日本テレビにて</t>
         </is>
       </c>
       <c r="H171" t="inlineStr"/>
@@ -9414,7 +9414,7 @@
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
         </is>
       </c>
     </row>
@@ -9432,7 +9432,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>ロメリア戦記</t>
+          <t>LEGO® ONE PIECE</t>
         </is>
       </c>
       <c r="E172" t="b">
@@ -9440,24 +9440,65 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>Atra</t>
-        </is>
-      </c>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>85</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>ロメリア戦記</t>
+        </is>
+      </c>
+      <c r="E173" t="b">
+        <v>0</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>2026年10月〜 TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Atra</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27077</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-20
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9746,7 +9746,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>647696</v>
+        <v>654932</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -9758,7 +9758,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-08-12T09:00:35</t>
+          <t>2026-08-20T09:00:32</t>
         </is>
       </c>
     </row>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>107863</v>
+        <v>114483</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -10371,7 +10371,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>254595</v>
+        <v>254678</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -10380,7 +10380,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-08-12T09:00:59</t>
+          <t>2026-08-20T09:00:55</t>
         </is>
       </c>
     </row>
@@ -10425,7 +10425,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>595487</v>
+        <v>691632</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>21288</v>
+        <v>23230</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -10447,7 +10447,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-08-12T09:01:07</t>
+          <t>2026-08-20T09:01:04</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10492,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>98409</v>
+        <v>108834</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -10505,7 +10505,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>98409</v>
+        <v>108834</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -10514,7 +10514,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-08-12T09:01:16</t>
+          <t>2026-08-20T09:01:13</t>
         </is>
       </c>
     </row>
@@ -10559,7 +10559,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>272349</v>
+        <v>301287</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -10572,7 +10572,7 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>272349</v>
+        <v>301287</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-08-12T09:01:27</t>
+          <t>2026-08-20T09:01:22</t>
         </is>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>6895451</v>
+        <v>6915723</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -10816,7 +10816,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>120685</v>
+        <v>130414</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -10825,7 +10825,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-08-12T09:01:38</t>
+          <t>2026-08-20T09:01:33</t>
         </is>
       </c>
     </row>
@@ -10937,7 +10937,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>242596</v>
+        <v>284264</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>89321</v>
+        <v>111799</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -10959,7 +10959,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-08-12T09:01:47</t>
+          <t>2026-08-20T09:01:42</t>
         </is>
       </c>
     </row>
@@ -11358,7 +11358,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>751431</v>
+        <v>873090</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>399006</v>
+        <v>459429</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -11380,7 +11380,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-08-12T09:01:57</t>
+          <t>2026-08-20T09:01:51</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>21076</v>
+        <v>23944</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -11628,7 +11628,7 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-08-12T09:02:28</t>
+          <t>2026-08-20T09:02:20</t>
         </is>
       </c>
     </row>
@@ -11673,7 +11673,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>74670</v>
+        <v>94247</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -11686,7 +11686,7 @@
         </is>
       </c>
       <c r="M35" t="n">
-        <v>1253721</v>
+        <v>1266492</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -11695,7 +11695,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-08-12T09:02:46</t>
+          <t>2026-08-20T09:02:40</t>
         </is>
       </c>
     </row>
@@ -11783,7 +11783,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>96365</v>
+        <v>111905</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -11796,7 +11796,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>96365</v>
+        <v>111905</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -11805,7 +11805,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-08-12T09:02:59</t>
+          <t>2026-08-20T09:02:52</t>
         </is>
       </c>
     </row>
@@ -11846,33 +11846,33 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=a09O2IYjvzk</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>103091</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>MYTH &amp; ROID Official Channel</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>33274</v>
-      </c>
-      <c r="K38" t="inlineStr">
+      <c r="M38" t="n">
+        <v>38477</v>
+      </c>
+      <c r="N38" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
-        <v>33274</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-08-12T09:03:08</t>
+          <t>2026-08-20T09:03:00</t>
         </is>
       </c>
     </row>
@@ -12051,7 +12051,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>2837279</v>
+        <v>5180757</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>2276312</v>
+        <v>2358996</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -12073,7 +12073,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-08-12T09:03:18</t>
+          <t>2026-08-20T09:03:09</t>
         </is>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>46619</v>
+        <v>50588</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -12332,7 +12332,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>46619</v>
+        <v>50588</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -12341,7 +12341,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-08-12T09:03:27</t>
+          <t>2026-08-20T09:03:19</t>
         </is>
       </c>
     </row>
@@ -13142,7 +13142,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>76511</v>
+        <v>81211</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -13155,7 +13155,7 @@
         </is>
       </c>
       <c r="M58" t="n">
-        <v>9559</v>
+        <v>10222</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-08-12T09:03:42</t>
+          <t>2026-08-20T09:03:33</t>
         </is>
       </c>
     </row>
@@ -13764,7 +13764,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>618066</v>
+        <v>729261</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -13777,7 +13777,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>219154</v>
+        <v>256666</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -13786,7 +13786,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-08-12T09:03:52</t>
+          <t>2026-08-20T09:03:42</t>
         </is>
       </c>
     </row>
@@ -14142,7 +14142,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1009213</v>
+        <v>1035165</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -14155,7 +14155,7 @@
         </is>
       </c>
       <c r="M74" t="n">
-        <v>153230</v>
+        <v>163780</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -14164,7 +14164,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-08-12T09:04:04</t>
+          <t>2026-08-20T09:03:53</t>
         </is>
       </c>
     </row>
@@ -14209,7 +14209,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>289357</v>
+        <v>321620</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -14221,7 +14221,7 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-08-12T09:04:15</t>
+          <t>2026-08-20T09:04:04</t>
         </is>
       </c>
     </row>
@@ -14266,7 +14266,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>2334849</v>
+        <v>2842301</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -14278,7 +14278,7 @@
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-08-12T09:04:43</t>
+          <t>2026-08-20T09:04:31</t>
         </is>
       </c>
     </row>
@@ -14691,7 +14691,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>11383</v>
+        <v>12477</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -14704,7 +14704,7 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>11383</v>
+        <v>12477</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -14713,7 +14713,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-08-12T09:04:56</t>
+          <t>2026-08-20T09:04:44</t>
         </is>
       </c>
     </row>
@@ -14892,7 +14892,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>9306927</v>
+        <v>9349156</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -14905,7 +14905,7 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>221419</v>
+        <v>231035</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -14914,7 +14914,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-08-12T09:05:06</t>
+          <t>2026-08-20T09:04:53</t>
         </is>
       </c>
     </row>
@@ -14959,7 +14959,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>221419</v>
+        <v>231035</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -14972,7 +14972,7 @@
         </is>
       </c>
       <c r="M87" t="n">
-        <v>221419</v>
+        <v>231035</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -14981,7 +14981,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-08-12T09:05:15</t>
+          <t>2026-08-20T09:05:02</t>
         </is>
       </c>
     </row>
@@ -15026,7 +15026,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>23704</v>
+        <v>30472</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -15039,7 +15039,7 @@
         </is>
       </c>
       <c r="M88" t="n">
-        <v>23704</v>
+        <v>30472</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -15048,7 +15048,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-08-12T09:05:24</t>
+          <t>2026-08-20T09:05:11</t>
         </is>
       </c>
     </row>
@@ -15093,7 +15093,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>128255</v>
+        <v>160376</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -15106,7 +15106,7 @@
         </is>
       </c>
       <c r="M89" t="n">
-        <v>19349</v>
+        <v>28323</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -15115,7 +15115,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-08-12T09:05:32</t>
+          <t>2026-08-20T09:05:20</t>
         </is>
       </c>
     </row>
@@ -15203,7 +15203,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>7955920</v>
+        <v>8166016</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -15216,7 +15216,7 @@
         </is>
       </c>
       <c r="M91" t="n">
-        <v>696232</v>
+        <v>781885</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -15225,7 +15225,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-08-12T09:05:49</t>
+          <t>2026-08-20T09:05:38</t>
         </is>
       </c>
     </row>
@@ -15514,7 +15514,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>66861</v>
+        <v>77810</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -15527,7 +15527,7 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>17341</v>
+        <v>21062</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -15536,7 +15536,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-08-12T09:06:02</t>
+          <t>2026-08-20T09:05:50</t>
         </is>
       </c>
     </row>
@@ -16069,7 +16069,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1635683</v>
+        <v>1641632</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -16082,7 +16082,7 @@
         </is>
       </c>
       <c r="M105" t="n">
-        <v>471319</v>
+        <v>475308</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -16091,7 +16091,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-08-12T09:06:21</t>
+          <t>2026-08-20T09:06:09</t>
         </is>
       </c>
     </row>
@@ -16136,7 +16136,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>1635683</v>
+        <v>1641632</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -16149,7 +16149,7 @@
         </is>
       </c>
       <c r="M106" t="n">
-        <v>471319</v>
+        <v>475308</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-08-12T09:06:30</t>
+          <t>2026-08-20T09:06:18</t>
         </is>
       </c>
     </row>
@@ -16197,37 +16197,13 @@
           <t>TAMAchan</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1g8PZWar8cY</t>
-        </is>
-      </c>
-      <c r="J107" t="n">
-        <v>4146</v>
-      </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L107" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1g8PZWar8cY</t>
-        </is>
-      </c>
-      <c r="M107" t="n">
-        <v>4146</v>
-      </c>
-      <c r="N107" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="O107" t="inlineStr">
-        <is>
-          <t>2026-08-12T09:06:34</t>
-        </is>
-      </c>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -16270,7 +16246,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>742153</v>
+        <v>827930</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -16279,11 +16255,11 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=9TTfyS5r3Ps</t>
+          <t>https://www.youtube.com/watch?v=Ech7Tj8ga0Y</t>
         </is>
       </c>
       <c r="M108" t="n">
-        <v>124452</v>
+        <v>697155</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -16292,7 +16268,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-08-12T09:06:43</t>
+          <t>2026-08-20T09:06:30</t>
         </is>
       </c>
     </row>
@@ -16337,7 +16313,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>811774</v>
+        <v>824253</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -16350,7 +16326,7 @@
         </is>
       </c>
       <c r="M109" t="n">
-        <v>138270</v>
+        <v>148614</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -16359,7 +16335,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-08-12T09:06:53</t>
+          <t>2026-08-20T09:06:39</t>
         </is>
       </c>
     </row>
@@ -16471,7 +16447,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>48792</v>
+        <v>156926</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -16484,7 +16460,7 @@
         </is>
       </c>
       <c r="M111" t="n">
-        <v>28857</v>
+        <v>32190</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -16493,7 +16469,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-08-12T09:07:02</t>
+          <t>2026-08-20T09:06:48</t>
         </is>
       </c>
     </row>
@@ -16739,7 +16715,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>842904</v>
+        <v>858366</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -16752,7 +16728,7 @@
         </is>
       </c>
       <c r="M115" t="n">
-        <v>196512</v>
+        <v>250743</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -16761,7 +16737,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-08-12T09:07:13</t>
+          <t>2026-08-20T09:06:58</t>
         </is>
       </c>
     </row>
@@ -16873,7 +16849,7 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>268405</v>
+        <v>268845</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -16886,7 +16862,7 @@
         </is>
       </c>
       <c r="M117" t="n">
-        <v>32974</v>
+        <v>35862</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
@@ -16895,7 +16871,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-08-12T09:07:23</t>
+          <t>2026-08-20T09:07:07</t>
         </is>
       </c>
     </row>
@@ -17447,7 +17423,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>21369</v>
+        <v>21733</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -17459,7 +17435,7 @@
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-08-12T09:07:52</t>
+          <t>2026-08-20T09:07:36</t>
         </is>
       </c>
     </row>
@@ -17882,7 +17858,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>31605</v>
+        <v>36509</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -17895,7 +17871,7 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>22978</v>
+        <v>25232</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -17904,7 +17880,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:06</t>
+          <t>2026-08-20T09:07:50</t>
         </is>
       </c>
     </row>
@@ -18193,7 +18169,7 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>4016</v>
+        <v>4492</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -18206,7 +18182,7 @@
         </is>
       </c>
       <c r="M139" t="n">
-        <v>4016</v>
+        <v>4492</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
@@ -18215,7 +18191,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:18</t>
+          <t>2026-08-20T09:08:02</t>
         </is>
       </c>
     </row>
@@ -18451,7 +18427,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>523872</v>
+        <v>589919</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -18464,7 +18440,7 @@
         </is>
       </c>
       <c r="M143" t="n">
-        <v>523872</v>
+        <v>589919</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -18473,7 +18449,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:27</t>
+          <t>2026-08-20T09:08:11</t>
         </is>
       </c>
     </row>
@@ -18518,7 +18494,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>11805532</v>
+        <v>11933492</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -18527,11 +18503,11 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
+          <t>https://www.youtube.com/watch?v=7igP1I4XWws</t>
         </is>
       </c>
       <c r="M144" t="n">
-        <v>142001</v>
+        <v>166076</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -18540,7 +18516,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-08-12T09:08:37</t>
+          <t>2026-08-20T09:08:20</t>
         </is>
       </c>
     </row>
@@ -18910,7 +18886,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>105436</v>
+        <v>120629</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -18922,7 +18898,7 @@
       <c r="N150" t="inlineStr"/>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:00</t>
+          <t>2026-08-20T09:08:42</t>
         </is>
       </c>
     </row>
@@ -19297,7 +19273,7 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>176941</v>
+        <v>194288</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -19310,7 +19286,7 @@
         </is>
       </c>
       <c r="M157" t="n">
-        <v>176941</v>
+        <v>194288</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -19319,7 +19295,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:11</t>
+          <t>2026-08-20T09:08:55</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19474,7 @@
         </is>
       </c>
       <c r="J160" t="n">
-        <v>17977</v>
+        <v>20775</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -19511,7 +19487,7 @@
         </is>
       </c>
       <c r="M160" t="n">
-        <v>17977</v>
+        <v>20775</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -19520,7 +19496,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:21</t>
+          <t>2026-08-20T09:09:04</t>
         </is>
       </c>
     </row>
@@ -19632,7 +19608,7 @@
         </is>
       </c>
       <c r="J162" t="n">
-        <v>300689</v>
+        <v>301272</v>
       </c>
       <c r="K162" t="inlineStr">
         <is>
@@ -19645,7 +19621,7 @@
         </is>
       </c>
       <c r="M162" t="n">
-        <v>300689</v>
+        <v>301272</v>
       </c>
       <c r="N162" t="inlineStr">
         <is>
@@ -19654,7 +19630,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-08-12T09:09:30</t>
+          <t>2026-08-20T09:09:13</t>
         </is>
       </c>
     </row>
@@ -21361,7 +21337,7 @@
         </is>
       </c>
       <c r="J197" t="n">
-        <v>304602</v>
+        <v>307069</v>
       </c>
       <c r="K197" t="inlineStr">
         <is>
@@ -21374,7 +21350,7 @@
         </is>
       </c>
       <c r="M197" t="n">
-        <v>304602</v>
+        <v>307069</v>
       </c>
       <c r="N197" t="inlineStr">
         <is>
@@ -21383,7 +21359,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-08-12T09:11:22</t>
+          <t>2026-08-20T09:12:04</t>
         </is>
       </c>
     </row>
@@ -21428,7 +21404,7 @@
         </is>
       </c>
       <c r="J198" t="n">
-        <v>304602</v>
+        <v>307070</v>
       </c>
       <c r="K198" t="inlineStr">
         <is>
@@ -21441,7 +21417,7 @@
         </is>
       </c>
       <c r="M198" t="n">
-        <v>304602</v>
+        <v>307070</v>
       </c>
       <c r="N198" t="inlineStr">
         <is>
@@ -21450,7 +21426,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-08-12T09:11:31</t>
+          <t>2026-08-20T09:12:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-21
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9679,7 +9679,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>11563</v>
+        <v>13111</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -9692,7 +9692,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>11563</v>
+        <v>13111</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -9701,7 +9701,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-08-13T09:00:16</t>
+          <t>2026-08-21T09:00:15</t>
         </is>
       </c>
     </row>
@@ -16197,13 +16197,37 @@
           <t>TAMAchan</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
-      <c r="M107" t="inlineStr"/>
-      <c r="N107" t="inlineStr"/>
-      <c r="O107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1g8PZWar8cY</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>4640</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1g8PZWar8cY</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>4640</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>2026-08-21T09:01:01</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -21021,13 +21045,37 @@
           <t>go!go!vanillas</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr"/>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
-      <c r="M191" t="inlineStr"/>
-      <c r="N191" t="inlineStr"/>
-      <c r="O191" t="inlineStr"/>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J191" t="n">
+        <v>17851</v>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M191" t="n">
+        <v>3801597</v>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>2026-08-21T09:03:35</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-24
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9803,7 +9803,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>101532</v>
+        <v>116477</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9816,7 +9816,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>101532</v>
+        <v>116477</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -9825,7 +9825,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-08-14T09:00:21</t>
+          <t>2026-08-24T09:00:24</t>
         </is>
       </c>
     </row>
@@ -9913,7 +9913,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>173748</v>
+        <v>179010</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -9926,7 +9926,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>173748</v>
+        <v>179010</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -9935,7 +9935,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-08-14T09:00:33</t>
+          <t>2026-08-24T09:00:35</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1734513</v>
+        <v>1756130</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>24460</v>
+        <v>26678</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -10002,7 +10002,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-08-14T09:00:43</t>
+          <t>2026-08-24T09:00:45</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10047,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>79712</v>
+        <v>85399</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -10060,7 +10060,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>79712</v>
+        <v>85399</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -10069,7 +10069,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-08-14T09:00:52</t>
+          <t>2026-08-24T09:00:54</t>
         </is>
       </c>
     </row>
@@ -10114,7 +10114,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>81531</v>
+        <v>104154</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -10127,7 +10127,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>32558</v>
+        <v>33755</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -10136,7 +10136,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-08-14T09:01:02</t>
+          <t>2026-08-24T09:01:03</t>
         </is>
       </c>
     </row>
@@ -10181,7 +10181,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>629682</v>
+        <v>663417</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -10194,7 +10194,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>127635</v>
+        <v>138361</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -10203,7 +10203,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-08-14T09:01:11</t>
+          <t>2026-08-24T09:01:12</t>
         </is>
       </c>
     </row>
@@ -10291,7 +10291,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>166616</v>
+        <v>176010</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -10300,20 +10300,20 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ilQY7YoJ8o4</t>
+          <t>https://www.youtube.com/watch?v=vFzSsnYprmY</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>4227</v>
+        <v>11738</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>tokusatsu vocalo channel</t>
+          <t>first</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-08-14T09:01:41</t>
+          <t>2026-08-24T09:01:31</t>
         </is>
       </c>
     </row>
@@ -10669,7 +10669,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>444209</v>
+        <v>494857</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -10682,7 +10682,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>314964</v>
+        <v>342150</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -10691,7 +10691,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-08-14T09:01:53</t>
+          <t>2026-08-24T09:01:43</t>
         </is>
       </c>
     </row>
@@ -10736,7 +10736,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>359123</v>
+        <v>361561</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -10749,7 +10749,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>132584</v>
+        <v>141261</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -10758,7 +10758,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-08-14T09:02:02</t>
+          <t>2026-08-24T09:01:51</t>
         </is>
       </c>
     </row>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>396097</v>
+        <v>402822</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -10883,7 +10883,7 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>13998</v>
+        <v>16006</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -10892,7 +10892,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-08-14T09:02:12</t>
+          <t>2026-08-24T09:02:01</t>
         </is>
       </c>
     </row>
@@ -11004,7 +11004,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>80870</v>
+        <v>88836</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -11017,7 +11017,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>80870</v>
+        <v>88836</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -11026,7 +11026,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-08-14T09:02:21</t>
+          <t>2026-08-24T09:02:10</t>
         </is>
       </c>
     </row>
@@ -11071,7 +11071,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>178610</v>
+        <v>189544</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>178610</v>
+        <v>189544</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -11093,7 +11093,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-08-14T09:02:31</t>
+          <t>2026-08-24T09:02:19</t>
         </is>
       </c>
     </row>
@@ -11138,7 +11138,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>2546091</v>
+        <v>2577038</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -11151,7 +11151,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>56533</v>
+        <v>61739</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -11160,7 +11160,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-08-14T09:02:40</t>
+          <t>2026-08-24T09:02:28</t>
         </is>
       </c>
     </row>
@@ -11205,7 +11205,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>1373842</v>
+        <v>1683585</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -11218,7 +11218,7 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>68482</v>
+        <v>75169</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -11227,7 +11227,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-08-14T09:02:50</t>
+          <t>2026-08-24T09:02:37</t>
         </is>
       </c>
     </row>
@@ -11425,7 +11425,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>79464</v>
+        <v>90823</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -11438,7 +11438,7 @@
         </is>
       </c>
       <c r="M31" t="n">
-        <v>79464</v>
+        <v>90823</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -11447,7 +11447,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-08-14T09:03:00</t>
+          <t>2026-08-24T09:02:46</t>
         </is>
       </c>
     </row>
@@ -11492,7 +11492,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>6512250</v>
+        <v>6554770</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -11505,7 +11505,7 @@
         </is>
       </c>
       <c r="M32" t="n">
-        <v>6512250</v>
+        <v>6554770</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -11514,7 +11514,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-08-14T09:03:10</t>
+          <t>2026-08-24T09:02:55</t>
         </is>
       </c>
     </row>
@@ -11559,7 +11559,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>134115</v>
+        <v>159297</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -11571,7 +11571,7 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-08-14T09:03:33</t>
+          <t>2026-08-24T09:03:18</t>
         </is>
       </c>
     </row>
@@ -11917,7 +11917,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>389173</v>
+        <v>428718</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -11930,7 +11930,7 @@
         </is>
       </c>
       <c r="M39" t="n">
-        <v>389173</v>
+        <v>428718</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -11939,7 +11939,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-08-14T09:03:45</t>
+          <t>2026-08-24T09:03:30</t>
         </is>
       </c>
     </row>
@@ -11984,7 +11984,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>60596</v>
+        <v>67519</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -11997,7 +11997,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>60596</v>
+        <v>67519</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -12006,7 +12006,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-08-14T09:03:54</t>
+          <t>2026-08-24T09:03:38</t>
         </is>
       </c>
     </row>
@@ -12118,7 +12118,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>2300855</v>
+        <v>2397308</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>299574</v>
+        <v>315575</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:04</t>
+          <t>2026-08-24T09:03:47</t>
         </is>
       </c>
     </row>
@@ -12185,7 +12185,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1851085</v>
+        <v>1858240</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -12198,7 +12198,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>1851085</v>
+        <v>1858240</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -12207,7 +12207,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:13</t>
+          <t>2026-08-24T09:03:56</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12252,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1851085</v>
+        <v>1858188</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -12265,7 +12265,7 @@
         </is>
       </c>
       <c r="M44" t="n">
-        <v>422190</v>
+        <v>425340</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -12274,7 +12274,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:22</t>
+          <t>2026-08-24T09:04:05</t>
         </is>
       </c>
     </row>
@@ -12386,7 +12386,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>22466</v>
+        <v>30166</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -12399,7 +12399,7 @@
         </is>
       </c>
       <c r="M46" t="n">
-        <v>21162</v>
+        <v>23958</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -12408,7 +12408,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:32</t>
+          <t>2026-08-24T09:04:14</t>
         </is>
       </c>
     </row>
@@ -12449,33 +12449,33 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=AAw-rKQz52s</t>
+          <t>https://www.youtube.com/watch?v=Cb-i3Ixhjt8</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>296535</v>
+        <v>333991</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
+          <t>キタニタツヤ / Tatsuya Kitani</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZcX905vF0j0</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>285329</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
           <t>VAP Official</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ZcX905vF0j0</t>
-        </is>
-      </c>
-      <c r="M47" t="n">
-        <v>245341</v>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>VAP Official</t>
-        </is>
-      </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:40</t>
+          <t>2026-08-24T09:04:23</t>
         </is>
       </c>
     </row>
@@ -12520,7 +12520,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>4833258</v>
+        <v>4858315</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         </is>
       </c>
       <c r="M48" t="n">
-        <v>33964</v>
+        <v>38620</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -12542,7 +12542,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:50</t>
+          <t>2026-08-24T09:04:32</t>
         </is>
       </c>
     </row>
@@ -12587,7 +12587,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>42008</v>
+        <v>52278</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -12600,7 +12600,7 @@
         </is>
       </c>
       <c r="M49" t="n">
-        <v>87373</v>
+        <v>97024</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -12609,7 +12609,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-08-14T09:04:59</t>
+          <t>2026-08-24T09:04:41</t>
         </is>
       </c>
     </row>
@@ -12654,7 +12654,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>9406</v>
+        <v>11367</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -12667,7 +12667,7 @@
         </is>
       </c>
       <c r="M50" t="n">
-        <v>20613</v>
+        <v>23215</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -12676,7 +12676,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-08-14T09:05:08</t>
+          <t>2026-08-24T09:04:51</t>
         </is>
       </c>
     </row>
@@ -12807,7 +12807,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>85949</v>
+        <v>92302</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="M53" t="n">
-        <v>85949</v>
+        <v>92302</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -12829,7 +12829,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-08-14T09:05:22</t>
+          <t>2026-08-24T09:05:05</t>
         </is>
       </c>
     </row>
@@ -12941,7 +12941,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>432720</v>
+        <v>488825</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -12954,7 +12954,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>432720</v>
+        <v>488825</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -12963,7 +12963,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-08-14T09:05:32</t>
+          <t>2026-08-24T09:05:14</t>
         </is>
       </c>
     </row>
@@ -13008,7 +13008,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>69421</v>
+        <v>82666</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -13021,7 +13021,7 @@
         </is>
       </c>
       <c r="M56" t="n">
-        <v>52085</v>
+        <v>61292</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -13030,7 +13030,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-08-14T09:05:41</t>
+          <t>2026-08-24T09:05:23</t>
         </is>
       </c>
     </row>
@@ -13075,7 +13075,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>471361</v>
+        <v>524973</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -13088,7 +13088,7 @@
         </is>
       </c>
       <c r="M57" t="n">
-        <v>46263</v>
+        <v>52466</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -13097,7 +13097,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-08-14T09:05:50</t>
+          <t>2026-08-24T09:05:32</t>
         </is>
       </c>
     </row>
@@ -13209,7 +13209,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>6598720</v>
+        <v>6637291</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -13222,7 +13222,7 @@
         </is>
       </c>
       <c r="M59" t="n">
-        <v>772761</v>
+        <v>790942</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:00</t>
+          <t>2026-08-24T09:05:41</t>
         </is>
       </c>
     </row>
@@ -13272,11 +13272,11 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7NgGbDb53M8</t>
+          <t>https://www.youtube.com/watch?v=kagoEGKHZvU</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>446796</v>
+        <v>364629723</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -13289,7 +13289,7 @@
         </is>
       </c>
       <c r="M60" t="n">
-        <v>100210</v>
+        <v>126066</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -13298,7 +13298,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:09</t>
+          <t>2026-08-24T09:05:50</t>
         </is>
       </c>
     </row>
@@ -13343,7 +13343,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>66310</v>
+        <v>70231</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -13356,7 +13356,7 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>66310</v>
+        <v>70231</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -13365,7 +13365,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:18</t>
+          <t>2026-08-24T09:05:59</t>
         </is>
       </c>
     </row>
@@ -13410,7 +13410,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>12668</v>
+        <v>14294</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         </is>
       </c>
       <c r="M62" t="n">
-        <v>12668</v>
+        <v>14294</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -13432,7 +13432,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:27</t>
+          <t>2026-08-24T09:06:08</t>
         </is>
       </c>
     </row>
@@ -13563,7 +13563,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>4684541</v>
+        <v>4843021</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -13576,7 +13576,7 @@
         </is>
       </c>
       <c r="M65" t="n">
-        <v>2082134</v>
+        <v>2128786</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -13585,7 +13585,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:36</t>
+          <t>2026-08-24T09:06:17</t>
         </is>
       </c>
     </row>
@@ -13630,7 +13630,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>362535</v>
+        <v>407449</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -13643,7 +13643,7 @@
         </is>
       </c>
       <c r="M66" t="n">
-        <v>362535</v>
+        <v>407449</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -13652,7 +13652,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:45</t>
+          <t>2026-08-24T09:06:26</t>
         </is>
       </c>
     </row>
@@ -13697,7 +13697,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>334590</v>
+        <v>349472</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -13710,7 +13710,7 @@
         </is>
       </c>
       <c r="M67" t="n">
-        <v>321566</v>
+        <v>329414</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -13719,7 +13719,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-08-14T09:06:55</t>
+          <t>2026-08-24T09:06:35</t>
         </is>
       </c>
     </row>
@@ -13831,7 +13831,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>35202</v>
+        <v>40554</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -13844,7 +13844,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>35202</v>
+        <v>40554</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -13853,7 +13853,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-08-14T09:07:04</t>
+          <t>2026-08-24T09:06:43</t>
         </is>
       </c>
     </row>
@@ -13894,33 +13894,33 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=W8yUZ6u3b3I</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>11983</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">インナージャーニー Inner Journey </t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=lrB8anaL9X4</t>
         </is>
       </c>
-      <c r="J70" t="n">
-        <v>10718</v>
-      </c>
-      <c r="K70" t="inlineStr">
+      <c r="M70" t="n">
+        <v>11927</v>
+      </c>
+      <c r="N70" t="inlineStr">
         <is>
           <t>KING AMUSEMENT CREATIVE official channel</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lrB8anaL9X4</t>
-        </is>
-      </c>
-      <c r="M70" t="n">
-        <v>10718</v>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>KING AMUSEMENT CREATIVE official channel</t>
-        </is>
-      </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-08-14T09:07:14</t>
+          <t>2026-08-24T09:06:52</t>
         </is>
       </c>
     </row>
@@ -13965,7 +13965,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>160156</v>
+        <v>180351</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -13978,7 +13978,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>160156</v>
+        <v>180351</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -13987,7 +13987,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-08-14T09:07:24</t>
+          <t>2026-08-24T09:07:01</t>
         </is>
       </c>
     </row>
@@ -14032,7 +14032,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>23377</v>
+        <v>28152</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -14045,7 +14045,7 @@
         </is>
       </c>
       <c r="M72" t="n">
-        <v>22465</v>
+        <v>25911</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
@@ -14054,7 +14054,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-08-14T09:07:33</t>
+          <t>2026-08-24T09:07:10</t>
         </is>
       </c>
     </row>
@@ -14323,7 +14323,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>140178</v>
+        <v>147035</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -14336,7 +14336,7 @@
         </is>
       </c>
       <c r="M77" t="n">
-        <v>29707</v>
+        <v>33208</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-08-14T09:07:44</t>
+          <t>2026-08-24T09:07:22</t>
         </is>
       </c>
     </row>
@@ -14390,7 +14390,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>766073</v>
+        <v>767656</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -14403,7 +14403,7 @@
         </is>
       </c>
       <c r="M78" t="n">
-        <v>766073</v>
+        <v>767656</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -14412,7 +14412,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-08-14T09:07:55</t>
+          <t>2026-08-24T09:07:30</t>
         </is>
       </c>
     </row>
@@ -14457,7 +14457,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>177928</v>
+        <v>179242</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -14470,7 +14470,7 @@
         </is>
       </c>
       <c r="M79" t="n">
-        <v>177928</v>
+        <v>179242</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -14479,7 +14479,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-08-14T09:08:07</t>
+          <t>2026-08-24T09:07:40</t>
         </is>
       </c>
     </row>
@@ -14524,7 +14524,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>387335</v>
+        <v>404657</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -14536,7 +14536,7 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-08-14T09:08:25</t>
+          <t>2026-08-24T09:07:58</t>
         </is>
       </c>
     </row>
@@ -14624,7 +14624,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>225887</v>
+        <v>227561</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -14637,7 +14637,7 @@
         </is>
       </c>
       <c r="M82" t="n">
-        <v>95741</v>
+        <v>101074</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -14646,7 +14646,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-08-14T09:08:37</t>
+          <t>2026-08-24T09:08:10</t>
         </is>
       </c>
     </row>
@@ -14754,33 +14754,33 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=QtlOSpxYoaE</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>1683039</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>SEKAI NO OWARI</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=_GlLp6hyM2E</t>
         </is>
       </c>
-      <c r="J84" t="n">
-        <v>1467016</v>
-      </c>
-      <c r="K84" t="inlineStr">
+      <c r="M84" t="n">
+        <v>1552544</v>
+      </c>
+      <c r="N84" t="inlineStr">
         <is>
           <t>tv asahi  animation YouTubeチャンネル</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=_GlLp6hyM2E</t>
-        </is>
-      </c>
-      <c r="M84" t="n">
-        <v>1467016</v>
-      </c>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>tv asahi  animation YouTubeチャンネル</t>
-        </is>
-      </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-08-14T09:08:46</t>
+          <t>2026-08-24T09:08:19</t>
         </is>
       </c>
     </row>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>816396</v>
+        <v>1226929</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -14838,7 +14838,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>292731</v>
+        <v>319695</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -14847,7 +14847,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-08-14T09:08:56</t>
+          <t>2026-08-24T09:08:28</t>
         </is>
       </c>
     </row>
@@ -15309,33 +15309,33 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=PX-b7KO3HOw</t>
+          <t>https://www.youtube.com/watch?v=NBHauNVLJa0</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>112928</v>
+        <v>119258</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>KyoaniChannel</t>
+          <t>Lantis Channel</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=PX-b7KO3HOw</t>
+          <t>https://www.youtube.com/watch?v=NBHauNVLJa0</t>
         </is>
       </c>
       <c r="M93" t="n">
-        <v>112928</v>
+        <v>119258</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>KyoaniChannel</t>
+          <t>Lantis Channel</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-08-14T09:09:15</t>
+          <t>2026-08-24T09:08:48</t>
         </is>
       </c>
     </row>
@@ -15380,7 +15380,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>95739</v>
+        <v>116997</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -15393,7 +15393,7 @@
         </is>
       </c>
       <c r="M94" t="n">
-        <v>51415</v>
+        <v>56981</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -15402,7 +15402,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-08-14T09:09:25</t>
+          <t>2026-08-24T09:08:57</t>
         </is>
       </c>
     </row>
@@ -15447,7 +15447,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>140078</v>
+        <v>150269</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -15460,7 +15460,7 @@
         </is>
       </c>
       <c r="M95" t="n">
-        <v>140078</v>
+        <v>150269</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -15469,7 +15469,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-08-14T09:09:34</t>
+          <t>2026-08-24T09:09:06</t>
         </is>
       </c>
     </row>
@@ -15667,7 +15667,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>469137</v>
+        <v>477514</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -15680,7 +15680,7 @@
         </is>
       </c>
       <c r="M99" t="n">
-        <v>469137</v>
+        <v>477514</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -15689,7 +15689,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-08-14T09:09:54</t>
+          <t>2026-08-24T09:09:24</t>
         </is>
       </c>
     </row>
@@ -15734,7 +15734,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>457369</v>
+        <v>497502</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -15747,7 +15747,7 @@
         </is>
       </c>
       <c r="M100" t="n">
-        <v>415580</v>
+        <v>431037</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -15756,7 +15756,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:04</t>
+          <t>2026-08-24T09:09:34</t>
         </is>
       </c>
     </row>
@@ -15801,7 +15801,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>398990</v>
+        <v>412790</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -15814,7 +15814,7 @@
         </is>
       </c>
       <c r="M101" t="n">
-        <v>355219</v>
+        <v>364123</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -15823,7 +15823,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:14</t>
+          <t>2026-08-24T09:09:43</t>
         </is>
       </c>
     </row>
@@ -15868,7 +15868,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>67866</v>
+        <v>70495</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -15881,7 +15881,7 @@
         </is>
       </c>
       <c r="M102" t="n">
-        <v>67866</v>
+        <v>70495</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -15890,7 +15890,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:23</t>
+          <t>2026-08-24T09:09:53</t>
         </is>
       </c>
     </row>
@@ -15935,7 +15935,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>59733</v>
+        <v>67631</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -15948,7 +15948,7 @@
         </is>
       </c>
       <c r="M103" t="n">
-        <v>59733</v>
+        <v>67631</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -15957,7 +15957,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:33</t>
+          <t>2026-08-24T09:10:01</t>
         </is>
       </c>
     </row>
@@ -16002,7 +16002,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>87087</v>
+        <v>103392</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -16015,7 +16015,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>87087</v>
+        <v>103392</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -16024,7 +16024,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:42</t>
+          <t>2026-08-24T09:10:10</t>
         </is>
       </c>
     </row>
@@ -16404,7 +16404,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>105409</v>
+        <v>123538</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -16417,7 +16417,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>105409</v>
+        <v>123538</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -16426,7 +16426,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:50</t>
+          <t>2026-08-24T09:10:19</t>
         </is>
       </c>
     </row>
@@ -16538,7 +16538,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>116698</v>
+        <v>134190</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -16551,7 +16551,7 @@
         </is>
       </c>
       <c r="M112" t="n">
-        <v>40040</v>
+        <v>44935</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -16560,7 +16560,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-08-14T09:10:59</t>
+          <t>2026-08-24T09:10:28</t>
         </is>
       </c>
     </row>
@@ -16605,7 +16605,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>23895</v>
+        <v>30323</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -16618,7 +16618,7 @@
         </is>
       </c>
       <c r="M113" t="n">
-        <v>19117</v>
+        <v>21698</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -16627,7 +16627,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-08-14T09:11:08</t>
+          <t>2026-08-24T09:10:37</t>
         </is>
       </c>
     </row>
@@ -16672,7 +16672,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>3479782</v>
+        <v>4882109</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -16685,7 +16685,7 @@
         </is>
       </c>
       <c r="M114" t="n">
-        <v>320546</v>
+        <v>394687</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -16694,7 +16694,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-08-14T09:11:18</t>
+          <t>2026-08-24T09:10:46</t>
         </is>
       </c>
     </row>
@@ -16806,7 +16806,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>567420</v>
+        <v>585181</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -16819,7 +16819,7 @@
         </is>
       </c>
       <c r="M116" t="n">
-        <v>567420</v>
+        <v>585181</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -16828,7 +16828,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-08-14T09:11:27</t>
+          <t>2026-08-24T09:10:55</t>
         </is>
       </c>
     </row>
@@ -16979,11 +16979,11 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IJONbpfIlUg</t>
+          <t>https://www.youtube.com/watch?v=9idm6v9jNbg</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>2026537</v>
+        <v>1951105</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -16996,7 +16996,7 @@
         </is>
       </c>
       <c r="M119" t="n">
-        <v>1620767</v>
+        <v>1951105</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -17005,7 +17005,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-08-14T09:11:40</t>
+          <t>2026-08-24T09:11:10</t>
         </is>
       </c>
     </row>
@@ -17046,11 +17046,11 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=9idm6v9jNbg</t>
+          <t>https://www.youtube.com/watch?v=E2c3V6nxjCw</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>1620767</v>
+        <v>1227795</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
@@ -17063,7 +17063,7 @@
         </is>
       </c>
       <c r="M120" t="n">
-        <v>1067245</v>
+        <v>1227795</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -17072,7 +17072,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-08-14T09:11:49</t>
+          <t>2026-08-24T09:11:20</t>
         </is>
       </c>
     </row>
@@ -17337,7 +17337,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>26916</v>
+        <v>30795</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -17350,7 +17350,7 @@
         </is>
       </c>
       <c r="M125" t="n">
-        <v>26916</v>
+        <v>30795</v>
       </c>
       <c r="N125" t="inlineStr">
         <is>
@@ -17359,7 +17359,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:10</t>
+          <t>2026-08-24T09:11:40</t>
         </is>
       </c>
     </row>
@@ -17571,7 +17571,7 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>106271</v>
+        <v>110549</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -17584,7 +17584,7 @@
         </is>
       </c>
       <c r="M129" t="n">
-        <v>106271</v>
+        <v>110549</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -17593,7 +17593,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:22</t>
+          <t>2026-08-24T09:11:51</t>
         </is>
       </c>
     </row>
@@ -17638,7 +17638,7 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>315546</v>
+        <v>330065</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -17651,7 +17651,7 @@
         </is>
       </c>
       <c r="M130" t="n">
-        <v>88494</v>
+        <v>92796</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -17660,7 +17660,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:31</t>
+          <t>2026-08-24T09:11:59</t>
         </is>
       </c>
     </row>
@@ -17701,33 +17701,33 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>646598</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
         </is>
       </c>
-      <c r="J131" t="n">
-        <v>481661</v>
-      </c>
-      <c r="K131" t="inlineStr">
+      <c r="M131" t="n">
+        <v>530844</v>
+      </c>
+      <c r="N131" t="inlineStr">
         <is>
           <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=_gBcPnxRXDY</t>
-        </is>
-      </c>
-      <c r="M131" t="n">
-        <v>481661</v>
-      </c>
-      <c r="N131" t="inlineStr">
-        <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
-        </is>
-      </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:41</t>
+          <t>2026-08-24T09:12:09</t>
         </is>
       </c>
     </row>
@@ -17772,7 +17772,7 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>644424</v>
+        <v>646598</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
@@ -17785,7 +17785,7 @@
         </is>
       </c>
       <c r="M132" t="n">
-        <v>110594</v>
+        <v>122838</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
@@ -17794,7 +17794,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-08-14T09:12:51</t>
+          <t>2026-08-24T09:12:18</t>
         </is>
       </c>
     </row>
@@ -17988,11 +17988,11 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=NEh3-Qmq1LE</t>
+          <t>https://www.youtube.com/watch?v=mUZEnAeUvgA</t>
         </is>
       </c>
       <c r="J136" t="n">
-        <v>4172283</v>
+        <v>7130264</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
@@ -18005,7 +18005,7 @@
         </is>
       </c>
       <c r="M136" t="n">
-        <v>247200</v>
+        <v>259618</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
@@ -18014,7 +18014,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:06</t>
+          <t>2026-08-24T09:12:34</t>
         </is>
       </c>
     </row>
@@ -18059,7 +18059,7 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>1389295</v>
+        <v>1394646</v>
       </c>
       <c r="K137" t="inlineStr">
         <is>
@@ -18072,7 +18072,7 @@
         </is>
       </c>
       <c r="M137" t="n">
-        <v>2583760</v>
+        <v>2609615</v>
       </c>
       <c r="N137" t="inlineStr">
         <is>
@@ -18081,7 +18081,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:26</t>
+          <t>2026-08-24T09:12:52</t>
         </is>
       </c>
     </row>
@@ -18126,7 +18126,7 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>48731</v>
+        <v>51394</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
@@ -18139,7 +18139,7 @@
         </is>
       </c>
       <c r="M138" t="n">
-        <v>15184</v>
+        <v>16719</v>
       </c>
       <c r="N138" t="inlineStr">
         <is>
@@ -18148,7 +18148,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:35</t>
+          <t>2026-08-24T09:13:01</t>
         </is>
       </c>
     </row>
@@ -18256,33 +18256,33 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=aRiVUVNUhIs</t>
+        </is>
+      </c>
+      <c r="J140" t="n">
+        <v>3716013</v>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>忘れらんねえよ</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
         </is>
       </c>
-      <c r="J140" t="n">
-        <v>1878435</v>
-      </c>
-      <c r="K140" t="inlineStr">
+      <c r="M140" t="n">
+        <v>2131230</v>
+      </c>
+      <c r="N140" t="inlineStr">
         <is>
           <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
         </is>
       </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=46Z-WQv_vFc</t>
-        </is>
-      </c>
-      <c r="M140" t="n">
-        <v>1878435</v>
-      </c>
-      <c r="N140" t="inlineStr">
-        <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
-        </is>
-      </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-08-14T09:13:45</t>
+          <t>2026-08-24T09:13:10</t>
         </is>
       </c>
     </row>
@@ -18327,29 +18327,19 @@
         </is>
       </c>
       <c r="J141" t="n">
-        <v>1878435</v>
+        <v>2131230</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
           <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TwumA6YhQp4</t>
-        </is>
-      </c>
-      <c r="M141" t="n">
-        <v>682471</v>
-      </c>
-      <c r="N141" t="inlineStr">
-        <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
-        </is>
-      </c>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:04</t>
+          <t>2026-08-24T09:13:39</t>
         </is>
       </c>
     </row>
@@ -18394,7 +18384,7 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>52502</v>
+        <v>56303</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
@@ -18406,7 +18396,7 @@
       <c r="N142" t="inlineStr"/>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:27</t>
+          <t>2026-08-24T09:14:01</t>
         </is>
       </c>
     </row>
@@ -18585,7 +18575,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>620248</v>
+        <v>623453</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -18598,7 +18588,7 @@
         </is>
       </c>
       <c r="M145" t="n">
-        <v>620248</v>
+        <v>623453</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -18607,7 +18597,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:37</t>
+          <t>2026-08-24T09:14:11</t>
         </is>
       </c>
     </row>
@@ -18648,33 +18638,33 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=G6u20QYskAU</t>
         </is>
       </c>
       <c r="J146" t="n">
-        <v>76836</v>
+        <v>88196</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
+          <t>Dannie May</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOyydxN5QFs</t>
+        </is>
+      </c>
+      <c r="M146" t="n">
+        <v>80173</v>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
           <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
         </is>
       </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
-        </is>
-      </c>
-      <c r="M146" t="n">
-        <v>76836</v>
-      </c>
-      <c r="N146" t="inlineStr">
-        <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
-        </is>
-      </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:47</t>
+          <t>2026-08-24T09:14:19</t>
         </is>
       </c>
     </row>
@@ -18719,7 +18709,7 @@
         </is>
       </c>
       <c r="J147" t="n">
-        <v>9540278</v>
+        <v>9557868</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -18732,7 +18722,7 @@
         </is>
       </c>
       <c r="M147" t="n">
-        <v>159358</v>
+        <v>160931</v>
       </c>
       <c r="N147" t="inlineStr">
         <is>
@@ -18741,7 +18731,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-08-14T09:14:57</t>
+          <t>2026-08-24T09:14:28</t>
         </is>
       </c>
     </row>
@@ -18786,7 +18776,7 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>82663</v>
+        <v>83197</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
@@ -18799,7 +18789,7 @@
         </is>
       </c>
       <c r="M148" t="n">
-        <v>82663</v>
+        <v>83197</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -18808,7 +18798,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-08-14T09:15:06</t>
+          <t>2026-08-24T09:14:43</t>
         </is>
       </c>
     </row>
@@ -18853,7 +18843,7 @@
         </is>
       </c>
       <c r="J149" t="n">
-        <v>17187</v>
+        <v>26827</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -18865,7 +18855,7 @@
       <c r="N149" t="inlineStr"/>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-08-14T09:15:28</t>
+          <t>2026-08-24T09:15:05</t>
         </is>
       </c>
     </row>
@@ -19053,7 +19043,7 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>15827</v>
+        <v>18986</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
@@ -19066,7 +19056,7 @@
         </is>
       </c>
       <c r="M153" t="n">
-        <v>15827</v>
+        <v>18986</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -19075,7 +19065,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-08-14T09:15:38</t>
+          <t>2026-08-24T09:15:15</t>
         </is>
       </c>
     </row>
@@ -19120,7 +19110,7 @@
         </is>
       </c>
       <c r="J154" t="n">
-        <v>60653</v>
+        <v>62164</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
@@ -19133,7 +19123,7 @@
         </is>
       </c>
       <c r="M154" t="n">
-        <v>60653</v>
+        <v>62164</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -19142,7 +19132,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-08-14T09:15:48</t>
+          <t>2026-08-24T09:15:25</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19220,7 @@
         </is>
       </c>
       <c r="J156" t="n">
-        <v>210495</v>
+        <v>218213</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -19243,7 +19233,7 @@
         </is>
       </c>
       <c r="M156" t="n">
-        <v>210495</v>
+        <v>218213</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -19252,7 +19242,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:00</t>
+          <t>2026-08-24T09:15:37</t>
         </is>
       </c>
     </row>
@@ -19364,7 +19354,7 @@
         </is>
       </c>
       <c r="J158" t="n">
-        <v>873424</v>
+        <v>913624</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -19377,7 +19367,7 @@
         </is>
       </c>
       <c r="M158" t="n">
-        <v>873424</v>
+        <v>913624</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -19386,7 +19376,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:09</t>
+          <t>2026-08-24T09:15:49</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19421,7 @@
         </is>
       </c>
       <c r="J159" t="n">
-        <v>220163</v>
+        <v>240147</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -19444,7 +19434,7 @@
         </is>
       </c>
       <c r="M159" t="n">
-        <v>84624</v>
+        <v>89739</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -19453,7 +19443,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:19</t>
+          <t>2026-08-24T09:15:58</t>
         </is>
       </c>
     </row>
@@ -19561,11 +19551,11 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+          <t>https://www.youtube.com/watch?v=6f78rxIxzV0</t>
         </is>
       </c>
       <c r="J161" t="n">
-        <v>327343</v>
+        <v>341078</v>
       </c>
       <c r="K161" t="inlineStr">
         <is>
@@ -19574,11 +19564,11 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+          <t>https://www.youtube.com/watch?v=6f78rxIxzV0</t>
         </is>
       </c>
       <c r="M161" t="n">
-        <v>327343</v>
+        <v>341078</v>
       </c>
       <c r="N161" t="inlineStr">
         <is>
@@ -19587,7 +19577,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:28</t>
+          <t>2026-08-24T09:16:08</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19689,7 @@
         </is>
       </c>
       <c r="J163" t="n">
-        <v>645741</v>
+        <v>659079</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19712,7 +19702,7 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>645741</v>
+        <v>659079</v>
       </c>
       <c r="N163" t="inlineStr">
         <is>
@@ -19721,7 +19711,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:38</t>
+          <t>2026-08-24T09:16:18</t>
         </is>
       </c>
     </row>
@@ -19809,7 +19799,7 @@
         </is>
       </c>
       <c r="J165" t="n">
-        <v>61702</v>
+        <v>66884</v>
       </c>
       <c r="K165" t="inlineStr">
         <is>
@@ -19822,7 +19812,7 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>621764</v>
+        <v>623677</v>
       </c>
       <c r="N165" t="inlineStr">
         <is>
@@ -19831,7 +19821,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-08-14T09:16:50</t>
+          <t>2026-08-24T09:16:30</t>
         </is>
       </c>
     </row>
@@ -20105,7 +20095,7 @@
         </is>
       </c>
       <c r="J171" t="n">
-        <v>187036</v>
+        <v>187718</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20118,7 +20108,7 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>187036</v>
+        <v>187718</v>
       </c>
       <c r="N171" t="inlineStr">
         <is>
@@ -20127,7 +20117,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-08-17T09:01:55</t>
+          <t>2026-08-24T09:17:05</t>
         </is>
       </c>
     </row>
@@ -20301,7 +20291,7 @@
         </is>
       </c>
       <c r="J175" t="n">
-        <v>121723</v>
+        <v>164875</v>
       </c>
       <c r="K175" t="inlineStr">
         <is>
@@ -20313,7 +20303,7 @@
       <c r="N175" t="inlineStr"/>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-08-17T09:02:20</t>
+          <t>2026-08-24T09:17:30</t>
         </is>
       </c>
     </row>
@@ -20530,7 +20520,7 @@
         </is>
       </c>
       <c r="J180" t="n">
-        <v>702298</v>
+        <v>711649</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
@@ -20543,7 +20533,7 @@
         </is>
       </c>
       <c r="M180" t="n">
-        <v>702298</v>
+        <v>711649</v>
       </c>
       <c r="N180" t="inlineStr">
         <is>
@@ -20552,7 +20542,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-08-14T09:17:59</t>
+          <t>2026-08-24T09:17:54</t>
         </is>
       </c>
     </row>
@@ -20597,7 +20587,7 @@
         </is>
       </c>
       <c r="J181" t="n">
-        <v>389648</v>
+        <v>397704</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
@@ -20610,7 +20600,7 @@
         </is>
       </c>
       <c r="M181" t="n">
-        <v>389648</v>
+        <v>397704</v>
       </c>
       <c r="N181" t="inlineStr">
         <is>
@@ -20619,7 +20609,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-08-14T09:18:08</t>
+          <t>2026-08-24T09:18:04</t>
         </is>
       </c>
     </row>
@@ -21204,7 +21194,7 @@
         </is>
       </c>
       <c r="J194" t="n">
-        <v>3908</v>
+        <v>4470</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -21217,7 +21207,7 @@
         </is>
       </c>
       <c r="M194" t="n">
-        <v>3908</v>
+        <v>4470</v>
       </c>
       <c r="N194" t="inlineStr">
         <is>
@@ -21226,7 +21216,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-08-14T09:19:30</t>
+          <t>2026-08-24T09:19:40</t>
         </is>
       </c>
     </row>
@@ -21271,7 +21261,7 @@
         </is>
       </c>
       <c r="J195" t="n">
-        <v>747589</v>
+        <v>757285</v>
       </c>
       <c r="K195" t="inlineStr">
         <is>
@@ -21283,7 +21273,7 @@
       <c r="N195" t="inlineStr"/>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-08-17T09:04:05</t>
+          <t>2026-08-24T09:19:55</t>
         </is>
       </c>
     </row>
@@ -21328,7 +21318,7 @@
         </is>
       </c>
       <c r="J196" t="n">
-        <v>107293</v>
+        <v>107820</v>
       </c>
       <c r="K196" t="inlineStr">
         <is>
@@ -21340,7 +21330,7 @@
       <c r="N196" t="inlineStr"/>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-08-14T09:19:44</t>
+          <t>2026-08-24T09:20:11</t>
         </is>
       </c>
     </row>
@@ -21648,7 +21638,7 @@
         </is>
       </c>
       <c r="J202" t="n">
-        <v>917131</v>
+        <v>973031</v>
       </c>
       <c r="K202" t="inlineStr">
         <is>
@@ -21661,7 +21651,7 @@
         </is>
       </c>
       <c r="M202" t="n">
-        <v>391594</v>
+        <v>401379</v>
       </c>
       <c r="N202" t="inlineStr">
         <is>
@@ -21670,7 +21660,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-08-14T09:20:08</t>
+          <t>2026-08-24T09:20:37</t>
         </is>
       </c>
     </row>
@@ -21715,7 +21705,7 @@
         </is>
       </c>
       <c r="J203" t="n">
-        <v>411712</v>
+        <v>434141</v>
       </c>
       <c r="K203" t="inlineStr">
         <is>
@@ -21728,7 +21718,7 @@
         </is>
       </c>
       <c r="M203" t="n">
-        <v>402485</v>
+        <v>409527</v>
       </c>
       <c r="N203" t="inlineStr">
         <is>
@@ -21737,7 +21727,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-08-14T09:20:18</t>
+          <t>2026-08-24T09:20:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-25
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M173"/>
+  <dimension ref="A1:M177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026年10月1日（木）〜 テレビ神奈川・CBCテレビにて</t>
+          <t>2026年10月1日（木）〜 テレビ神奈川ほか</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026年10月6日（火）～ TOKYO MX・MBS ほか</t>
+          <t>2026年10月6日（火）～ TOKYO MX・ＢＳ日テレほか</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX ほか</t>
+          <t>2026年10月～ TOKYO MX・関西テレビほか</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -6389,7 +6389,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026年秋 Netflixにて</t>
+          <t>2026年10月20日（火）～ Netflixにて</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月7日（水）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -6986,12 +6986,20 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>風の中は走るっきゃないっ！</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>三月のパンタシア</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
@@ -7145,7 +7153,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7158,37 +7166,29 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+          <t>2026年10月～ BSフジ・フジテレビほか</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>OLM</t>
+          <t>Production +h.</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
-        </is>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>SUPER★DRAGON</t>
-        </is>
-      </c>
+          <t>BUCK∞TICK</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27123</t>
         </is>
       </c>
     </row>
@@ -7206,7 +7206,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7219,17 +7219,37 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
+          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Let's Go Crazy</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
         </is>
       </c>
     </row>
@@ -7247,7 +7267,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7260,37 +7280,21 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ TOKYO MX・BS11ほか</t>
+          <t>2026年10月4日（日）～ テレ東系にて</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>DALALA</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>SiM</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>SYNC</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>Daoko</t>
-        </is>
-      </c>
+          <t>アカツキメディアスタジオ</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -7308,7 +7312,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7321,21 +7325,37 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月4日（日）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>ENGI</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
+          <t>ポリゴン・ピクチュアズ</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>DALALA</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Daoko</t>
+        </is>
+      </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -7353,7 +7373,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7366,37 +7386,21 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>feel.</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>ライアー</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>陽炎</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
+          <t>ENGI</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7418,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7427,21 +7431,37 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年10月6日（火）〜 カンテレ・フジテレビ系全国ネットにて</t>
+          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
+          <t>feel.</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>ライアー</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>陽炎</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>サイダーガール</t>
+        </is>
+      </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7479,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7472,12 +7492,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月6日（火）〜 カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I131" t="inlineStr"/>
@@ -7486,7 +7506,7 @@
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -7504,7 +7524,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7517,29 +7537,21 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>わたし未来線</t>
-        </is>
-      </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -7557,7 +7569,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7575,16 +7587,24 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>わたし未来線</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+        </is>
+      </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -7602,7 +7622,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7610,34 +7630,42 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年11月6日（金） Prime Videoにて</t>
+          <t>2026年10月2日（金）～ TOKYO MX・BS11にて</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Production I.G</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
+          <t>Re:name</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Ray of Emotion</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>導凰</t>
+        </is>
+      </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -7655,7 +7683,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7663,26 +7691,34 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年11月6日（金） Prime Videoにて</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
-        </is>
-      </c>
-      <c r="I135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
+          <t>Production I.G</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>シンカ</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Ado</t>
+        </is>
+      </c>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
         </is>
       </c>
     </row>
@@ -7700,7 +7736,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7708,26 +7744,42 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月9日（金）〜 デュエル・マスターズ公式YouTubeチャンネルにて</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
-        </is>
-      </c>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
-      <c r="L136" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>あやかしあやし</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>朔日 feat. 吉乃</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>月詠み</t>
+        </is>
+      </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27820</t>
         </is>
       </c>
     </row>
@@ -7745,7 +7797,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7758,37 +7810,21 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>studio MOTHER</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -7806,7 +7842,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7819,37 +7855,21 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ TOKYO MX ほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>DREAM OF BUTTERFLY</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>FZMZ</t>
-        </is>
-      </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>バリバリBuddy</t>
-        </is>
-      </c>
-      <c r="L138" t="inlineStr">
-        <is>
-          <t>花冷え。</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -7867,7 +7887,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7880,37 +7900,37 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>FelixFilm</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7928,7 +7948,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7941,37 +7961,37 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年10月7日（水）～ TOKYO MX ほか</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>JO1</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7989,7 +8009,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -8002,17 +8022,37 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H141" t="inlineStr"/>
-      <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
+          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Ghost Sequence</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>原子崩し(メルトダウナー)</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -8030,7 +8070,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -8043,21 +8083,37 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>IGNITE</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>トリックスター</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -8075,7 +8131,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -8088,7 +8144,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
         </is>
       </c>
       <c r="H143" t="inlineStr"/>
@@ -8098,7 +8154,7 @@
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -8116,7 +8172,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>dreamland</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -8129,17 +8185,21 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年10月～ ABCテレビ・テレビ朝日ほか</t>
-        </is>
-      </c>
-      <c r="H144" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28811</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -8157,7 +8217,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8165,26 +8225,22 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年9月5日（土）～ YouTube「TOHO animation」チャンネルほか</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8258,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>dreamland</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8215,7 +8271,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ NHK Eテレにて</t>
+          <t>2026年10月～ ABCテレビ・テレビ朝日ほか</t>
         </is>
       </c>
       <c r="H146" t="inlineStr"/>
@@ -8225,7 +8281,7 @@
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26728</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28811</t>
         </is>
       </c>
     </row>
@@ -8243,7 +8299,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8251,17 +8307,17 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
+          <t>2026年9月5日（土）～ YouTube「TOHO animation」チャンネルほか</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -8270,7 +8326,7 @@
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -8288,7 +8344,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8301,7 +8357,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月3日（土）～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H148" t="inlineStr"/>
@@ -8311,7 +8367,7 @@
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26728</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8385,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8342,25 +8398,21 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>パンどろぼうのうた</t>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
+          <t>2026年10月3日（土）～ TOKYO MX・BS11ほか</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -8378,7 +8430,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>人付き合いが苦手な未亡人の雪女さんと呪いの指輪</t>
+          <t>Bass X Machina: バス X マキナ</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8386,26 +8438,22 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>studio HōKIBOSHI</t>
-        </is>
-      </c>
+          <t>2026年11月3日（火）～ Netflixにて</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28885</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28983</t>
         </is>
       </c>
     </row>
@@ -8423,7 +8471,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8436,7 +8484,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H151" t="inlineStr"/>
@@ -8446,7 +8494,7 @@
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8512,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8477,21 +8525,25 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026年10月〜 TBS・BS11にて</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
+          <t>2026年10月〜 NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>パンどろぼうのうた</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -8509,7 +8561,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>人付き合いが苦手な未亡人の雪女さんと呪いの指輪</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8522,29 +8574,21 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>studio HōKIBOSHI</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28885</t>
         </is>
       </c>
     </row>
@@ -8562,7 +8606,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>僕らが選んだベストアドベンチャー</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E154" t="b">
@@ -8575,7 +8619,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ フジテレビほか</t>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
         </is>
       </c>
       <c r="H154" t="inlineStr"/>
@@ -8585,7 +8629,7 @@
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16416</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -8603,7 +8647,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E155" t="b">
@@ -8616,29 +8660,37 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月8日（木）～ TBS・BS11にて</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Diamond Dust</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Sizuk</t>
+        </is>
+      </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
+          <t>内田真礼</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -8656,7 +8708,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>フールナイト</t>
         </is>
       </c>
       <c r="E156" t="b">
@@ -8664,17 +8716,17 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年11月26日（木）～ Netflixにて</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>サンライズ</t>
         </is>
       </c>
       <c r="I156" t="inlineStr"/>
@@ -8683,7 +8735,7 @@
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28621</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8753,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E157" t="b">
@@ -8719,16 +8771,24 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -8746,7 +8806,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>僕らが選んだベストアドベンチャー</t>
         </is>
       </c>
       <c r="E158" t="b">
@@ -8759,21 +8819,17 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>WHITE FOX</t>
-        </is>
-      </c>
+          <t>2026年10月4日（日）～ フジテレビほか</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16416</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8847,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E159" t="b">
@@ -8804,21 +8860,29 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年10月9日（金）～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
       <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>夢心地</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>TOOBOE</t>
+        </is>
+      </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -8836,7 +8900,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E160" t="b">
@@ -8849,29 +8913,21 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月4日（日）～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>MOZU STUDIOS</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
       <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -8889,7 +8945,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E161" t="b">
@@ -8902,37 +8958,21 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr">
-        <is>
-          <t>Bubee</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K161" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>ブリッジ</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8950,7 +8990,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E162" t="b">
@@ -8963,12 +9003,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ NHK Eテレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I162" t="inlineStr"/>
@@ -8977,7 +9017,7 @@
       <c r="L162" t="inlineStr"/>
       <c r="M162" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8995,7 +9035,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E163" t="b">
@@ -9008,37 +9048,21 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J163" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K163" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L163" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
       <c r="M163" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -9056,7 +9080,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E164" t="b">
@@ -9069,29 +9093,29 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MXほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>ワオワールド</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -9109,7 +9133,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>ゆうさんち！from 遊ハち</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E165" t="b">
@@ -9122,21 +9146,37 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026年10月～ フジテレビ・カンテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>ファンワークス</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28884</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -9154,7 +9194,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E166" t="b">
@@ -9167,12 +9207,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年10月3日（土）～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -9181,7 +9221,7 @@
       <c r="L166" t="inlineStr"/>
       <c r="M166" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -9199,7 +9239,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E167" t="b">
@@ -9212,37 +9252,37 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
+          <t>studio A-CAT</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Shalala</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
+          <t>ASTERISM</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -9260,7 +9300,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="E168" t="b">
@@ -9273,21 +9313,29 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月〜 TOKYO MXほか</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
+          <t>ワオワールド</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
       <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27288</t>
         </is>
       </c>
     </row>
@@ -9305,7 +9353,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>楽楽飯店</t>
+          <t>ゆうさんち！from 遊ハち</t>
         </is>
       </c>
       <c r="E169" t="b">
@@ -9313,22 +9361,26 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026年9月下旬 公式YouTubeチャンネルにて</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr"/>
+          <t>2026年10月～ フジテレビ・カンテレにて</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>ファンワークス</t>
+        </is>
+      </c>
       <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28945</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28884</t>
         </is>
       </c>
     </row>
@@ -9346,11 +9398,11 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E170" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -9359,12 +9411,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>Imagica Infos</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -9373,7 +9425,7 @@
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -9391,7 +9443,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E171" t="b">
@@ -9404,17 +9456,37 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ 日本テレビにて</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr"/>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -9432,7 +9504,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E172" t="b">
@@ -9440,22 +9512,26 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>寿門堂</t>
+        </is>
+      </c>
       <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -9473,7 +9549,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ロメリア戦記</t>
+          <t>楽楽飯店</t>
         </is>
       </c>
       <c r="E173" t="b">
@@ -9481,24 +9557,192 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>Atra</t>
-        </is>
-      </c>
+          <t>2026年9月下旬 公式YouTubeチャンネルにて</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28945</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>86</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+        </is>
+      </c>
+      <c r="E174" t="b">
+        <v>1</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>87</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>らんま1/2 第3期</t>
+        </is>
+      </c>
+      <c r="E175" t="b">
+        <v>0</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>2026年10月3日（土）～ 日本テレビにて</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>88</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E176" t="b">
+        <v>0</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>89</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>ロメリア戦記</t>
+        </is>
+      </c>
+      <c r="E177" t="b">
+        <v>0</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>2026年10月〜 TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Atra</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27077</t>
         </is>
@@ -9515,7 +9759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O203"/>
+  <dimension ref="A1:O211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12874,7 +13118,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>20934</v>
+        <v>21948</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -12887,7 +13131,7 @@
         </is>
       </c>
       <c r="M54" t="n">
-        <v>20934</v>
+        <v>21948</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -12896,7 +13140,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-08-18T09:03:46</t>
+          <t>2026-08-25T09:05:19</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17404,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>2342523</v>
+        <v>2362151</v>
       </c>
       <c r="K122" t="inlineStr">
         <is>
@@ -17173,7 +17417,7 @@
         </is>
       </c>
       <c r="M122" t="n">
-        <v>2342523</v>
+        <v>2362151</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -17182,7 +17426,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-08-18T09:05:05</t>
+          <t>2026-08-25T09:06:48</t>
         </is>
       </c>
     </row>
@@ -17227,7 +17471,7 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>224085</v>
+        <v>230943</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -17240,7 +17484,7 @@
         </is>
       </c>
       <c r="M123" t="n">
-        <v>224085</v>
+        <v>230943</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
@@ -17249,7 +17493,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-08-18T09:05:15</t>
+          <t>2026-08-25T09:06:59</t>
         </is>
       </c>
     </row>
@@ -17504,7 +17748,7 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>160367</v>
+        <v>160554</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -17517,7 +17761,7 @@
         </is>
       </c>
       <c r="M128" t="n">
-        <v>160367</v>
+        <v>160554</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -17526,7 +17770,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-08-18T09:05:26</t>
+          <t>2026-08-25T09:07:11</t>
         </is>
       </c>
     </row>
@@ -20038,19 +20282,29 @@
         </is>
       </c>
       <c r="J170" t="n">
-        <v>1189561</v>
+        <v>1545312</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
           <t>TOHO animation</t>
         </is>
       </c>
-      <c r="L170" t="inlineStr"/>
-      <c r="M170" t="inlineStr"/>
-      <c r="N170" t="inlineStr"/>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
+        </is>
+      </c>
+      <c r="M170" t="n">
+        <v>7582011</v>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-08-18T09:06:27</t>
+          <t>2026-08-25T09:08:32</t>
         </is>
       </c>
     </row>
@@ -20318,7 +20572,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -20334,12 +20588,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>風の中は走るっきゃないっ！</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>三月のパンタシア</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -20361,7 +20615,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -20369,7 +20623,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -20377,12 +20631,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -20404,7 +20658,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -20420,12 +20674,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I178" t="inlineStr"/>
@@ -20447,7 +20701,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -20463,12 +20717,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>SUPER★DRAGON</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -20490,7 +20744,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -20506,45 +20760,21 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J180" t="n">
-        <v>711649</v>
-      </c>
-      <c r="K180" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L180" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M180" t="n">
-        <v>711649</v>
-      </c>
-      <c r="N180" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O180" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:17:54</t>
-        </is>
-      </c>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -20557,7 +20787,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -20573,45 +20803,21 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="J181" t="n">
-        <v>397704</v>
-      </c>
-      <c r="K181" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L181" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M181" t="n">
-        <v>397704</v>
-      </c>
-      <c r="N181" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O181" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:18:04</t>
-        </is>
-      </c>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -20624,7 +20830,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -20632,7 +20838,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -20640,21 +20846,45 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr"/>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
-      <c r="M182" t="inlineStr"/>
-      <c r="N182" t="inlineStr"/>
-      <c r="O182" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>711649</v>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M182" t="n">
+        <v>711649</v>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:17:54</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -20667,7 +20897,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -20675,7 +20905,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -20683,21 +20913,45 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr"/>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
-      <c r="M183" t="inlineStr"/>
-      <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>397704</v>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M183" t="n">
+        <v>397704</v>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:18:04</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -20710,7 +20964,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -20718,7 +20972,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -20726,12 +20980,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
@@ -20753,7 +21007,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -20761,7 +21015,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -20769,12 +21023,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>Re:name</t>
         </is>
       </c>
       <c r="I185" t="inlineStr"/>
@@ -20796,7 +21050,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -20804,7 +21058,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -20812,12 +21066,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>FZMZ</t>
+          <t>導凰</t>
         </is>
       </c>
       <c r="I186" t="inlineStr"/>
@@ -20839,7 +21093,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D187" t="b">
@@ -20847,7 +21101,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -20855,12 +21109,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I187" t="inlineStr"/>
@@ -20882,7 +21136,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D188" t="b">
@@ -20898,21 +21152,35 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr"/>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+        </is>
+      </c>
+      <c r="J188" t="n">
+        <v>48992</v>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr"/>
-      <c r="O188" t="inlineStr"/>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:10:14</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -20925,7 +21193,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D189" t="b">
@@ -20941,21 +21209,45 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr"/>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
-      <c r="O189" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J189" t="n">
+        <v>46450</v>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M189" t="n">
+        <v>46450</v>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:10:21</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -20968,7 +21260,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D190" t="b">
@@ -20984,12 +21276,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>JO1</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I190" t="inlineStr"/>
@@ -21011,7 +21303,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D191" t="b">
@@ -21027,45 +21319,21 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
-        </is>
-      </c>
-      <c r="J191" t="n">
-        <v>17851</v>
-      </c>
-      <c r="K191" t="inlineStr">
-        <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M191" t="n">
-        <v>3801597</v>
-      </c>
-      <c r="N191" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
-      <c r="O191" t="inlineStr">
-        <is>
-          <t>2026-08-21T09:03:35</t>
-        </is>
-      </c>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
+      <c r="N191" t="inlineStr"/>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -21078,7 +21346,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D192" t="b">
@@ -21086,7 +21354,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -21094,12 +21362,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I192" t="inlineStr"/>
@@ -21121,7 +21389,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -21129,7 +21397,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -21137,12 +21405,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I193" t="inlineStr"/>
@@ -21164,7 +21432,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D194" t="b">
@@ -21180,45 +21448,21 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J194" t="n">
-        <v>4470</v>
-      </c>
-      <c r="K194" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L194" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M194" t="n">
-        <v>4470</v>
-      </c>
-      <c r="N194" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O194" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:19:40</t>
-        </is>
-      </c>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="inlineStr"/>
+      <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -21231,7 +21475,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D195" t="b">
@@ -21247,35 +21491,21 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J195" t="n">
-        <v>757285</v>
-      </c>
-      <c r="K195" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr"/>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:19:55</t>
-        </is>
-      </c>
+      <c r="O195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -21288,7 +21518,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D196" t="b">
@@ -21304,35 +21534,21 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
-        </is>
-      </c>
-      <c r="J196" t="n">
-        <v>107820</v>
-      </c>
-      <c r="K196" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr"/>
       <c r="L196" t="inlineStr"/>
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr"/>
-      <c r="O196" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:20:11</t>
-        </is>
-      </c>
+      <c r="O196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -21345,7 +21561,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D197" t="b">
@@ -21353,7 +21569,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -21361,43 +21577,43 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>go!go!vanillas</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
         </is>
       </c>
       <c r="J197" t="n">
-        <v>307069</v>
+        <v>17851</v>
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
+          <t>go!go!vanillas</t>
         </is>
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
         </is>
       </c>
       <c r="M197" t="n">
-        <v>307069</v>
+        <v>3801597</v>
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
+          <t>TV anime "Tokyo Revengers"</t>
         </is>
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-08-20T09:12:04</t>
+          <t>2026-08-21T09:03:35</t>
         </is>
       </c>
     </row>
@@ -21412,7 +21628,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D198" t="b">
@@ -21420,7 +21636,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -21428,45 +21644,21 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J198" t="n">
-        <v>307070</v>
-      </c>
-      <c r="K198" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L198" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M198" t="n">
-        <v>307070</v>
-      </c>
-      <c r="N198" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O198" t="inlineStr">
-        <is>
-          <t>2026-08-20T09:12:14</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr"/>
+      <c r="L198" t="inlineStr"/>
+      <c r="M198" t="inlineStr"/>
+      <c r="N198" t="inlineStr"/>
+      <c r="O198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -21479,7 +21671,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D199" t="b">
@@ -21495,12 +21687,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
       <c r="I199" t="inlineStr"/>
@@ -21522,7 +21714,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D200" t="b">
@@ -21530,7 +21722,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -21538,12 +21730,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
+          <t>Sizuk</t>
         </is>
       </c>
       <c r="I200" t="inlineStr"/>
@@ -21565,7 +21757,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D201" t="b">
@@ -21573,7 +21765,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -21581,12 +21773,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>内田真礼</t>
         </is>
       </c>
       <c r="I201" t="inlineStr"/>
@@ -21608,7 +21800,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D202" t="b">
@@ -21624,43 +21816,43 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J202" t="n">
-        <v>973031</v>
+        <v>4470</v>
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+          <t>Anime Trailer アニメ</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="M202" t="n">
-        <v>401379</v>
+        <v>4470</v>
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t>NBCUniversal Anime/Music</t>
+          <t>Anime Trailer アニメ</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-08-24T09:20:37</t>
+          <t>2026-08-24T09:19:40</t>
         </is>
       </c>
     </row>
@@ -21675,7 +21867,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D203" t="b">
@@ -21691,41 +21883,485 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
+          <t>夢心地</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>TOOBOE</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+        </is>
+      </c>
+      <c r="J203" t="n">
+        <v>757285</v>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr"/>
+      <c r="M203" t="inlineStr"/>
+      <c r="N203" t="inlineStr"/>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:19:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D204" t="b">
+        <v>0</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>1</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J204" t="n">
+        <v>107820</v>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="inlineStr"/>
+      <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:20:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+        </is>
+      </c>
+      <c r="D205" t="b">
+        <v>0</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>1</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J205" t="n">
+        <v>307069</v>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M205" t="n">
+        <v>307069</v>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>2026-08-20T09:12:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+        </is>
+      </c>
+      <c r="D206" t="b">
+        <v>0</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>1</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J206" t="n">
+        <v>307070</v>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M206" t="n">
+        <v>307070</v>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>2026-08-20T09:12:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+        </is>
+      </c>
+      <c r="D207" t="b">
+        <v>0</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>1</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr"/>
+      <c r="L207" t="inlineStr"/>
+      <c r="M207" t="inlineStr"/>
+      <c r="N207" t="inlineStr"/>
+      <c r="O207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+        </is>
+      </c>
+      <c r="D208" t="b">
+        <v>0</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>1</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr"/>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr"/>
+      <c r="L208" t="inlineStr"/>
+      <c r="M208" t="inlineStr"/>
+      <c r="N208" t="inlineStr"/>
+      <c r="O208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>野生のラスボスが現れた！ 第2期</t>
+        </is>
+      </c>
+      <c r="D209" t="b">
+        <v>0</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>1</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
+      <c r="N209" t="inlineStr"/>
+      <c r="O209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D210" t="b">
+        <v>0</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>1</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J210" t="n">
+        <v>973031</v>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M210" t="n">
+        <v>401379</v>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:20:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D211" t="b">
+        <v>0</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>1</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr">
+      <c r="H211" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I203" t="inlineStr">
+      <c r="I211" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
-      <c r="J203" t="n">
+      <c r="J211" t="n">
         <v>434141</v>
       </c>
-      <c r="K203" t="inlineStr">
+      <c r="K211" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="L203" t="inlineStr">
+      <c r="L211" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M203" t="n">
+      <c r="M211" t="n">
         <v>409527</v>
       </c>
-      <c r="N203" t="inlineStr">
+      <c r="N211" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O203" t="inlineStr">
+      <c r="O211" t="inlineStr">
         <is>
           <t>2026-08-24T09:20:46</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-28
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -5620,7 +5620,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>アオのハコ 第2期</t>
+          <t>アオのハコ Season2</t>
         </is>
       </c>
       <c r="E92" t="b">
@@ -5641,10 +5641,26 @@
           <t>エレクトリックサーカス</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>あなたの花の色</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>aiko</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>blue in</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>エルスウェア紀行</t>
+        </is>
+      </c>
       <c r="M92" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
@@ -8725,7 +8741,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月7日（水）〜 フジテレビ「B8station」にて</t>
         </is>
       </c>
       <c r="H156" t="inlineStr"/>
@@ -9914,7 +9930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O214"/>
+  <dimension ref="A1:O216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10145,7 +10161,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>654932</v>
+        <v>662388</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10157,7 +10173,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-08-20T09:00:32</t>
+          <t>2026-08-28T09:00:33</t>
         </is>
       </c>
     </row>
@@ -10757,7 +10773,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>114483</v>
+        <v>120396</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -10770,7 +10786,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>254678</v>
+        <v>254804</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -10779,7 +10795,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-08-20T09:00:55</t>
+          <t>2026-08-28T09:00:57</t>
         </is>
       </c>
     </row>
@@ -10824,29 +10840,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>691632</v>
+        <v>789146</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>MARUMOCHI from HoneyWorks</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=waOUdRPozDY</t>
-        </is>
-      </c>
-      <c r="M15" t="n">
-        <v>23230</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>GOOD SMILE CHANNEL</t>
-        </is>
-      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-08-20T09:01:04</t>
+          <t>2026-08-28T09:01:16</t>
         </is>
       </c>
     </row>
@@ -10891,7 +10897,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>108834</v>
+        <v>118446</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -10904,7 +10910,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>108834</v>
+        <v>118446</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -10913,7 +10919,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-08-20T09:01:13</t>
+          <t>2026-08-28T09:01:25</t>
         </is>
       </c>
     </row>
@@ -10958,7 +10964,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>301287</v>
+        <v>329147</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -10971,7 +10977,7 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>301287</v>
+        <v>329147</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -10980,7 +10986,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-08-20T09:01:22</t>
+          <t>2026-08-28T09:01:35</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11208,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>6915723</v>
+        <v>6935648</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -11215,7 +11221,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>130414</v>
+        <v>139143</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -11224,7 +11230,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-08-20T09:01:33</t>
+          <t>2026-08-28T09:01:47</t>
         </is>
       </c>
     </row>
@@ -11336,7 +11342,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>284264</v>
+        <v>322061</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -11349,7 +11355,7 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>111799</v>
+        <v>128501</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -11358,7 +11364,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-08-20T09:01:42</t>
+          <t>2026-08-28T09:01:55</t>
         </is>
       </c>
     </row>
@@ -11757,7 +11763,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>873090</v>
+        <v>1026443</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -11770,7 +11776,7 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>459429</v>
+        <v>536939</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -11779,7 +11785,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-08-20T09:01:51</t>
+          <t>2026-08-28T09:02:05</t>
         </is>
       </c>
     </row>
@@ -12015,7 +12021,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>23944</v>
+        <v>27550</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -12027,7 +12033,7 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-08-20T09:02:20</t>
+          <t>2026-08-28T09:02:37</t>
         </is>
       </c>
     </row>
@@ -12072,7 +12078,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>94247</v>
+        <v>110702</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -12085,7 +12091,7 @@
         </is>
       </c>
       <c r="M35" t="n">
-        <v>1266492</v>
+        <v>1280989</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -12094,7 +12100,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-08-20T09:02:40</t>
+          <t>2026-08-28T09:02:56</t>
         </is>
       </c>
     </row>
@@ -12182,7 +12188,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>111905</v>
+        <v>126774</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -12195,7 +12201,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>111905</v>
+        <v>126774</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -12204,7 +12210,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-08-20T09:02:52</t>
+          <t>2026-08-28T09:03:07</t>
         </is>
       </c>
     </row>
@@ -12249,7 +12255,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>103091</v>
+        <v>117514</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -12262,7 +12268,7 @@
         </is>
       </c>
       <c r="M38" t="n">
-        <v>38477</v>
+        <v>42990</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -12271,7 +12277,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-08-20T09:03:00</t>
+          <t>2026-08-28T09:03:17</t>
         </is>
       </c>
     </row>
@@ -12450,7 +12456,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>5180757</v>
+        <v>5762940</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12463,7 +12469,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>2358996</v>
+        <v>2435995</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -12472,7 +12478,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-08-20T09:03:09</t>
+          <t>2026-08-28T09:03:26</t>
         </is>
       </c>
     </row>
@@ -12718,7 +12724,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>50588</v>
+        <v>54311</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -12731,7 +12737,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>50588</v>
+        <v>54311</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -12740,7 +12746,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-08-20T09:03:19</t>
+          <t>2026-08-28T09:03:36</t>
         </is>
       </c>
     </row>
@@ -13541,7 +13547,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>81211</v>
+        <v>86057</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -13554,7 +13560,7 @@
         </is>
       </c>
       <c r="M58" t="n">
-        <v>10222</v>
+        <v>10801</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -13563,7 +13569,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-08-20T09:03:33</t>
+          <t>2026-08-28T09:03:51</t>
         </is>
       </c>
     </row>
@@ -14163,7 +14169,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>729261</v>
+        <v>770184</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -14176,7 +14182,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>256666</v>
+        <v>295552</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -14185,7 +14191,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-08-20T09:03:42</t>
+          <t>2026-08-28T09:03:59</t>
         </is>
       </c>
     </row>
@@ -14541,7 +14547,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1035165</v>
+        <v>1061983</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -14554,7 +14560,7 @@
         </is>
       </c>
       <c r="M74" t="n">
-        <v>163780</v>
+        <v>173395</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -14563,7 +14569,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-08-20T09:03:53</t>
+          <t>2026-08-28T09:04:11</t>
         </is>
       </c>
     </row>
@@ -14608,7 +14614,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>321620</v>
+        <v>359445</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -14620,7 +14626,7 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-08-20T09:04:04</t>
+          <t>2026-08-28T09:04:22</t>
         </is>
       </c>
     </row>
@@ -14665,7 +14671,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>2842301</v>
+        <v>2963835</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -14677,7 +14683,7 @@
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-08-20T09:04:31</t>
+          <t>2026-08-28T09:04:50</t>
         </is>
       </c>
     </row>
@@ -15090,7 +15096,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>12477</v>
+        <v>13539</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -15103,7 +15109,7 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>12477</v>
+        <v>13539</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -15112,7 +15118,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-08-20T09:04:44</t>
+          <t>2026-08-28T09:05:03</t>
         </is>
       </c>
     </row>
@@ -15291,7 +15297,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>9349156</v>
+        <v>9393174</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -15304,7 +15310,7 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>231035</v>
+        <v>239455</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -15313,7 +15319,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-08-20T09:04:53</t>
+          <t>2026-08-28T09:05:13</t>
         </is>
       </c>
     </row>
@@ -15358,7 +15364,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>231035</v>
+        <v>239455</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -15371,7 +15377,7 @@
         </is>
       </c>
       <c r="M87" t="n">
-        <v>231035</v>
+        <v>239455</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -15380,7 +15386,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-08-20T09:05:02</t>
+          <t>2026-08-28T09:05:22</t>
         </is>
       </c>
     </row>
@@ -15425,7 +15431,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>30472</v>
+        <v>36229</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -15438,7 +15444,7 @@
         </is>
       </c>
       <c r="M88" t="n">
-        <v>30472</v>
+        <v>36229</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -15447,7 +15453,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-08-20T09:05:11</t>
+          <t>2026-08-28T09:05:32</t>
         </is>
       </c>
     </row>
@@ -15492,7 +15498,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>160376</v>
+        <v>184894</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -15505,7 +15511,7 @@
         </is>
       </c>
       <c r="M89" t="n">
-        <v>28323</v>
+        <v>36754</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -15514,7 +15520,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-08-20T09:05:20</t>
+          <t>2026-08-28T09:05:42</t>
         </is>
       </c>
     </row>
@@ -15602,7 +15608,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>8166016</v>
+        <v>8449820</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -15615,7 +15621,7 @@
         </is>
       </c>
       <c r="M91" t="n">
-        <v>781885</v>
+        <v>857033</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -15624,7 +15630,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-08-20T09:05:38</t>
+          <t>2026-08-28T09:06:00</t>
         </is>
       </c>
     </row>
@@ -15913,7 +15919,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>77810</v>
+        <v>89363</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -15926,7 +15932,7 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>21062</v>
+        <v>24518</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -15935,7 +15941,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-08-20T09:05:50</t>
+          <t>2026-08-28T09:06:12</t>
         </is>
       </c>
     </row>
@@ -16468,7 +16474,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1641632</v>
+        <v>1646909</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -16481,7 +16487,7 @@
         </is>
       </c>
       <c r="M105" t="n">
-        <v>475308</v>
+        <v>478873</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -16490,7 +16496,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-08-20T09:06:09</t>
+          <t>2026-08-28T09:06:31</t>
         </is>
       </c>
     </row>
@@ -16535,7 +16541,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>1641632</v>
+        <v>1646909</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -16548,7 +16554,7 @@
         </is>
       </c>
       <c r="M106" t="n">
-        <v>475308</v>
+        <v>478873</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -16557,7 +16563,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-08-20T09:06:18</t>
+          <t>2026-08-28T09:06:40</t>
         </is>
       </c>
     </row>
@@ -16602,7 +16608,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>4640</v>
+        <v>4988</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -16615,7 +16621,7 @@
         </is>
       </c>
       <c r="M107" t="n">
-        <v>4640</v>
+        <v>4988</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -16624,7 +16630,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-08-21T09:01:01</t>
+          <t>2026-08-28T09:06:44</t>
         </is>
       </c>
     </row>
@@ -16669,7 +16675,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>827930</v>
+        <v>915300</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -16678,11 +16684,11 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Ech7Tj8ga0Y</t>
+          <t>https://www.youtube.com/watch?v=9TTfyS5r3Ps</t>
         </is>
       </c>
       <c r="M108" t="n">
-        <v>697155</v>
+        <v>190396</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -16691,7 +16697,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-08-20T09:06:30</t>
+          <t>2026-08-28T09:06:53</t>
         </is>
       </c>
     </row>
@@ -16736,7 +16742,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>824253</v>
+        <v>841936</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -16749,7 +16755,7 @@
         </is>
       </c>
       <c r="M109" t="n">
-        <v>148614</v>
+        <v>155447</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -16758,7 +16764,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-08-20T09:06:39</t>
+          <t>2026-08-28T09:07:02</t>
         </is>
       </c>
     </row>
@@ -16870,7 +16876,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>156926</v>
+        <v>194143</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -16883,7 +16889,7 @@
         </is>
       </c>
       <c r="M111" t="n">
-        <v>32190</v>
+        <v>35735</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -16892,7 +16898,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-08-20T09:06:48</t>
+          <t>2026-08-28T09:07:12</t>
         </is>
       </c>
     </row>
@@ -17138,7 +17144,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>858366</v>
+        <v>868047</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -17151,7 +17157,7 @@
         </is>
       </c>
       <c r="M115" t="n">
-        <v>250743</v>
+        <v>293160</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -17160,7 +17166,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-08-20T09:06:58</t>
+          <t>2026-08-28T09:07:21</t>
         </is>
       </c>
     </row>
@@ -17268,11 +17274,11 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=PWN4MO0ILIM</t>
+          <t>https://www.youtube.com/watch?v=PCpMF_19VQk</t>
         </is>
       </c>
       <c r="J117" t="n">
-        <v>268845</v>
+        <v>72104</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -17285,7 +17291,7 @@
         </is>
       </c>
       <c r="M117" t="n">
-        <v>35862</v>
+        <v>38416</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
@@ -17294,7 +17300,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-08-20T09:07:07</t>
+          <t>2026-08-28T09:07:31</t>
         </is>
       </c>
     </row>
@@ -17846,7 +17852,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>21733</v>
+        <v>22179</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -17858,7 +17864,7 @@
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-08-20T09:07:36</t>
+          <t>2026-08-28T09:08:01</t>
         </is>
       </c>
     </row>
@@ -18281,7 +18287,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>36509</v>
+        <v>41429</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -18294,7 +18300,7 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>25232</v>
+        <v>27445</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -18303,7 +18309,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-08-20T09:07:50</t>
+          <t>2026-08-28T09:08:16</t>
         </is>
       </c>
     </row>
@@ -18592,7 +18598,7 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>4492</v>
+        <v>5137</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -18605,7 +18611,7 @@
         </is>
       </c>
       <c r="M139" t="n">
-        <v>4492</v>
+        <v>5137</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
@@ -18614,7 +18620,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-08-20T09:08:02</t>
+          <t>2026-08-28T09:08:28</t>
         </is>
       </c>
     </row>
@@ -18840,7 +18846,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>589919</v>
+        <v>647165</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -18853,7 +18859,7 @@
         </is>
       </c>
       <c r="M143" t="n">
-        <v>589919</v>
+        <v>647165</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -18862,7 +18868,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-08-20T09:08:11</t>
+          <t>2026-08-28T09:08:37</t>
         </is>
       </c>
     </row>
@@ -18907,7 +18913,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>11933492</v>
+        <v>12058152</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -18920,7 +18926,7 @@
         </is>
       </c>
       <c r="M144" t="n">
-        <v>166076</v>
+        <v>192521</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -18929,7 +18935,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-08-20T09:08:20</t>
+          <t>2026-08-28T09:08:46</t>
         </is>
       </c>
     </row>
@@ -19299,7 +19305,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>120629</v>
+        <v>135689</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -19311,7 +19317,7 @@
       <c r="N150" t="inlineStr"/>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-08-20T09:08:42</t>
+          <t>2026-08-28T09:09:09</t>
         </is>
       </c>
     </row>
@@ -19686,7 +19692,7 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>194288</v>
+        <v>210414</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -19699,7 +19705,7 @@
         </is>
       </c>
       <c r="M157" t="n">
-        <v>194288</v>
+        <v>210414</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -19708,7 +19714,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-08-20T09:08:55</t>
+          <t>2026-08-28T09:09:21</t>
         </is>
       </c>
     </row>
@@ -19887,7 +19893,7 @@
         </is>
       </c>
       <c r="J160" t="n">
-        <v>20775</v>
+        <v>23393</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -19900,7 +19906,7 @@
         </is>
       </c>
       <c r="M160" t="n">
-        <v>20775</v>
+        <v>23393</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -19909,7 +19915,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-08-20T09:09:04</t>
+          <t>2026-08-28T09:09:30</t>
         </is>
       </c>
     </row>
@@ -20021,7 +20027,7 @@
         </is>
       </c>
       <c r="J162" t="n">
-        <v>301272</v>
+        <v>301718</v>
       </c>
       <c r="K162" t="inlineStr">
         <is>
@@ -20034,7 +20040,7 @@
         </is>
       </c>
       <c r="M162" t="n">
-        <v>301272</v>
+        <v>301718</v>
       </c>
       <c r="N162" t="inlineStr">
         <is>
@@ -20043,7 +20049,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-08-20T09:09:13</t>
+          <t>2026-08-28T09:09:40</t>
         </is>
       </c>
     </row>
@@ -20125,7 +20131,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>FX戦士くるみちゃん</t>
+          <t>アオのハコ Season2</t>
         </is>
       </c>
       <c r="D164" t="b">
@@ -20133,7 +20139,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -20141,21 +20147,45 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>$・¥・€ （ドル・エン・ユーロ）</t>
+          <t>あなたの花の色</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>福賀くるみ（CV：鈴木愛奈）</t>
-        </is>
-      </c>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
-      <c r="M164" t="inlineStr"/>
-      <c r="N164" t="inlineStr"/>
-      <c r="O164" t="inlineStr"/>
+          <t>aiko</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=d0jg9hNHqn8</t>
+        </is>
+      </c>
+      <c r="J164" t="n">
+        <v>10086016</v>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=d0jg9hNHqn8</t>
+        </is>
+      </c>
+      <c r="M164" t="n">
+        <v>10086016</v>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:09:49</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -20168,7 +20198,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
+          <t>アオのハコ Season2</t>
         </is>
       </c>
       <c r="D165" t="b">
@@ -20176,7 +20206,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -20184,45 +20214,21 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Escape</t>
+          <t>blue in</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Kis-My-Ft2</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
-        </is>
-      </c>
-      <c r="J165" t="n">
-        <v>66884</v>
-      </c>
-      <c r="K165" t="inlineStr">
-        <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
-        </is>
-      </c>
-      <c r="L165" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
-        </is>
-      </c>
-      <c r="M165" t="n">
-        <v>623677</v>
-      </c>
-      <c r="N165" t="inlineStr">
-        <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
-        </is>
-      </c>
-      <c r="O165" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:16:30</t>
-        </is>
-      </c>
+          <t>エルスウェア紀行</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr"/>
+      <c r="M165" t="inlineStr"/>
+      <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -20235,7 +20241,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="D166" t="b">
@@ -20243,7 +20249,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -20251,12 +20257,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>$・¥・€ （ドル・エン・ユーロ）</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>THE RAMPAGE</t>
+          <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -20278,7 +20284,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="D167" t="b">
@@ -20286,7 +20292,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -20294,21 +20300,45 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>Escape</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr"/>
-      <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
-      <c r="M167" t="inlineStr"/>
-      <c r="N167" t="inlineStr"/>
-      <c r="O167" t="inlineStr"/>
+          <t>Kis-My-Ft2</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+        </is>
+      </c>
+      <c r="J167" t="n">
+        <v>66884</v>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
+        </is>
+      </c>
+      <c r="M167" t="n">
+        <v>623677</v>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:16:30</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -20321,7 +20351,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D168" t="b">
@@ -20329,7 +20359,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -20337,12 +20367,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>krage</t>
+          <t>THE RAMPAGE</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -20364,7 +20394,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D169" t="b">
@@ -20380,12 +20410,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>リスポーン!!</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>角巻わため</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -20407,7 +20437,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D170" t="b">
@@ -20415,7 +20445,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -20423,45 +20453,21 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>雲を抜け風下へ私だけ</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>ヨルシカ</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
-        </is>
-      </c>
-      <c r="J170" t="n">
-        <v>1545312</v>
-      </c>
-      <c r="K170" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="L170" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
-        </is>
-      </c>
-      <c r="M170" t="n">
-        <v>7582011</v>
-      </c>
-      <c r="N170" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="O170" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:08:32</t>
-        </is>
-      </c>
+          <t>krage</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -20474,7 +20480,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="D171" t="b">
@@ -20490,45 +20496,21 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>リスポーン!!</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>amazarashi</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="J171" t="n">
-        <v>187718</v>
-      </c>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="L171" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="M171" t="n">
-        <v>187718</v>
-      </c>
-      <c r="N171" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="O171" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:17:05</t>
-        </is>
-      </c>
+          <t>角巻わため</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -20541,7 +20523,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>ごーすと・みーつ・ぎゃる！</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="D172" t="b">
@@ -20549,7 +20531,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20557,21 +20539,45 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>にこいちミライ</t>
+          <t>雲を抜け風下へ私だけ</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr"/>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr"/>
+          <t>ヨルシカ</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>1545312</v>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
+        </is>
+      </c>
+      <c r="M172" t="n">
+        <v>7582011</v>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:08:32</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -20584,7 +20590,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -20600,21 +20606,45 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr"/>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
-      <c r="M173" t="inlineStr"/>
-      <c r="N173" t="inlineStr"/>
-      <c r="O173" t="inlineStr"/>
+          <t>amazarashi</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="J173" t="n">
+        <v>187718</v>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="M173" t="n">
+        <v>187718</v>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:17:05</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -20627,7 +20657,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -20635,7 +20665,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -20643,12 +20673,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -20670,7 +20700,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -20678,7 +20708,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -20686,35 +20716,21 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
-        </is>
-      </c>
-      <c r="J175" t="n">
-        <v>164875</v>
-      </c>
-      <c r="K175" t="inlineStr">
-        <is>
-          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
-        </is>
-      </c>
+          <t>西川貴教</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr"/>
-      <c r="O175" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:17:30</t>
-        </is>
-      </c>
+      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -20727,7 +20743,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -20743,12 +20759,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>風の中は走るっきゃないっ！</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>三月のパンタシア</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -20770,7 +20786,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>DARK MACHINE THE ANIMATION</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -20778,7 +20794,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -20786,21 +20802,35 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>存在理由 改</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>BUCK∞TICK</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v>164875</v>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:17:30</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -20813,7 +20843,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -20829,12 +20859,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>風の中は走るっきゃないっ！</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>三月のパンタシア</t>
         </is>
       </c>
       <c r="I178" t="inlineStr"/>
@@ -20856,7 +20886,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -20864,7 +20894,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -20872,12 +20902,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -20899,7 +20929,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -20915,12 +20945,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -20942,7 +20972,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -20958,12 +20988,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>SUPER★DRAGON</t>
         </is>
       </c>
       <c r="I181" t="inlineStr"/>
@@ -20985,7 +21015,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -21001,12 +21031,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>この心臓に花束を</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>心梅</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -21028,7 +21058,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -21044,35 +21074,21 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>白昼夢</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>カグラナナ</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
-        </is>
-      </c>
-      <c r="J183" t="n">
-        <v>2557872</v>
-      </c>
-      <c r="K183" t="inlineStr">
-        <is>
-          <t>カグラナナchannel／ななかぐら</t>
-        </is>
-      </c>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr">
-        <is>
-          <t>2026-08-27T09:02:46</t>
-        </is>
-      </c>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -21085,7 +21101,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -21101,45 +21117,21 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>この心臓に花束を</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J184" t="n">
-        <v>711649</v>
-      </c>
-      <c r="K184" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M184" t="n">
-        <v>711649</v>
-      </c>
-      <c r="N184" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O184" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:17:54</t>
-        </is>
-      </c>
+          <t>心梅</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -21152,7 +21144,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -21168,43 +21160,33 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>白昼夢</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
+          <t>カグラナナ</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
         </is>
       </c>
       <c r="J185" t="n">
-        <v>397704</v>
+        <v>2557872</v>
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L185" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M185" t="n">
-        <v>397704</v>
-      </c>
-      <c r="N185" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>カグラナナchannel／ななかぐら</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-08-24T09:18:04</t>
+          <t>2026-08-27T09:02:46</t>
         </is>
       </c>
     </row>
@@ -21219,7 +21201,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -21227,7 +21209,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -21235,21 +21217,45 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr"/>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr"/>
-      <c r="M186" t="inlineStr"/>
-      <c r="N186" t="inlineStr"/>
-      <c r="O186" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J186" t="n">
+        <v>711649</v>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M186" t="n">
+        <v>711649</v>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:17:54</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -21262,7 +21268,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D187" t="b">
@@ -21270,7 +21276,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -21278,21 +21284,45 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Re:name</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr"/>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
-      <c r="M187" t="inlineStr"/>
-      <c r="N187" t="inlineStr"/>
-      <c r="O187" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J187" t="n">
+        <v>397704</v>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M187" t="n">
+        <v>397704</v>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:18:04</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -21305,7 +21335,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D188" t="b">
@@ -21321,12 +21351,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Ray of Emotion</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>導凰</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I188" t="inlineStr"/>
@@ -21348,7 +21378,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D189" t="b">
@@ -21364,12 +21394,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>Ado</t>
+          <t>Re:name</t>
         </is>
       </c>
       <c r="I189" t="inlineStr"/>
@@ -21391,7 +21421,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D190" t="b">
@@ -21399,7 +21429,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -21407,35 +21437,21 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>あやかしあやし</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
-        </is>
-      </c>
-      <c r="J190" t="n">
-        <v>48992</v>
-      </c>
-      <c r="K190" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+          <t>導凰</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr"/>
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr"/>
-      <c r="O190" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:10:14</t>
-        </is>
-      </c>
+      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -21448,7 +21464,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D191" t="b">
@@ -21456,7 +21472,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -21464,45 +21480,21 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>朔日 feat. 吉乃</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>月詠み</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="J191" t="n">
-        <v>46450</v>
-      </c>
-      <c r="K191" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="M191" t="n">
-        <v>46450</v>
-      </c>
-      <c r="N191" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="O191" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:10:21</t>
-        </is>
-      </c>
+          <t>Ado</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
+      <c r="N191" t="inlineStr"/>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -21515,7 +21507,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D192" t="b">
@@ -21531,21 +21523,35 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+        </is>
+      </c>
+      <c r="J192" t="n">
+        <v>48992</v>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
       <c r="L192" t="inlineStr"/>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr"/>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:10:14</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -21558,7 +21564,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -21574,21 +21580,45 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
-      <c r="N193" t="inlineStr"/>
-      <c r="O193" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J193" t="n">
+        <v>46450</v>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M193" t="n">
+        <v>46450</v>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:10:21</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -21601,7 +21631,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D194" t="b">
@@ -21617,12 +21647,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>FZMZ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I194" t="inlineStr"/>
@@ -21644,7 +21674,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D195" t="b">
@@ -21660,12 +21690,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I195" t="inlineStr"/>
@@ -21687,7 +21717,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D196" t="b">
@@ -21703,12 +21733,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I196" t="inlineStr"/>
@@ -21730,7 +21760,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D197" t="b">
@@ -21746,12 +21776,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I197" t="inlineStr"/>
@@ -21773,7 +21803,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D198" t="b">
@@ -21789,12 +21819,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>JO1</t>
+          <t>East Of Eden</t>
         </is>
       </c>
       <c r="I198" t="inlineStr"/>
@@ -21816,7 +21846,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D199" t="b">
@@ -21832,45 +21862,21 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
-        </is>
-      </c>
-      <c r="J199" t="n">
-        <v>17851</v>
-      </c>
-      <c r="K199" t="inlineStr">
-        <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L199" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M199" t="n">
-        <v>3801597</v>
-      </c>
-      <c r="N199" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
-      <c r="O199" t="inlineStr">
-        <is>
-          <t>2026-08-21T09:03:35</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
+      <c r="L199" t="inlineStr"/>
+      <c r="M199" t="inlineStr"/>
+      <c r="N199" t="inlineStr"/>
+      <c r="O199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -21883,7 +21889,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D200" t="b">
@@ -21891,7 +21897,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -21899,21 +21905,35 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
-        </is>
-      </c>
-      <c r="I200" t="inlineStr"/>
-      <c r="J200" t="inlineStr"/>
-      <c r="K200" t="inlineStr"/>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
+        </is>
+      </c>
+      <c r="J200" t="n">
+        <v>75253</v>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
       <c r="L200" t="inlineStr"/>
       <c r="M200" t="inlineStr"/>
       <c r="N200" t="inlineStr"/>
-      <c r="O200" t="inlineStr"/>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:38</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -21926,7 +21946,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D201" t="b">
@@ -21934,7 +21954,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -21942,21 +21962,45 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
-      <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr"/>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr"/>
-      <c r="M201" t="inlineStr"/>
-      <c r="N201" t="inlineStr"/>
-      <c r="O201" t="inlineStr"/>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J201" t="n">
+        <v>92436</v>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M201" t="n">
+        <v>3815771</v>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:50</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -21969,7 +22013,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D202" t="b">
@@ -21977,7 +22021,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -21985,12 +22029,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Diamond Dust</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Sizuk</t>
+          <t>東京スカパラダイスオーケストラ</t>
         </is>
       </c>
       <c r="I202" t="inlineStr"/>
@@ -22012,7 +22056,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D203" t="b">
@@ -22020,7 +22064,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F203" t="n">
@@ -22028,12 +22072,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>COMPRESSION :[</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>内田真礼</t>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
       <c r="I203" t="inlineStr"/>
@@ -22055,7 +22099,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D204" t="b">
@@ -22071,45 +22115,21 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J204" t="n">
-        <v>4470</v>
-      </c>
-      <c r="K204" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L204" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M204" t="n">
-        <v>4470</v>
-      </c>
-      <c r="N204" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O204" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:19:40</t>
-        </is>
-      </c>
+          <t>Sizuk</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr"/>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="inlineStr"/>
+      <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -22122,7 +22142,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D205" t="b">
@@ -22138,35 +22158,21 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I205" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J205" t="n">
-        <v>757285</v>
-      </c>
-      <c r="K205" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>内田真礼</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr"/>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr"/>
       <c r="L205" t="inlineStr"/>
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr"/>
-      <c r="O205" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:19:55</t>
-        </is>
-      </c>
+      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -22179,7 +22185,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D206" t="b">
@@ -22195,33 +22201,43 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J206" t="n">
-        <v>107820</v>
+        <v>4470</v>
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L206" t="inlineStr"/>
-      <c r="M206" t="inlineStr"/>
-      <c r="N206" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M206" t="n">
+        <v>4470</v>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-08-24T09:20:11</t>
+          <t>2026-08-24T09:19:40</t>
         </is>
       </c>
     </row>
@@ -22236,7 +22252,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D207" t="b">
@@ -22252,25 +22268,25 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>ReMind</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>Daisy×Daisy</t>
+          <t>TOOBOE</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
         </is>
       </c>
       <c r="J207" t="n">
-        <v>77536</v>
+        <v>757285</v>
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+          <t>john / TOOBOE</t>
         </is>
       </c>
       <c r="L207" t="inlineStr"/>
@@ -22278,7 +22294,7 @@
       <c r="N207" t="inlineStr"/>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-08-27T09:04:35</t>
+          <t>2026-08-24T09:19:55</t>
         </is>
       </c>
     </row>
@@ -22293,7 +22309,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D208" t="b">
@@ -22309,43 +22325,33 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J208" t="n">
-        <v>307069</v>
+        <v>107820</v>
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L208" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M208" t="n">
-        <v>307069</v>
-      </c>
-      <c r="N208" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr"/>
+      <c r="M208" t="inlineStr"/>
+      <c r="N208" t="inlineStr"/>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-08-20T09:12:04</t>
+          <t>2026-08-24T09:20:11</t>
         </is>
       </c>
     </row>
@@ -22360,7 +22366,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D209" t="b">
@@ -22376,43 +22382,33 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>ReMind</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>Daisy×Daisy</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
         </is>
       </c>
       <c r="J209" t="n">
-        <v>307070</v>
+        <v>77536</v>
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M209" t="n">
-        <v>307070</v>
-      </c>
-      <c r="N209" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr"/>
+      <c r="N209" t="inlineStr"/>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-08-20T09:12:14</t>
+          <t>2026-08-27T09:04:35</t>
         </is>
       </c>
     </row>
@@ -22427,7 +22423,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D210" t="b">
@@ -22443,21 +22439,45 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I210" t="inlineStr"/>
-      <c r="J210" t="inlineStr"/>
-      <c r="K210" t="inlineStr"/>
-      <c r="L210" t="inlineStr"/>
-      <c r="M210" t="inlineStr"/>
-      <c r="N210" t="inlineStr"/>
-      <c r="O210" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J210" t="n">
+        <v>309603</v>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M210" t="n">
+        <v>309603</v>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:31</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -22470,7 +22490,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D211" t="b">
@@ -22486,21 +22506,45 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I211" t="inlineStr"/>
-      <c r="J211" t="inlineStr"/>
-      <c r="K211" t="inlineStr"/>
-      <c r="L211" t="inlineStr"/>
-      <c r="M211" t="inlineStr"/>
-      <c r="N211" t="inlineStr"/>
-      <c r="O211" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J211" t="n">
+        <v>309598</v>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M211" t="n">
+        <v>309598</v>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:41</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -22513,7 +22557,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D212" t="b">
@@ -22529,12 +22573,12 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I212" t="inlineStr"/>
@@ -22556,7 +22600,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D213" t="b">
@@ -22564,7 +22608,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -22572,45 +22616,21 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J213" t="n">
-        <v>973031</v>
-      </c>
-      <c r="K213" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L213" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M213" t="n">
-        <v>401379</v>
-      </c>
-      <c r="N213" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O213" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:20:37</t>
-        </is>
-      </c>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr"/>
+      <c r="K213" t="inlineStr"/>
+      <c r="L213" t="inlineStr"/>
+      <c r="M213" t="inlineStr"/>
+      <c r="N213" t="inlineStr"/>
+      <c r="O213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -22623,7 +22643,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="D214" t="b">
@@ -22631,7 +22651,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -22639,41 +22659,151 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr"/>
+      <c r="K214" t="inlineStr"/>
+      <c r="L214" t="inlineStr"/>
+      <c r="M214" t="inlineStr"/>
+      <c r="N214" t="inlineStr"/>
+      <c r="O214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D215" t="b">
+        <v>0</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>1</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J215" t="n">
+        <v>973031</v>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M215" t="n">
+        <v>401379</v>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:20:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D216" t="b">
+        <v>0</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>1</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr">
+      <c r="H216" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I214" t="inlineStr">
+      <c r="I216" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
-      <c r="J214" t="n">
+      <c r="J216" t="n">
         <v>434141</v>
       </c>
-      <c r="K214" t="inlineStr">
+      <c r="K216" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="L214" t="inlineStr">
+      <c r="L216" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M214" t="n">
+      <c r="M216" t="n">
         <v>409527</v>
       </c>
-      <c r="N214" t="inlineStr">
+      <c r="N216" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O214" t="inlineStr">
+      <c r="O216" t="inlineStr">
         <is>
           <t>2026-08-24T09:20:46</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-08-31
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -6753,7 +6753,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月5日（月）～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -7145,10 +7145,26 @@
           <t>ブリッジ</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>影響力∞アイドル</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>星を巡る</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>ロクデナシ</t>
+        </is>
+      </c>
       <c r="M124" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
@@ -9930,7 +9946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O216"/>
+  <dimension ref="A1:O218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10094,7 +10110,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>13111</v>
+        <v>15429</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10107,7 +10123,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>13111</v>
+        <v>15429</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -10116,7 +10132,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-08-21T09:00:15</t>
+          <t>2026-08-31T09:00:18</t>
         </is>
       </c>
     </row>
@@ -20886,7 +20902,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>DARK MACHINE THE ANIMATION</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -20902,12 +20918,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>存在理由 改</t>
+          <t>影響力∞アイドル</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>BUCK∞TICK</t>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -20929,7 +20945,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -20937,7 +20953,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -20945,12 +20961,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>星を巡る</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>ロクデナシ</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -20972,7 +20988,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -20980,7 +20996,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -20988,12 +21004,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I181" t="inlineStr"/>
@@ -21015,7 +21031,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -21031,12 +21047,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -21058,7 +21074,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -21074,12 +21090,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>SUPER★DRAGON</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -21101,7 +21117,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D184" t="b">
@@ -21117,12 +21133,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>この心臓に花束を</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>心梅</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
@@ -21144,7 +21160,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D185" t="b">
@@ -21160,35 +21176,21 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>白昼夢</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>カグラナナ</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
-        </is>
-      </c>
-      <c r="J185" t="n">
-        <v>2557872</v>
-      </c>
-      <c r="K185" t="inlineStr">
-        <is>
-          <t>カグラナナchannel／ななかぐら</t>
-        </is>
-      </c>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr"/>
       <c r="N185" t="inlineStr"/>
-      <c r="O185" t="inlineStr">
-        <is>
-          <t>2026-08-27T09:02:46</t>
-        </is>
-      </c>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -21201,7 +21203,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D186" t="b">
@@ -21217,45 +21219,21 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>この心臓に花束を</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J186" t="n">
-        <v>711649</v>
-      </c>
-      <c r="K186" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L186" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M186" t="n">
-        <v>711649</v>
-      </c>
-      <c r="N186" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O186" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:17:54</t>
-        </is>
-      </c>
+          <t>心梅</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -21268,7 +21246,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D187" t="b">
@@ -21284,43 +21262,33 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>白昼夢</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
+          <t>カグラナナ</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
         </is>
       </c>
       <c r="J187" t="n">
-        <v>397704</v>
+        <v>2557872</v>
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L187" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M187" t="n">
-        <v>397704</v>
-      </c>
-      <c r="N187" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>カグラナナchannel／ななかぐら</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="inlineStr"/>
+      <c r="N187" t="inlineStr"/>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-08-24T09:18:04</t>
+          <t>2026-08-27T09:02:46</t>
         </is>
       </c>
     </row>
@@ -21335,7 +21303,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D188" t="b">
@@ -21343,7 +21311,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -21351,21 +21319,45 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr"/>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
-      <c r="M188" t="inlineStr"/>
-      <c r="N188" t="inlineStr"/>
-      <c r="O188" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J188" t="n">
+        <v>711649</v>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M188" t="n">
+        <v>711649</v>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:17:54</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -21378,7 +21370,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D189" t="b">
@@ -21386,7 +21378,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -21394,21 +21386,45 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>Re:name</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr"/>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
-      <c r="O189" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J189" t="n">
+        <v>397704</v>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M189" t="n">
+        <v>397704</v>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:18:04</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -21421,7 +21437,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D190" t="b">
@@ -21437,12 +21453,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Ray of Emotion</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>導凰</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I190" t="inlineStr"/>
@@ -21464,7 +21480,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D191" t="b">
@@ -21480,12 +21496,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Ado</t>
+          <t>Re:name</t>
         </is>
       </c>
       <c r="I191" t="inlineStr"/>
@@ -21507,7 +21523,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D192" t="b">
@@ -21515,7 +21531,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -21523,35 +21539,21 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>あやかしあやし</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
-        </is>
-      </c>
-      <c r="J192" t="n">
-        <v>48992</v>
-      </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+          <t>導凰</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr"/>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:10:14</t>
-        </is>
-      </c>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -21564,7 +21566,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D193" t="b">
@@ -21572,7 +21574,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -21580,45 +21582,21 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>朔日 feat. 吉乃</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>月詠み</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="J193" t="n">
-        <v>46450</v>
-      </c>
-      <c r="K193" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="L193" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="M193" t="n">
-        <v>46450</v>
-      </c>
-      <c r="N193" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="O193" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:10:21</t>
-        </is>
-      </c>
+          <t>Ado</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="inlineStr"/>
+      <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -21631,7 +21609,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D194" t="b">
@@ -21647,21 +21625,35 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+        </is>
+      </c>
+      <c r="J194" t="n">
+        <v>48992</v>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
       <c r="L194" t="inlineStr"/>
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr"/>
-      <c r="O194" t="inlineStr"/>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:10:14</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -21674,7 +21666,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D195" t="b">
@@ -21690,21 +21682,45 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr"/>
-      <c r="M195" t="inlineStr"/>
-      <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J195" t="n">
+        <v>46450</v>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M195" t="n">
+        <v>46450</v>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:10:21</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -21717,7 +21733,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D196" t="b">
@@ -21733,12 +21749,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>FZMZ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I196" t="inlineStr"/>
@@ -21760,7 +21776,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D197" t="b">
@@ -21776,12 +21792,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I197" t="inlineStr"/>
@@ -21803,7 +21819,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D198" t="b">
@@ -21819,12 +21835,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I198" t="inlineStr"/>
@@ -21846,7 +21862,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D199" t="b">
@@ -21862,12 +21878,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I199" t="inlineStr"/>
@@ -21889,7 +21905,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D200" t="b">
@@ -21905,35 +21921,21 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
-        </is>
-      </c>
-      <c r="J200" t="n">
-        <v>75253</v>
-      </c>
-      <c r="K200" t="inlineStr">
-        <is>
-          <t>JO1</t>
-        </is>
-      </c>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr"/>
       <c r="L200" t="inlineStr"/>
       <c r="M200" t="inlineStr"/>
       <c r="N200" t="inlineStr"/>
-      <c r="O200" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:38</t>
-        </is>
-      </c>
+      <c r="O200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -21946,7 +21948,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D201" t="b">
@@ -21962,45 +21964,21 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
-        </is>
-      </c>
-      <c r="J201" t="n">
-        <v>92436</v>
-      </c>
-      <c r="K201" t="inlineStr">
-        <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L201" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M201" t="n">
-        <v>3815771</v>
-      </c>
-      <c r="N201" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
-      <c r="O201" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:50</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="inlineStr"/>
+      <c r="M201" t="inlineStr"/>
+      <c r="N201" t="inlineStr"/>
+      <c r="O201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -22013,7 +21991,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D202" t="b">
@@ -22021,7 +21999,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -22029,21 +22007,35 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
-        </is>
-      </c>
-      <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
+        </is>
+      </c>
+      <c r="J202" t="n">
+        <v>75253</v>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
       <c r="L202" t="inlineStr"/>
       <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr"/>
-      <c r="O202" t="inlineStr"/>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:38</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -22056,7 +22048,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D203" t="b">
@@ -22064,7 +22056,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F203" t="n">
@@ -22072,21 +22064,45 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
-      <c r="I203" t="inlineStr"/>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr"/>
-      <c r="M203" t="inlineStr"/>
-      <c r="N203" t="inlineStr"/>
-      <c r="O203" t="inlineStr"/>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J203" t="n">
+        <v>92436</v>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M203" t="n">
+        <v>3815771</v>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:50</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -22099,7 +22115,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D204" t="b">
@@ -22107,7 +22123,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F204" t="n">
@@ -22115,12 +22131,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Diamond Dust</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Sizuk</t>
+          <t>東京スカパラダイスオーケストラ</t>
         </is>
       </c>
       <c r="I204" t="inlineStr"/>
@@ -22142,7 +22158,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D205" t="b">
@@ -22150,7 +22166,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F205" t="n">
@@ -22158,12 +22174,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>COMPRESSION :[</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>内田真礼</t>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
       <c r="I205" t="inlineStr"/>
@@ -22185,7 +22201,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D206" t="b">
@@ -22201,45 +22217,21 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J206" t="n">
-        <v>4470</v>
-      </c>
-      <c r="K206" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L206" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M206" t="n">
-        <v>4470</v>
-      </c>
-      <c r="N206" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O206" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:19:40</t>
-        </is>
-      </c>
+          <t>Sizuk</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr"/>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr"/>
+      <c r="L206" t="inlineStr"/>
+      <c r="M206" t="inlineStr"/>
+      <c r="N206" t="inlineStr"/>
+      <c r="O206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -22252,7 +22244,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D207" t="b">
@@ -22268,35 +22260,21 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J207" t="n">
-        <v>757285</v>
-      </c>
-      <c r="K207" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>内田真礼</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr"/>
       <c r="L207" t="inlineStr"/>
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr"/>
-      <c r="O207" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:19:55</t>
-        </is>
-      </c>
+      <c r="O207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -22309,7 +22287,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D208" t="b">
@@ -22325,33 +22303,43 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J208" t="n">
-        <v>107820</v>
+        <v>4470</v>
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L208" t="inlineStr"/>
-      <c r="M208" t="inlineStr"/>
-      <c r="N208" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M208" t="n">
+        <v>4470</v>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-08-24T09:20:11</t>
+          <t>2026-08-24T09:19:40</t>
         </is>
       </c>
     </row>
@@ -22366,7 +22354,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D209" t="b">
@@ -22382,25 +22370,25 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>ReMind</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Daisy×Daisy</t>
+          <t>TOOBOE</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
         </is>
       </c>
       <c r="J209" t="n">
-        <v>77536</v>
+        <v>757285</v>
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+          <t>john / TOOBOE</t>
         </is>
       </c>
       <c r="L209" t="inlineStr"/>
@@ -22408,7 +22396,7 @@
       <c r="N209" t="inlineStr"/>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-08-27T09:04:35</t>
+          <t>2026-08-24T09:19:55</t>
         </is>
       </c>
     </row>
@@ -22423,7 +22411,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D210" t="b">
@@ -22439,43 +22427,33 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J210" t="n">
-        <v>309603</v>
+        <v>107820</v>
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M210" t="n">
-        <v>309603</v>
-      </c>
-      <c r="N210" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
+      <c r="M210" t="inlineStr"/>
+      <c r="N210" t="inlineStr"/>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-08-28T09:13:31</t>
+          <t>2026-08-24T09:20:11</t>
         </is>
       </c>
     </row>
@@ -22490,7 +22468,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D211" t="b">
@@ -22506,43 +22484,33 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>ReMind</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>Daisy×Daisy</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
         </is>
       </c>
       <c r="J211" t="n">
-        <v>309598</v>
+        <v>77536</v>
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L211" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M211" t="n">
-        <v>309598</v>
-      </c>
-      <c r="N211" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr"/>
+      <c r="M211" t="inlineStr"/>
+      <c r="N211" t="inlineStr"/>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-08-28T09:13:41</t>
+          <t>2026-08-27T09:04:35</t>
         </is>
       </c>
     </row>
@@ -22557,7 +22525,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D212" t="b">
@@ -22573,21 +22541,45 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr"/>
-      <c r="J212" t="inlineStr"/>
-      <c r="K212" t="inlineStr"/>
-      <c r="L212" t="inlineStr"/>
-      <c r="M212" t="inlineStr"/>
-      <c r="N212" t="inlineStr"/>
-      <c r="O212" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J212" t="n">
+        <v>309603</v>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M212" t="n">
+        <v>309603</v>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:31</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -22600,7 +22592,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D213" t="b">
@@ -22616,21 +22608,45 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr"/>
-      <c r="J213" t="inlineStr"/>
-      <c r="K213" t="inlineStr"/>
-      <c r="L213" t="inlineStr"/>
-      <c r="M213" t="inlineStr"/>
-      <c r="N213" t="inlineStr"/>
-      <c r="O213" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J213" t="n">
+        <v>309598</v>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M213" t="n">
+        <v>309598</v>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:41</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -22643,7 +22659,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D214" t="b">
@@ -22659,12 +22675,12 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I214" t="inlineStr"/>
@@ -22686,7 +22702,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D215" t="b">
@@ -22694,7 +22710,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F215" t="n">
@@ -22702,45 +22718,21 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I215" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J215" t="n">
-        <v>973031</v>
-      </c>
-      <c r="K215" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M215" t="n">
-        <v>401379</v>
-      </c>
-      <c r="N215" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O215" t="inlineStr">
-        <is>
-          <t>2026-08-24T09:20:37</t>
-        </is>
-      </c>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="inlineStr"/>
+      <c r="L215" t="inlineStr"/>
+      <c r="M215" t="inlineStr"/>
+      <c r="N215" t="inlineStr"/>
+      <c r="O215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -22753,7 +22745,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="D216" t="b">
@@ -22761,7 +22753,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F216" t="n">
@@ -22769,41 +22761,151 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr"/>
+      <c r="J216" t="inlineStr"/>
+      <c r="K216" t="inlineStr"/>
+      <c r="L216" t="inlineStr"/>
+      <c r="M216" t="inlineStr"/>
+      <c r="N216" t="inlineStr"/>
+      <c r="O216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D217" t="b">
+        <v>0</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>1</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J217" t="n">
+        <v>973031</v>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M217" t="n">
+        <v>401379</v>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>2026-08-24T09:20:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D218" t="b">
+        <v>0</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>1</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr">
+      <c r="H218" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I216" t="inlineStr">
+      <c r="I218" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
-      <c r="J216" t="n">
+      <c r="J218" t="n">
         <v>434141</v>
       </c>
-      <c r="K216" t="inlineStr">
+      <c r="K218" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="L216" t="inlineStr">
+      <c r="L218" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M216" t="n">
+      <c r="M218" t="n">
         <v>409527</v>
       </c>
-      <c r="N216" t="inlineStr">
+      <c r="N218" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O216" t="inlineStr">
+      <c r="O218" t="inlineStr">
         <is>
           <t>2026-08-24T09:20:46</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-02
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M133"/>
+  <dimension ref="A1:M134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +629,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月1日（木）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -637,8 +637,16 @@
           <t>パッショーネ</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>FX戦士くるみちゃん</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>福賀くるみ（CV：鈴木愛奈）</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>$・¥・€ （ドル・エン・ユーロ）</t>
@@ -4994,19 +5002,19 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>93</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>あかね噺 第2期</t>
+          <t>わたしの幸せな結婚 特別篇</t>
         </is>
       </c>
       <c r="E94" t="b">
@@ -5019,17 +5027,29 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2027年1月～ テレビ朝日系全国24局ネット“IMAnimation”枠・BS朝日ほか</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr"/>
+          <t>2026年10月25日（日）～ TOKYO MXほかにて</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>キネマシトラス</t>
+        </is>
+      </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>プレリュードの手前に ～for me&amp;you～</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28590</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25803</t>
         </is>
       </c>
     </row>
@@ -5043,11 +5063,11 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>アルカナディア</t>
+          <t>あかね噺 第2期</t>
         </is>
       </c>
       <c r="E95" t="b">
@@ -5060,21 +5080,17 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2027年1月〜 テレビ朝日系ほか</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>横浜アニメーションラボ</t>
-        </is>
-      </c>
+          <t>2027年1月～ テレビ朝日系全国24局ネット“IMAnimation”枠・BS朝日ほか</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28590</t>
         </is>
       </c>
     </row>
@@ -5088,11 +5104,11 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>異世界転生騒動記</t>
+          <t>アルカナディア</t>
         </is>
       </c>
       <c r="E96" t="b">
@@ -5105,17 +5121,21 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr"/>
+          <t>2027年1月〜 テレビ朝日系ほか</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>横浜アニメーションラボ</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27924</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25380</t>
         </is>
       </c>
     </row>
@@ -5129,11 +5149,11 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>一式さんは恋を知りたい。</t>
+          <t>異世界転生騒動記</t>
         </is>
       </c>
       <c r="E97" t="b">
@@ -5146,21 +5166,17 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>作楽クリエイト</t>
-        </is>
-      </c>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26981</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27924</t>
         </is>
       </c>
     </row>
@@ -5174,11 +5190,11 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>えぶりでいホスト 続編</t>
+          <t>一式さんは恋を知りたい。</t>
         </is>
       </c>
       <c r="E98" t="b">
@@ -5191,17 +5207,21 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr"/>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>作楽クリエイト</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27178</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26981</t>
         </is>
       </c>
     </row>
@@ -5215,11 +5235,11 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>欠けた月のメルセデス～吸血鬼の貴族に転生したけど捨てられそうなのでダンジョンを制覇する～</t>
+          <t>えぶりでいホスト 続編</t>
         </is>
       </c>
       <c r="E99" t="b">
@@ -5232,21 +5252,17 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>テディ―</t>
-        </is>
-      </c>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28808</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27178</t>
         </is>
       </c>
     </row>
@@ -5260,11 +5276,11 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>風を継ぐもの</t>
+          <t>欠けた月のメルセデス～吸血鬼の貴族に転生したけど捨てられそうなのでダンジョンを制覇する～</t>
         </is>
       </c>
       <c r="E100" t="b">
@@ -5277,12 +5293,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2027年1月～ CBC/TBS系全国28局ネットにて 【劇場先行上映】 2026年</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Live2D Creative Studio×</t>
+          <t>テディ―</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -5291,7 +5307,7 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26790</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28808</t>
         </is>
       </c>
     </row>
@@ -5305,11 +5321,11 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
+          <t>風を継ぐもの</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -5322,12 +5338,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ CBC/TBS系全国28局ネットにて 【劇場先行上映】 2026年</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>ゼロジー</t>
+          <t>Live2D Creative Studio×</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -5336,7 +5352,7 @@
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28643</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26790</t>
         </is>
       </c>
     </row>
@@ -5350,11 +5366,11 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>カリスマ</t>
+          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -5367,12 +5383,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2027年1月～ TBS系にて</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>PIERROT FILMS（</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -5381,7 +5397,7 @@
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27177</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28643</t>
         </is>
       </c>
     </row>
@@ -5395,11 +5411,11 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>傷口と包帯</t>
+          <t>カリスマ</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -5412,12 +5428,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2027年1月～ ABCテレビ・テレビ朝日系全国ネットANiMAZiNG!!!にて</t>
+          <t>2027年1月～ TBS系にて</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>PIERROT FILMS（</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -5426,7 +5442,7 @@
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28777</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27177</t>
         </is>
       </c>
     </row>
@@ -5440,11 +5456,11 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>気になってる人が男じゃなかった</t>
+          <t>傷口と包帯</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -5457,25 +5473,21 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>Breed</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
+          <t>2027年1月～ ABCテレビ・テレビ朝日系全国ネットANiMAZiNG!!!にて</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25569</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28777</t>
         </is>
       </c>
     </row>
@@ -5489,11 +5501,11 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>黒岩メダカに私の可愛いが通じない Season2</t>
+          <t>気になってる人が男じゃなかった</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -5509,18 +5521,22 @@
           <t>2027年1月～</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Breed</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28331</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25569</t>
         </is>
       </c>
     </row>
@@ -5534,11 +5550,11 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>ゲーム世界転生〈ダン活〉～ゲーマーは【ダンジョン就活のススメ】を〈はじめから〉プレイする～</t>
+          <t>黒岩メダカに私の可愛いが通じない Season2</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -5556,7 +5572,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>STUDIO MASSKET</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -5565,7 +5581,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27910</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28331</t>
         </is>
       </c>
     </row>
@@ -5579,11 +5595,11 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>結界師の一輪華</t>
+          <t>ゲーム世界転生〈ダン活〉～ゲーマーは【ダンジョン就活のススメ】を〈はじめから〉プレイする～</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -5601,7 +5617,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>TROYCA</t>
+          <t>STUDIO MASSKET</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -5610,7 +5626,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27910</t>
         </is>
       </c>
     </row>
@@ -5624,11 +5640,11 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>ゴールデンカムイ 最終章「暴走列車編」</t>
+          <t>結界師の一輪華</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -5641,17 +5657,21 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2027年冬</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr"/>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>TROYCA</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=21895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26630</t>
         </is>
       </c>
     </row>
@@ -5665,34 +5685,34 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>こまどり モフモフパレード</t>
+          <t>ゴールデンカムイ 最終章「暴走列車編」</t>
         </is>
       </c>
       <c r="E109" t="b">
         <v>0</v>
       </c>
-      <c r="F109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2027年1月～ テレ東系列6局ネットにて</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>ドワーフスタジオ</t>
-        </is>
-      </c>
+          <t>2027年冬</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27414</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=21895</t>
         </is>
       </c>
     </row>
@@ -5706,29 +5726,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>SAKAMOTO DAYS 第2期</t>
+          <t>こまどり モフモフパレード</t>
         </is>
       </c>
       <c r="E110" t="b">
         <v>0</v>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>TVアニメ</t>
-        </is>
-      </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ テレ東系列6局ネットにて</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>トムス・エンタテインメント</t>
+          <t>ドワーフスタジオ</t>
         </is>
       </c>
       <c r="I110" t="inlineStr"/>
@@ -5737,7 +5753,7 @@
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27287</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27414</t>
         </is>
       </c>
     </row>
@@ -5751,11 +5767,11 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>雑用付与術師が自分の最強に気付くまで</t>
+          <t>SAKAMOTO DAYS 第2期</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -5768,12 +5784,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2027年1月〜 TOKYO MX ほか</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>トムス・エンタテインメント</t>
         </is>
       </c>
       <c r="I111" t="inlineStr"/>
@@ -5782,7 +5798,7 @@
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27970</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27287</t>
         </is>
       </c>
     </row>
@@ -5796,11 +5812,11 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>THE ONE PIECE</t>
+          <t>雑用付与術師が自分の最強に気付くまで</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -5808,17 +5824,17 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2027年2月～ Netflixにて</t>
+          <t>2027年1月〜 TOKYO MX ほか</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>WIT STUDIO</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -5827,7 +5843,7 @@
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23247</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27970</t>
         </is>
       </c>
     </row>
@@ -5841,11 +5857,11 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>シャングリラ・フロンティア 3rd season</t>
+          <t>THE ONE PIECE</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -5853,17 +5869,17 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2027年1月〜 MBS／TBS系全国28局ネットほか</t>
+          <t>2027年2月～ Netflixにて</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>WIT STUDIO</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -5872,7 +5888,7 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25755</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23247</t>
         </is>
       </c>
     </row>
@@ -5886,11 +5902,11 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>じょせまる</t>
+          <t>シャングリラ・フロンティア 3rd season</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -5903,12 +5919,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
+          <t>2027年1月〜 MBS／TBS系全国28局ネットほか</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>株式会社フローエンタテイメント</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -5917,7 +5933,7 @@
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28562</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25755</t>
         </is>
       </c>
     </row>
@@ -5931,11 +5947,11 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>地雷なんですか？地原さん</t>
+          <t>じょせまる</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -5948,12 +5964,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2027年1月～ MBS・TBSほか</t>
+          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>SynergySP</t>
+          <t>株式会社フローエンタテイメント</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -5962,7 +5978,7 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27363</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28562</t>
         </is>
       </c>
     </row>
@@ -5976,11 +5992,11 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>すだちの魔王城</t>
+          <t>地雷なんですか？地原さん</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -5993,12 +6009,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ MBS・TBSほか</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>project No.9</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -6007,7 +6023,7 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28645</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27363</t>
         </is>
       </c>
     </row>
@@ -6021,11 +6037,11 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
+          <t>すだちの魔王城</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6038,12 +6054,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2027年1月～ AT-Xにて</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Acca effe×フロンティアエンジン</t>
+          <t>project No.9</t>
         </is>
       </c>
       <c r="I117" t="inlineStr"/>
@@ -6052,7 +6068,7 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23537</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28645</t>
         </is>
       </c>
     </row>
@@ -6066,11 +6082,11 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>ディズニー ツイステッドワンダーランド ザ アニメーション ～エピソード オブ サバナクロー～</t>
+          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6078,22 +6094,26 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年12月～</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr"/>
+          <t>2027年1月～ AT-Xにて</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Acca effe×フロンティアエンジン</t>
+        </is>
+      </c>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25212</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23537</t>
         </is>
       </c>
     </row>
@@ -6107,11 +6127,11 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>BanG Dream! It's MyGO!!!!!／Ave Mujica（続編）</t>
+          <t>ディズニー ツイステッドワンダーランド ザ アニメーション ～エピソード オブ サバナクロー～</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6119,12 +6139,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2027年1月～ 日本テレビ系全国30局ネットにて</t>
+          <t>2026年12月～</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -6134,7 +6154,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25765</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25212</t>
         </is>
       </c>
     </row>
@@ -6148,11 +6168,11 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ヒストリエ</t>
+          <t>BanG Dream! It's MyGO!!!!!／Ave Mujica（続編）</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6165,21 +6185,17 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
+          <t>2027年1月～ 日本テレビ系全国30局ネットにて</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr"/>
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27368</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25765</t>
         </is>
       </c>
     </row>
@@ -6193,11 +6209,11 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>姫騎士様のヒモ</t>
+          <t>ヒストリエ</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6215,7 +6231,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>BLADE</t>
+          <t>ライデンフィルム</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -6224,7 +6240,7 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25551</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27368</t>
         </is>
       </c>
     </row>
@@ -6238,11 +6254,11 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ひらやすみ</t>
+          <t>姫騎士様のヒモ</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6255,12 +6271,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2027年1月～ NHK総合テレビ</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Production +h.</t>
+          <t>BLADE</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -6269,7 +6285,7 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26471</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25551</t>
         </is>
       </c>
     </row>
@@ -6283,11 +6299,11 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>BLUE EYE SAMURAI/ブルーアイ・サムライ</t>
+          <t>ひらやすみ</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -6295,22 +6311,26 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>シーズン1：2023年11月3日（金）～ シーズン2：2027年1月～ シーズン3：未発表 Netflixにて</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr"/>
+          <t>2027年1月～ NHK総合テレビ</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Production +h.</t>
+        </is>
+      </c>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28984</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26471</t>
         </is>
       </c>
     </row>
@@ -6324,11 +6344,11 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>ペンと手錠と事実婚</t>
+          <t>BLUE EYE SAMURAI/ブルーアイ・サムライ</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -6336,26 +6356,22 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>EMTスクエアード</t>
-        </is>
-      </c>
+          <t>シーズン1：2023年11月3日（金）～ シーズン2：2027年1月～ シーズン3：未発表 Netflixにて</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28250</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28984</t>
         </is>
       </c>
     </row>
@@ -6369,11 +6385,11 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>魔入りました！入間くん if Episode of 魔フィア</t>
+          <t>ペンと手錠と事実婚</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -6386,17 +6402,21 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2027年1月～ NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr"/>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>EMTスクエアード</t>
+        </is>
+      </c>
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27609</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28250</t>
         </is>
       </c>
     </row>
@@ -6410,11 +6430,11 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>マッシュル-MASHLE- 三魔対争神覚者最終試験編</t>
+          <t>魔入りました！入間くん if Episode of 魔フィア</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -6427,7 +6447,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ NHK総合にて</t>
         </is>
       </c>
       <c r="H126" t="inlineStr"/>
@@ -6437,7 +6457,7 @@
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24109</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27609</t>
         </is>
       </c>
     </row>
@@ -6451,11 +6471,11 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>マッシュル-MASHLE- 三魔対争神覚者最終試験編</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -6468,29 +6488,17 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2027年1月〜 TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>MAHO FILM</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>花噺</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>KANA-BOON</t>
-        </is>
-      </c>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26896</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24109</t>
         </is>
       </c>
     </row>
@@ -6504,11 +6512,11 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>マリッジトキシン 第2期</t>
+          <t>茉莉花官吏伝</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -6521,21 +6529,29 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月〜 TOKYO MXほか</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>ボンズ</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
+          <t>MAHO FILM</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>花噺</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>KANA-BOON</t>
+        </is>
+      </c>
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28681</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26896</t>
         </is>
       </c>
     </row>
@@ -6549,11 +6565,11 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>MURCIÉLAGO-ムルシエラゴ-</t>
+          <t>マリッジトキシン 第2期</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -6566,12 +6582,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>サテライト</t>
+          <t>ボンズ</t>
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
@@ -6580,7 +6596,7 @@
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28714</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28681</t>
         </is>
       </c>
     </row>
@@ -6594,11 +6610,11 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>モモモ！ニニモ</t>
+          <t>MURCIÉLAGO-ムルシエラゴ-</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -6611,17 +6627,21 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr"/>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>サテライト</t>
+        </is>
+      </c>
       <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr"/>
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28563</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28714</t>
         </is>
       </c>
     </row>
@@ -6635,11 +6655,11 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>悠久の愚者アズリーの、賢者のすゝめ</t>
+          <t>モモモ！ニニモ</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -6652,21 +6672,17 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>スタジオエル</t>
-        </is>
-      </c>
+          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27618</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28563</t>
         </is>
       </c>
     </row>
@@ -6680,11 +6696,11 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ラーメン赤猫 其の二</t>
+          <t>悠久の愚者アズリーの、賢者のすゝめ</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -6702,7 +6718,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>スタジオエル</t>
         </is>
       </c>
       <c r="I132" t="inlineStr"/>
@@ -6711,7 +6727,7 @@
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25390</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27618</t>
         </is>
       </c>
     </row>
@@ -6725,11 +6741,11 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>業物語 かれんオウガ</t>
+          <t>ラーメン赤猫 其の二</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -6742,12 +6758,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026年冬</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>シャフト</t>
+          <t>E&amp;H production</t>
         </is>
       </c>
       <c r="I133" t="inlineStr"/>
@@ -6755,6 +6771,51 @@
       <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=25390</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>40</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>業物語 かれんオウガ</t>
+        </is>
+      </c>
+      <c r="E134" t="b">
+        <v>0</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2026年冬</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>シャフト</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26354</t>
         </is>
@@ -6771,7 +6832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6980,7 +7041,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -6988,7 +7049,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$・¥・€ （ドル・エン・ユーロ）</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -6996,13 +7057,37 @@
           <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7rxIZ3z0S4s</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>793667</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7rxIZ3z0S4s</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>793667</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:00:21</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -7015,7 +7100,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -7023,7 +7108,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -7031,45 +7116,21 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Escape</t>
+          <t>$・¥・€ （ドル・エン・ユーロ）</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Kis-My-Ft2</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>72219</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>625638</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:00:29</t>
-        </is>
-      </c>
+          <t>福賀くるみ（CV：鈴木愛奈）</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -7082,7 +7143,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -7098,21 +7159,45 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>Escape</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>THE RAMPAGE</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+          <t>Kis-My-Ft2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>72219</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>625638</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:00:29</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -7125,7 +7210,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D7" t="b">
@@ -7133,7 +7218,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -7141,12 +7226,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>THE RAMPAGE</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -7176,7 +7261,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -7184,12 +7269,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>krage</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -7211,7 +7296,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -7219,7 +7304,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -7227,12 +7312,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>リスポーン!!</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>角巻わため</t>
+          <t>krage</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -7254,7 +7339,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -7270,45 +7355,21 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>雲を抜け風下へ私だけ</t>
+          <t>リスポーン!!</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ヨルシカ</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>1545312</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>7582011</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:08:32</t>
-        </is>
-      </c>
+          <t>角巻わため</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -7321,7 +7382,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -7337,43 +7398,43 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>雲を抜け風下へ私だけ</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>amazarashi</t>
+          <t>ヨルシカ</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>188410</v>
+        <v>1661451</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>KONAMI公式</t>
+          <t>TOHO animation</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>188410</v>
+        <v>7621731</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>KONAMI公式</t>
+          <t>TOHO animation</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-09-01T09:01:08</t>
+          <t>2026-09-02T09:01:15</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7449,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ごーすと・みーつ・ぎゃる！</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D12" t="b">
@@ -7396,7 +7457,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -7404,21 +7465,45 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>にこいちミライ</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+          <t>amazarashi</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>188410</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>188410</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:01:08</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -7431,7 +7516,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D13" t="b">
@@ -7439,7 +7524,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -7447,12 +7532,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -7474,7 +7559,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -7490,12 +7575,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -7525,7 +7610,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -7533,35 +7618,21 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>178700</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
-        </is>
-      </c>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:01:34</t>
-        </is>
-      </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -7574,7 +7645,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D16" t="b">
@@ -7582,7 +7653,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -7590,21 +7661,35 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>風の中は走るっきゃないっ！</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>三月のパンタシア</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>178700</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:01:34</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -7617,7 +7702,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -7633,12 +7718,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>影響力∞アイドル</t>
+          <t>風の中は走るっきゃないっ！</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>HoneyWorks feat.ハコニワリリィ</t>
+          <t>三月のパンタシア</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -7668,7 +7753,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -7676,12 +7761,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>星を巡る</t>
+          <t>影響力∞アイドル</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ロクデナシ</t>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -7703,7 +7788,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DARK MACHINE THE ANIMATION</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D19" t="b">
@@ -7711,7 +7796,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -7719,12 +7804,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>存在理由 改</t>
+          <t>星を巡る</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>BUCK∞TICK</t>
+          <t>ロクデナシ</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -7746,7 +7831,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -7762,12 +7847,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -7797,7 +7882,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -7805,12 +7890,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -7832,7 +7917,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -7840,7 +7925,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -7848,12 +7933,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>SUPER★DRAGON</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -7883,7 +7968,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -7891,12 +7976,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -7918,7 +8003,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -7926,7 +8011,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -7934,12 +8019,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>この心臓に花束を</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>心梅</t>
+          <t>Daoko</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -7969,7 +8054,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -7977,35 +8062,21 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>白昼夢</t>
+          <t>この心臓に花束を</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>カグラナナ</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>2557872</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>カグラナナchannel／ななかぐら</t>
-        </is>
-      </c>
+          <t>心梅</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>2026-08-27T09:02:46</t>
-        </is>
-      </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -8018,7 +8089,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -8026,7 +8097,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -8034,43 +8105,33 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>白昼夢</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Kucci</t>
+          <t>カグラナナ</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>722270</v>
+        <v>2557872</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M26" t="n">
-        <v>722270</v>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>カグラナナchannel／ななかぐら</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-09-01T09:02:20</t>
+          <t>2026-08-27T09:02:46</t>
         </is>
       </c>
     </row>
@@ -8093,7 +8154,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -8101,21 +8162,21 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
+          <t>Kucci</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>405099</v>
+        <v>722270</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -8124,11 +8185,11 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
         </is>
       </c>
       <c r="M27" t="n">
-        <v>405099</v>
+        <v>722270</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -8137,7 +8198,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-09-01T09:02:30</t>
+          <t>2026-09-01T09:02:20</t>
         </is>
       </c>
     </row>
@@ -8152,7 +8213,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8168,21 +8229,45 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>405099</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>405099</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:02:30</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -8195,7 +8280,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8203,7 +8288,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -8211,12 +8296,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Re:name</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -8246,7 +8331,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8254,12 +8339,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Ray of Emotion</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>導凰</t>
+          <t>Re:name</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8281,7 +8366,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8289,7 +8374,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -8297,12 +8382,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Ado</t>
+          <t>導凰</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8324,7 +8409,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8340,35 +8425,21 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>あやかしあやし</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>48992</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+          <t>Ado</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>2026-08-25T09:10:14</t>
-        </is>
-      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8389,7 +8460,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -8397,43 +8468,33 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>朔日 feat. 吉乃</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>月詠み</t>
+          <t>伊東歌詞太郎</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>46450</v>
+        <v>49379</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>デュエチューブ-DM公式-</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="M33" t="n">
-        <v>46450</v>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-08-25T09:10:21</t>
+          <t>2026-09-02T09:02:46</t>
         </is>
       </c>
     </row>
@@ -8448,7 +8509,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8456,7 +8517,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8464,21 +8525,45 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>47605</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>47605</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:02:51</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -8499,7 +8584,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -8507,12 +8592,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8534,7 +8619,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8542,7 +8627,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -8550,12 +8635,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>FZMZ</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8585,7 +8670,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8593,12 +8678,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -8620,7 +8705,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8628,7 +8713,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8636,12 +8721,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -8671,7 +8756,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -8679,12 +8764,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>East Of Eden</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -8706,7 +8791,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -8714,7 +8799,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -8722,35 +8807,21 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>75253</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>JO1</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:38</t>
-        </is>
-      </c>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -8771,7 +8842,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -8779,43 +8850,33 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
+          <t>JO1</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>92436</v>
+        <v>75253</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M41" t="n">
-        <v>3815771</v>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-08-28T09:12:50</t>
+          <t>2026-08-28T09:12:38</t>
         </is>
       </c>
     </row>
@@ -8830,7 +8891,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8838,7 +8899,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -8846,21 +8907,45 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>92436</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>3815771</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:50</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -8873,7 +8958,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -8881,7 +8966,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -8889,12 +8974,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+          <t>東京スカパラダイスオーケストラ</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8916,7 +9001,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -8932,12 +9017,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Diamond Dust</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Sizuk</t>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8967,7 +9052,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -8975,35 +9060,21 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>COMPRESSION :[</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>内田真礼</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
-        </is>
-      </c>
-      <c r="J45" t="n">
-        <v>7057</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
-        </is>
-      </c>
+          <t>Sizuk</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:11</t>
-        </is>
-      </c>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9016,7 +9087,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -9024,7 +9095,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -9032,43 +9103,33 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>内田真礼</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>4887</v>
+        <v>7057</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
-        <v>4887</v>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
+          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-09-01T09:04:18</t>
+          <t>2026-09-01T09:04:11</t>
         </is>
       </c>
     </row>
@@ -9083,7 +9144,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -9091,7 +9152,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -9099,33 +9160,43 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>771368</v>
+        <v>4887</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>4887</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-09-01T09:04:33</t>
+          <t>2026-09-01T09:04:18</t>
         </is>
       </c>
     </row>
@@ -9140,7 +9211,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -9148,7 +9219,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -9156,21 +9227,35 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>MOUSE DRIVE</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Maware Isogavva</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
+          <t>TOOBOE</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>771368</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:04:33</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9183,7 +9268,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -9191,7 +9276,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -9199,12 +9284,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Remedy</t>
+          <t>MOUSE DRIVE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>ASCA</t>
+          <t>Maware Isogavva</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -9234,7 +9319,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -9242,7 +9327,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Double Wings</t>
+          <t>Remedy</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -9269,7 +9354,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -9277,7 +9362,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -9285,35 +9370,21 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Double Wings</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>108508</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:05:02</t>
-        </is>
-      </c>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9334,7 +9405,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -9342,21 +9413,21 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>ReMind</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Daisy×Daisy</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>77536</v>
+        <v>108508</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -9368,7 +9439,7 @@
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-08-27T09:04:35</t>
+          <t>2026-09-01T09:05:02</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9454,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9391,7 +9462,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -9399,43 +9470,33 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>ReMind</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>Daisy×Daisy</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>309603</v>
+        <v>77536</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M53" t="n">
-        <v>309603</v>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-08-28T09:13:31</t>
+          <t>2026-08-27T09:04:35</t>
         </is>
       </c>
     </row>
@@ -9458,7 +9519,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -9466,12 +9527,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -9480,7 +9541,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>309598</v>
+        <v>309603</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -9493,7 +9554,7 @@
         </is>
       </c>
       <c r="M54" t="n">
-        <v>309598</v>
+        <v>309603</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -9502,7 +9563,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-08-28T09:13:41</t>
+          <t>2026-08-28T09:13:31</t>
         </is>
       </c>
     </row>
@@ -9517,7 +9578,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9525,7 +9586,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -9533,21 +9594,45 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>309598</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>309598</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:41</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -9568,7 +9653,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -9576,12 +9661,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -9603,15 +9688,15 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D57" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -9619,12 +9704,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>BOW AND ARROW</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>米津玄師</t>
+          <t>ASTERISM</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9654,7 +9739,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -9662,12 +9747,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>アタシのドレス</t>
+          <t>BOW AND ARROW</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>ねぐせ。</t>
+          <t>米津玄師</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -9689,15 +9774,15 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -9705,12 +9790,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>アタシのドレス</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>ねぐせ。</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -9732,7 +9817,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9748,45 +9833,21 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>Melodic Impact</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J60" t="n">
-        <v>1026619</v>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M60" t="n">
-        <v>411016</v>
-      </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:05:26</t>
-        </is>
-      </c>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -9807,7 +9868,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -9815,34 +9876,34 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Shalala</t>
+          <t>What's "KAZOKU"</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
+          <t>櫻坂46</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>454972</v>
+        <v>1026619</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
         </is>
       </c>
       <c r="M61" t="n">
-        <v>416490</v>
+        <v>411016</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -9851,22 +9912,22 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-09-01T09:05:35</t>
+          <t>2026-09-01T09:05:26</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>気になってる人が男じゃなかった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -9874,7 +9935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -9882,48 +9943,58 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Breed</t>
+          <t>Shalala</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Nirvana</t>
+          <t>ピラフ星人</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
+          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>8804348</v>
+        <v>454972</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>416490</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-09-01T09:06:04</t>
+          <t>2026-09-01T09:05:35</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>わたしの幸せな結婚 特別篇</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -9931,7 +10002,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -9939,41 +10010,141 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
+          <t>プレリュードの手前に ～for me&amp;you～</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>気になってる人が男じゃなかった</t>
+        </is>
+      </c>
+      <c r="D64" t="b">
+        <v>0</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Breed</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>8804348</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:06:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>茉莉花官吏伝</t>
+        </is>
+      </c>
+      <c r="D65" t="b">
+        <v>0</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
           <t>花噺</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H65" t="inlineStr">
         <is>
           <t>KANA-BOON</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="J63" t="n">
+      <c r="J65" t="n">
         <v>96835</v>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L65" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="M63" t="n">
+      <c r="M65" t="n">
         <v>96835</v>
       </c>
-      <c r="N63" t="inlineStr">
+      <c r="N65" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
+      <c r="O65" t="inlineStr">
         <is>
           <t>2026-09-01T09:06:09</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-04
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -935,10 +935,26 @@
           <t>スタジオディーン</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>逃光行</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>原因は自分にある。</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>光の側で</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>名無し之太郎</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27963</t>
@@ -3368,14 +3384,30 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
+          <t>2026年10月11日（日）～ フジテレビほか</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>オノガミ</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>メガテラ・ゼロ</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>完璧のペキ</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>ビッケブランカ</t>
+        </is>
+      </c>
       <c r="M59" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
@@ -6889,7 +6921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7439,7 +7471,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>彼方から</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -7447,7 +7479,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -7455,12 +7487,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>逃光行</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>THE RAMPAGE</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -7482,7 +7514,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>彼方から</t>
         </is>
       </c>
       <c r="D12" t="b">
@@ -7490,7 +7522,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -7498,12 +7530,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>光の側で</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>名無し之太郎</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -7525,7 +7557,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D13" t="b">
@@ -7533,7 +7565,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -7541,12 +7573,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>krage</t>
+          <t>THE RAMPAGE</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -7568,7 +7600,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -7584,12 +7616,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>リスポーン!!</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>角巻わため</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -7611,7 +7643,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D15" t="b">
@@ -7619,7 +7651,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -7627,45 +7659,21 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>雲を抜け風下へ私だけ</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>ヨルシカ</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>1661451</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
-        </is>
-      </c>
-      <c r="M15" t="n">
-        <v>7621731</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>2026-09-02T09:01:15</t>
-        </is>
-      </c>
+          <t>krage</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -7678,7 +7686,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="D16" t="b">
@@ -7694,45 +7702,21 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>リスポーン!!</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>amazarashi</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>188410</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="M16" t="n">
-        <v>188410</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:01:08</t>
-        </is>
-      </c>
+          <t>角巻わため</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -7745,7 +7729,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ごーすと・みーつ・ぎゃる！</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -7753,7 +7737,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -7761,21 +7745,45 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>にこいちミライ</t>
+          <t>雲を抜け風下へ私だけ</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+          <t>ヨルシカ</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>1661451</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>7621731</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:01:15</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -7788,7 +7796,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D18" t="b">
@@ -7804,21 +7812,45 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+          <t>amazarashi</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>188410</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>188410</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:01:08</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -7831,7 +7863,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D19" t="b">
@@ -7839,7 +7871,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -7847,12 +7879,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -7874,7 +7906,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -7882,7 +7914,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -7890,35 +7922,21 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>178700</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
-        </is>
-      </c>
+          <t>西川貴教</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:01:34</t>
-        </is>
-      </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -7931,7 +7949,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -7947,12 +7965,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>風の中は走るっきゃないっ！</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>三月のパンタシア</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -7974,7 +7992,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -7982,7 +8000,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -7990,21 +8008,35 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>影響力∞アイドル</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>HoneyWorks feat.ハコニワリリィ</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>178700</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:01:34</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -8017,7 +8049,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="D23" t="b">
@@ -8025,7 +8057,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -8033,12 +8065,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>星を巡る</t>
+          <t>風の中は走るっきゃないっ！</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ロクデナシ</t>
+          <t>三月のパンタシア</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -8060,7 +8092,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DARK MACHINE THE ANIMATION</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -8076,12 +8108,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>存在理由 改</t>
+          <t>影響力∞アイドル</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>BUCK∞TICK</t>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -8103,7 +8135,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -8111,7 +8143,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -8119,12 +8151,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>星を巡る</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>ロクデナシ</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -8146,7 +8178,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -8154,7 +8186,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -8162,12 +8194,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -8189,7 +8221,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -8205,12 +8237,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -8232,7 +8264,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8248,12 +8280,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>SUPER★DRAGON</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -8275,7 +8307,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8291,12 +8323,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>この心臓に花束を</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>心梅</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -8318,7 +8350,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -8334,35 +8366,21 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>白昼夢</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>カグラナナ</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>2557872</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>カグラナナchannel／ななかぐら</t>
-        </is>
-      </c>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>2026-08-27T09:02:46</t>
-        </is>
-      </c>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -8375,7 +8393,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8391,45 +8409,21 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>この心臓に花束を</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>722270</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M31" t="n">
-        <v>722270</v>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:02:20</t>
-        </is>
-      </c>
+          <t>心梅</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -8442,7 +8436,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8458,43 +8452,33 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>白昼夢</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
+          <t>カグラナナ</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>405099</v>
+        <v>2562896</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M32" t="n">
-        <v>405099</v>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>カグラナナchannel／ななかぐら</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-09-01T09:02:30</t>
+          <t>2026-09-04T09:02:40</t>
         </is>
       </c>
     </row>
@@ -8509,7 +8493,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -8517,7 +8501,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -8525,21 +8509,45 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>722270</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>722270</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:02:20</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -8552,7 +8560,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8560,7 +8568,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8568,21 +8576,45 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Re:name</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>405099</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>405099</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:02:30</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -8595,7 +8627,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8611,12 +8643,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Ray of Emotion</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>導凰</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8638,7 +8670,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8654,12 +8686,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Ado</t>
+          <t>Re:name</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8681,7 +8713,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -8689,7 +8721,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8697,35 +8729,21 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>あやかしあやし</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>49379</v>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+          <t>導凰</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>2026-09-02T09:02:46</t>
-        </is>
-      </c>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -8738,7 +8756,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8746,7 +8764,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8754,45 +8772,21 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>朔日 feat. 吉乃</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>月詠み</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>47605</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
-        <v>47605</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>2026-09-02T09:02:51</t>
-        </is>
-      </c>
+          <t>Ado</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -8805,7 +8799,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -8821,21 +8815,35 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>49379</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:02:46</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -8848,7 +8856,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -8864,21 +8872,45 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>47605</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>47605</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:02:51</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -8891,7 +8923,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -8907,12 +8939,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>FZMZ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8934,7 +8966,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8950,12 +8982,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8977,7 +9009,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -8993,12 +9025,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -9020,7 +9052,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -9036,12 +9068,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -9063,7 +9095,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -9079,35 +9111,21 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
-        </is>
-      </c>
-      <c r="J45" t="n">
-        <v>75253</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>JO1</t>
-        </is>
-      </c>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:38</t>
-        </is>
-      </c>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9120,7 +9138,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -9136,45 +9154,21 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
-        </is>
-      </c>
-      <c r="J46" t="n">
-        <v>92436</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
-        <v>3815771</v>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:50</t>
-        </is>
-      </c>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9187,7 +9181,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -9195,7 +9189,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -9203,21 +9197,35 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>75253</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:38</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9230,7 +9238,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -9238,7 +9246,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -9246,21 +9254,45 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>92436</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>3815771</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:12:50</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9273,7 +9305,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -9289,21 +9321,45 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Diamond Dust</t>
+          <t>オノガミ</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Sizuk</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
+          <t>メガテラ・ゼロ</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>1485</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>hyou - Anime on Piano</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>1485</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>hyou - Anime on Piano</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:03:51</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9316,7 +9372,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -9332,35 +9388,21 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>COMPRESSION :[</t>
+          <t>完璧のペキ</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>内田真礼</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
-        </is>
-      </c>
-      <c r="J50" t="n">
-        <v>7057</v>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
-        </is>
-      </c>
+          <t>ビッケブランカ</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:11</t>
-        </is>
-      </c>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -9373,7 +9415,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -9381,7 +9423,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -9389,45 +9431,21 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>4887</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
-        <v>4887</v>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:18</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9440,7 +9458,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -9448,7 +9466,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -9456,35 +9474,21 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J52" t="n">
-        <v>771368</v>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:33</t>
-        </is>
-      </c>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9497,7 +9501,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9505,7 +9509,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -9513,12 +9517,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>MOUSE DRIVE</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Maware Isogavva</t>
+          <t>Sizuk</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -9540,7 +9544,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9548,7 +9552,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -9556,21 +9560,35 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Remedy</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>ASCA</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
+          <t>内田真礼</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>7057</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:04:11</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -9583,7 +9601,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9591,7 +9609,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -9599,21 +9617,45 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Double Wings</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>ASCA</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+          <t>WANIMA</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>4887</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>4887</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:04:18</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -9626,7 +9668,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9634,7 +9676,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -9642,25 +9684,25 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>TOOBOE</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>108508</v>
+        <v>771368</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+          <t>john / TOOBOE</t>
         </is>
       </c>
       <c r="L56" t="inlineStr"/>
@@ -9668,7 +9710,7 @@
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-09-01T09:05:02</t>
+          <t>2026-09-01T09:04:33</t>
         </is>
       </c>
     </row>
@@ -9683,7 +9725,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9691,7 +9733,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -9699,35 +9741,21 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>ReMind</t>
+          <t>MOUSE DRIVE</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Daisy×Daisy</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
-        </is>
-      </c>
-      <c r="J57" t="n">
-        <v>77536</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>Maware Isogavva</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>2026-08-27T09:04:35</t>
-        </is>
-      </c>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -9740,7 +9768,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -9756,45 +9784,21 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>Remedy</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J58" t="n">
-        <v>309603</v>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M58" t="n">
-        <v>309603</v>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:13:31</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -9807,7 +9811,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9823,45 +9827,21 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>Double Wings</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J59" t="n">
-        <v>309598</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M59" t="n">
-        <v>309598</v>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:13:41</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -9874,7 +9854,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9890,21 +9870,35 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>108508</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:05:02</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -9917,7 +9911,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -9933,21 +9927,35 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>ReMind</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
+          <t>Daisy×Daisy</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>80979</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:04:59</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -9960,11 +9968,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -9976,21 +9984,45 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>BOW AND ARROW</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>米津玄師</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>309603</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>309603</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:31</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10003,11 +10035,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D63" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -10019,21 +10051,45 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>アタシのドレス</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>ねぐせ。</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>309598</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>309598</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>2026-08-28T09:13:41</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10046,7 +10102,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -10062,12 +10118,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -10089,7 +10145,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -10097,7 +10153,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -10105,45 +10161,21 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J65" t="n">
-        <v>1026619</v>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M65" t="n">
-        <v>411016</v>
-      </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:05:26</t>
-        </is>
-      </c>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10156,15 +10188,15 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -10172,45 +10204,21 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Shalala</t>
+          <t>BOW AND ARROW</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
-        </is>
-      </c>
-      <c r="J66" t="n">
-        <v>454972</v>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
-        </is>
-      </c>
-      <c r="M66" t="n">
-        <v>416490</v>
-      </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:05:35</t>
-        </is>
-      </c>
+          <t>米津玄師</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10223,11 +10231,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>わたしの幸せな結婚 特別篇</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -10239,12 +10247,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>プレリュードの手前に ～for me&amp;you～</t>
+          <t>アタシのドレス</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
+          <t>ねぐせ。</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -10257,16 +10265,16 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>気になってる人が男じゃなかった</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -10282,48 +10290,34 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Breed</t>
+          <t>Melodic Impact</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
-        </is>
-      </c>
-      <c r="J68" t="n">
-        <v>8804348</v>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:06:04</t>
-        </is>
-      </c>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -10339,41 +10333,275 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>1026619</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>411016</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:05:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D70" t="b">
+        <v>0</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>454972</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>416490</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:05:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>わたしの幸せな結婚 特別篇</t>
+        </is>
+      </c>
+      <c r="D71" t="b">
+        <v>0</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>プレリュードの手前に ～for me&amp;you～</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>気になってる人が男じゃなかった</t>
+        </is>
+      </c>
+      <c r="D72" t="b">
+        <v>0</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Breed</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>8804348</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:06:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>茉莉花官吏伝</t>
+        </is>
+      </c>
+      <c r="D73" t="b">
+        <v>0</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
           <t>花噺</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H73" t="inlineStr">
         <is>
           <t>KANA-BOON</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="J69" t="n">
+      <c r="J73" t="n">
         <v>96835</v>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="K73" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="M69" t="n">
+      <c r="M73" t="n">
         <v>96835</v>
       </c>
-      <c r="N69" t="inlineStr">
+      <c r="N73" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr">
+      <c r="O73" t="inlineStr">
         <is>
           <t>2026-09-01T09:06:09</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-07
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -588,10 +588,26 @@
           <t>トムス・エンタテインメント</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fortress Defense</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>10-FEET</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>トライアングル</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>ヒグチアイ</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
@@ -1470,10 +1486,26 @@
           <t>スタジオKAI</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>エスコート</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>THE BEAT GARDEN</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>花蔭</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Superfly</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
@@ -2255,7 +2287,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月4日（日）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2960,7 +2992,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年9月27日（日）～ CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3744,7 +3776,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月4日（日）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4426,7 +4458,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月4日（日）～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -6921,7 +6953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O73"/>
+  <dimension ref="A1:O79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7184,7 +7216,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>アオのハコ Season2</t>
+          <t>アオアシ Season2</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -7200,45 +7232,21 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>あなたの花の色</t>
+          <t>Fortress Defense</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>aiko</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d0jg9hNHqn8</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>10086016</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=d0jg9hNHqn8</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>10086016</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:09:49</t>
-        </is>
-      </c>
+          <t>10-FEET</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -7251,7 +7259,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>アオのハコ Season2</t>
+          <t>アオアシ Season2</t>
         </is>
       </c>
       <c r="D7" t="b">
@@ -7267,12 +7275,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>blue in</t>
+          <t>トライアングル</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>エルスウェア紀行</t>
+          <t>ヒグチアイ</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -7294,7 +7302,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FX戦士くるみちゃん</t>
+          <t>アオのハコ Season2</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -7310,43 +7318,43 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>FX戦士くるみちゃん</t>
+          <t>あなたの花の色</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>福賀くるみ（CV：鈴木愛奈）</t>
+          <t>aiko</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7rxIZ3z0S4s</t>
+          <t>https://www.youtube.com/watch?v=d0jg9hNHqn8</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>793667</v>
+        <v>10153236</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
+          <t>TMSアニメ公式チャンネル</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7rxIZ3z0S4s</t>
+          <t>https://www.youtube.com/watch?v=d0jg9hNHqn8</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>793667</v>
+        <v>10153236</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
+          <t>TMSアニメ公式チャンネル</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-09-02T09:00:21</t>
+          <t>2026-09-07T09:00:48</t>
         </is>
       </c>
     </row>
@@ -7361,7 +7369,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FX戦士くるみちゃん</t>
+          <t>アオのハコ Season2</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -7377,12 +7385,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>$・¥・€ （ドル・エン・ユーロ）</t>
+          <t>blue in</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>福賀くるみ（CV：鈴木愛奈）</t>
+          <t>エルスウェア紀行</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -7404,7 +7412,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -7412,7 +7420,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -7420,43 +7428,43 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Escape</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Kis-My-Ft2</t>
+          <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+          <t>https://www.youtube.com/watch?v=7rxIZ3z0S4s</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>72219</v>
+        <v>793667</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
+          <t>https://www.youtube.com/watch?v=7rxIZ3z0S4s</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>625638</v>
+        <v>793667</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+          <t>KADOKAWAanime</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-09-01T09:00:29</t>
+          <t>2026-09-02T09:00:21</t>
         </is>
       </c>
     </row>
@@ -7471,7 +7479,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>彼方から</t>
+          <t>FX戦士くるみちゃん</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -7479,7 +7487,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -7487,12 +7495,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>逃光行</t>
+          <t>$・¥・€ （ドル・エン・ユーロ）</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -7514,7 +7522,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>彼方から</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="D12" t="b">
@@ -7522,7 +7530,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -7530,21 +7538,45 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>光の側で</t>
+          <t>Escape</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>名無し之太郎</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+          <t>Kis-My-Ft2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zxgmRfemSMI</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>72219</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GrGLgc6XKjs</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>625638</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:00:29</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -7557,7 +7589,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>彼方から</t>
         </is>
       </c>
       <c r="D13" t="b">
@@ -7565,7 +7597,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -7573,12 +7605,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>逃光行</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>THE RAMPAGE</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -7600,7 +7632,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>彼方から</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -7608,7 +7640,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -7616,12 +7648,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>光の側で</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>名無し之太郎</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -7643,7 +7675,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="D15" t="b">
@@ -7651,7 +7683,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -7659,21 +7691,45 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Everlasting</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>krage</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+          <t>THE RAMPAGE</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7nmvfmUiWEE</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>293138</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>THE RAMPAGE from EXILE TRIBE</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7nmvfmUiWEE</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>293138</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>THE RAMPAGE from EXILE TRIBE</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:01:30</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -7686,7 +7742,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D16" t="b">
@@ -7702,12 +7758,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>リスポーン!!</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>角巻わため</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -7729,7 +7785,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -7737,7 +7793,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -7745,45 +7801,21 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>雲を抜け風下へ私だけ</t>
+          <t>Everlasting</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ヨルシカ</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>1661451</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
-        </is>
-      </c>
-      <c r="M17" t="n">
-        <v>7621731</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>2026-09-02T09:01:15</t>
-        </is>
-      </c>
+          <t>krage</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -7796,7 +7828,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="D18" t="b">
@@ -7812,45 +7844,21 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>悲しみさえ大人びて</t>
+          <t>リスポーン!!</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>amazarashi</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>188410</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
-        </is>
-      </c>
-      <c r="M18" t="n">
-        <v>188410</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>KONAMI公式</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:01:08</t>
-        </is>
-      </c>
+          <t>角巻わため</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -7863,7 +7871,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ごーすと・みーつ・ぎゃる！</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="D19" t="b">
@@ -7871,7 +7879,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -7879,21 +7887,45 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>にこいちミライ</t>
+          <t>雲を抜け風下へ私だけ</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+          <t>ヨルシカ</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9rProUQlD-I</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>1661451</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HrRxvh4bkHE</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>7621731</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:01:15</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -7906,7 +7938,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -7922,21 +7954,45 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>悲しみさえ大人びて</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+          <t>amazarashi</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>188410</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>188410</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>KONAMI公式</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:01:08</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -7949,7 +8005,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>ごーすと・みーつ・ぎゃる！</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -7957,7 +8013,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -7965,21 +8021,45 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>にこいちミライ</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+          <t>夢限大みゅーたいぷ</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CcAE0TcmOjQ</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>15314</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CcAE0TcmOjQ</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>15314</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:02:05</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -7992,7 +8072,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>氷の城壁 第2期</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -8000,7 +8080,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -8008,35 +8088,21 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>エスコート</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>178700</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
-        </is>
-      </c>
+          <t>THE BEAT GARDEN</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:01:34</t>
-        </is>
-      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -8049,7 +8115,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>氷の城壁 第2期</t>
         </is>
       </c>
       <c r="D23" t="b">
@@ -8057,7 +8123,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -8065,12 +8131,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>風の中は走るっきゃないっ！</t>
+          <t>花蔭</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>三月のパンタシア</t>
+          <t>Superfly</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -8092,7 +8158,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -8108,12 +8174,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>影響力∞アイドル</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>HoneyWorks feat.ハコニワリリィ</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -8135,7 +8201,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -8143,7 +8209,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -8151,12 +8217,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>星を巡る</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>ロクデナシ</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -8178,7 +8244,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DARK MACHINE THE ANIMATION</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -8186,7 +8252,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -8194,21 +8260,35 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>存在理由 改</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>BUCK∞TICK</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>178700</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:01:34</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -8221,7 +8301,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -8237,12 +8317,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>風の中は走るっきゃないっ！</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>三月のパンタシア</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -8264,7 +8344,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8272,7 +8352,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -8280,12 +8360,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>影響力∞アイドル</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -8307,7 +8387,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8315,7 +8395,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -8323,12 +8403,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>星を巡る</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>ロクデナシ</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -8350,7 +8430,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -8358,7 +8438,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8366,12 +8446,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8393,7 +8473,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8409,12 +8489,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>この心臓に花束を</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>心梅</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8436,7 +8516,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8452,35 +8532,21 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>白昼夢</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>カグラナナ</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>2562896</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>カグラナナchannel／ななかぐら</t>
-        </is>
-      </c>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>2026-09-04T09:02:40</t>
-        </is>
-      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8493,7 +8559,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -8509,45 +8575,21 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J33" t="n">
-        <v>722270</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M33" t="n">
-        <v>722270</v>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:02:20</t>
-        </is>
-      </c>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -8560,7 +8602,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8576,45 +8618,21 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="J34" t="n">
-        <v>405099</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M34" t="n">
-        <v>405099</v>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:02:30</t>
-        </is>
-      </c>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -8627,7 +8645,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8635,7 +8653,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -8643,12 +8661,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>この心臓に花束を</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+          <t>心梅</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8670,7 +8688,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8678,7 +8696,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -8686,21 +8704,35 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>白昼夢</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Re:name</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
+          <t>カグラナナ</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>2562896</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>カグラナナchannel／ななかぐら</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:02:40</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -8713,7 +8745,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -8721,7 +8753,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8729,21 +8761,45 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Ray of Emotion</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>導凰</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>722270</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>722270</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:02:20</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -8756,7 +8812,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8764,7 +8820,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8772,21 +8828,45 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>405099</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>405099</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:02:30</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -8799,7 +8879,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -8807,7 +8887,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -8815,35 +8895,21 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>あやかしあやし</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>49379</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>2026-09-02T09:02:46</t>
-        </is>
-      </c>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -8856,7 +8922,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -8864,7 +8930,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -8872,45 +8938,21 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>朔日 feat. 吉乃</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>月詠み</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>47605</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="M40" t="n">
-        <v>47605</v>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>2026-09-02T09:02:51</t>
-        </is>
-      </c>
+          <t>Re:name</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -8923,7 +8965,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -8931,7 +8973,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -8939,12 +8981,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>導凰</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8966,7 +9008,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8974,7 +9016,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -8982,12 +9024,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -9009,7 +9051,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -9025,21 +9067,35 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>FZMZ</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>49379</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:02:46</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9052,7 +9108,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -9068,21 +9124,45 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>花冷え。</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>47605</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>47605</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:02:51</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -9095,7 +9175,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -9111,12 +9191,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -9138,7 +9218,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -9154,12 +9234,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -9181,7 +9261,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -9197,35 +9277,21 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>75253</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>JO1</t>
-        </is>
-      </c>
+          <t>FZMZ</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:38</t>
-        </is>
-      </c>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9238,7 +9304,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -9254,45 +9320,21 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>92436</v>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M48" t="n">
-        <v>3815771</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:12:50</t>
-        </is>
-      </c>
+          <t>花冷え。</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9305,7 +9347,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -9321,45 +9363,21 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>オノガミ</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>メガテラ・ゼロ</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>1485</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>hyou - Anime on Piano</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
-        </is>
-      </c>
-      <c r="M49" t="n">
-        <v>1485</v>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>hyou - Anime on Piano</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>2026-09-04T09:03:51</t>
-        </is>
-      </c>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9372,7 +9390,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -9388,12 +9406,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>完璧のペキ</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>ビッケブランカ</t>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -9415,7 +9433,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -9423,7 +9441,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -9431,21 +9449,35 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>139300</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:04:27</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9458,7 +9490,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -9466,7 +9498,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -9474,21 +9506,45 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>151085</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>3846269</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:04:39</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9501,7 +9557,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9517,21 +9573,45 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Diamond Dust</t>
+          <t>オノガミ</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Sizuk</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+          <t>メガテラ・ゼロ</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>1485</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>hyou - Anime on Piano</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>1485</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>hyou - Anime on Piano</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:03:51</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -9544,7 +9624,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9560,35 +9640,21 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>COMPRESSION :[</t>
+          <t>完璧のペキ</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>内田真礼</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
-        </is>
-      </c>
-      <c r="J54" t="n">
-        <v>7057</v>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
-        </is>
-      </c>
+          <t>ビッケブランカ</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:11</t>
-        </is>
-      </c>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -9601,7 +9667,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9609,7 +9675,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -9617,45 +9683,21 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J55" t="n">
-        <v>4887</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M55" t="n">
-        <v>4887</v>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:18</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -9668,7 +9710,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9676,7 +9718,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -9684,35 +9726,21 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J56" t="n">
-        <v>771368</v>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:04:33</t>
-        </is>
-      </c>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -9725,7 +9753,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9733,7 +9761,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -9741,12 +9769,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>MOUSE DRIVE</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Maware Isogavva</t>
+          <t>Sizuk</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9768,7 +9796,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -9776,7 +9804,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -9784,21 +9812,35 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Remedy</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>ASCA</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
+          <t>内田真礼</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>7057</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:04:11</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -9811,7 +9853,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9819,7 +9861,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -9827,21 +9869,45 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Double Wings</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>ASCA</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
+          <t>WANIMA</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>4887</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>4887</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:04:18</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -9854,7 +9920,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9862,7 +9928,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -9870,25 +9936,25 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>TOOBOE</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>108508</v>
+        <v>771368</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+          <t>john / TOOBOE</t>
         </is>
       </c>
       <c r="L60" t="inlineStr"/>
@@ -9896,7 +9962,7 @@
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-09-01T09:05:02</t>
+          <t>2026-09-01T09:04:33</t>
         </is>
       </c>
     </row>
@@ -9911,7 +9977,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -9919,7 +9985,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -9927,35 +9993,21 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>ReMind</t>
+          <t>MOUSE DRIVE</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Daisy×Daisy</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
-        </is>
-      </c>
-      <c r="J61" t="n">
-        <v>80979</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>Maware Isogavva</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t>2026-09-04T09:04:59</t>
-        </is>
-      </c>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -9968,7 +10020,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -9984,45 +10036,21 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>Remedy</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J62" t="n">
-        <v>309603</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M62" t="n">
-        <v>309603</v>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:13:31</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10035,7 +10063,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -10051,45 +10079,21 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>Double Wings</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J63" t="n">
-        <v>309598</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M63" t="n">
-        <v>309598</v>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>2026-08-28T09:13:41</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10102,7 +10106,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -10118,21 +10122,35 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>108508</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:05:02</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10145,7 +10163,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -10161,21 +10179,35 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>ReMind</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
+          <t>Daisy×Daisy</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>80979</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:04:59</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10188,11 +10220,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -10204,21 +10236,45 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>BOW AND ARROW</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>米津玄師</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>314538</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>314538</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:05:41</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10231,28 +10287,28 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>アタシのドレス</t>
+          <t>Swingin' Magic</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>ねぐせ。</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -10274,7 +10330,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -10282,7 +10338,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -10290,21 +10346,45 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>314538</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>314538</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:05:54</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10317,7 +10397,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -10325,53 +10405,29 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>どりぃむアラモード</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J69" t="n">
-        <v>1026619</v>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M69" t="n">
-        <v>411016</v>
-      </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:05:26</t>
-        </is>
-      </c>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10384,7 +10440,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -10392,7 +10448,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -10400,45 +10456,21 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Shalala</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
-        </is>
-      </c>
-      <c r="J70" t="n">
-        <v>454972</v>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
-        </is>
-      </c>
-      <c r="M70" t="n">
-        <v>416490</v>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:05:35</t>
-        </is>
-      </c>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10451,7 +10483,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>わたしの幸せな結婚 特別篇</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -10467,12 +10499,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>プレリュードの手前に ～for me&amp;you～</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
+          <t>ASTERISM</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -10485,20 +10517,20 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>気になってる人が男じゃなかった</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -10510,56 +10542,42 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Breed</t>
+          <t>BOW AND ARROW</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
-        </is>
-      </c>
-      <c r="J72" t="n">
-        <v>8804348</v>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
+          <t>米津玄師</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>2026-09-01T09:06:04</t>
-        </is>
-      </c>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -10567,41 +10585,361 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
+          <t>アタシのドレス</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ねぐせ。</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>野生のラスボスが現れた！ 第2期</t>
+        </is>
+      </c>
+      <c r="D74" t="b">
+        <v>0</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D75" t="b">
+        <v>0</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>1026619</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>411016</v>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:05:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>454972</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>416490</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:05:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>わたしの幸せな結婚 特別篇</t>
+        </is>
+      </c>
+      <c r="D77" t="b">
+        <v>0</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>プレリュードの手前に ～for me&amp;you～</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>気になってる人が男じゃなかった</t>
+        </is>
+      </c>
+      <c r="D78" t="b">
+        <v>0</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Breed</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>8804348</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>2026-09-01T09:06:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>茉莉花官吏伝</t>
+        </is>
+      </c>
+      <c r="D79" t="b">
+        <v>0</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
           <t>花噺</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H79" t="inlineStr">
         <is>
           <t>KANA-BOON</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="J73" t="n">
+      <c r="J79" t="n">
         <v>96835</v>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="K79" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr">
+      <c r="L79" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="M73" t="n">
+      <c r="M79" t="n">
         <v>96835</v>
       </c>
-      <c r="N73" t="inlineStr">
+      <c r="N79" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr">
+      <c r="O79" t="inlineStr">
         <is>
           <t>2026-09-01T09:06:09</t>
         </is>

</xml_diff>